<commit_message>
Add Yellow Peel, Tattoo Removal, Snow White Facial, and Eye Light brochures
Batch 1 continuation of the sitemap-driven build-out: each scraped from
its isaacluxe.co page (mechanism, actives/technology, what it treats,
benefits, protocol, candidacy). None of the four source pages had
before/after images, so none were added -- no fabricated photos.

Yellow Peel added under Peel; Snow White Facial and Eye Light added
under Facial (clean fits). Tattoo Removal also placed under Facial as
the closest existing category, though it's an imperfect fit (laser
treatment, not strictly a facial) -- flagged in brochure.xlsx remarks
in case a dedicated category is wanted instead.

brochure.xlsx updated: all 5 brochures from this session (BioRePeel,
Yellow Peel, Tattoo Removal, Snow White Facial, Eye Light) marked
Completed with source notes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -1183,10 +1183,10 @@
         <v>Tattoo Removal</v>
       </c>
       <c r="C56" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D56" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/tattoo-removal/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html.</v>
       </c>
     </row>
     <row r="57">
@@ -1981,10 +1981,10 @@
         <v>Eye Light</v>
       </c>
       <c r="C113" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D113" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/eye-light/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html.</v>
       </c>
     </row>
     <row r="114">
@@ -2345,10 +2345,10 @@
         <v>Snow White Facial</v>
       </c>
       <c r="C139" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D139" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/snow-white-facial/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html.</v>
       </c>
     </row>
     <row r="140">
@@ -3367,10 +3367,10 @@
         <v>Yellow Peel</v>
       </c>
       <c r="C212" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D212" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/yellow-peel-treatment-in-mumbai/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html.</v>
       </c>
     </row>
     <row r="213">

</xml_diff>

<commit_message>
Add 105 sitemap-only treatments to brochure.xlsx
Reverse-checked all 307 sitemap URLs against the Excel by name overlap
to catch treatments that exist on the live site but were never in the
clinic's service-menu export. After filtering out pure location pages,
city-variant SEO duplicates of already-covered treatments, and site
utility pages, 105 genuinely distinct treatments remain (Gynaecomastia,
Vaginal Fillers, Cryolipolysis, Eyebrow Transplant, Ulthera Face
Lifting, Ilha, etc.) -- added as new rows with best-effort category
assignment and "To Build" status, sourced from their sitemap URL.

Total tracked scope is now 390 rows: 40 Completed, 136 To Build (source
available), 134 Missing - No Source, 79 Out of Scope, 1 blank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -5,6 +5,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$285</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,12 +400,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D285"/>
+  <dimension ref="A1:D391"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+    <col min="4" max="4" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4395,9 +4398,1493 @@
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v/>
+      </c>
+      <c r="B286" t="str">
+        <v/>
+      </c>
+      <c r="C286" t="str">
+        <v/>
+      </c>
+      <c r="D286" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B287" t="str">
+        <v>Gynaecomastia</v>
+      </c>
+      <c r="C287" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D287" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/gynaecomastia/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B288" t="str">
+        <v>Liposuction Surgery</v>
+      </c>
+      <c r="C288" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D288" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liposuction-surgery/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B289" t="str">
+        <v>Non-Surgical Breast Lift</v>
+      </c>
+      <c r="C289" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-breast-lift/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B290" t="str">
+        <v>Cryolipolysis</v>
+      </c>
+      <c r="C290" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryolipolysis-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B291" t="str">
+        <v>Instasculpt</v>
+      </c>
+      <c r="C291" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/instasculpt/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B292" t="str">
+        <v>House of Sculpt</v>
+      </c>
+      <c r="C292" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D292" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-sculpt/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B293" t="str">
+        <v>House of Proportion</v>
+      </c>
+      <c r="C293" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-proportion/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B294" t="str">
+        <v>Tummy Tightening</v>
+      </c>
+      <c r="C294" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tummy-tightening/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B295" t="str">
+        <v>Tight Pro</v>
+      </c>
+      <c r="C295" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D295" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tight-pro/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B296" t="str">
+        <v>Ballancer Pro</v>
+      </c>
+      <c r="C296" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ballancer-pro-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B297" t="str">
+        <v>Femme 360 Vaginal Tightening</v>
+      </c>
+      <c r="C297" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D297" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/femme-360-vaginal-tightening/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B298" t="str">
+        <v>Vaginal Fillers</v>
+      </c>
+      <c r="C298" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D298" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/vaginal-fillers/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B299" t="str">
+        <v>Multipolar Radio Frequency</v>
+      </c>
+      <c r="C299" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/multipolar-radio-frequency-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B300" t="str">
+        <v>HIFU Skin Tightening</v>
+      </c>
+      <c r="C300" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Skin Tightening Treatment</v>
+      </c>
+      <c r="C301" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-tightening-treatment-in-vasant-vihar/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Sculpt Tone Plus</v>
+      </c>
+      <c r="C302" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sculptone-plus/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>Body Contouring</v>
+      </c>
+      <c r="B303" t="str">
+        <v>Cool Tech</v>
+      </c>
+      <c r="C303" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cool-tech/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B304" t="str">
+        <v>Ulthera Face Lifting</v>
+      </c>
+      <c r="C304" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ulthera-face-lifting/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B305" t="str">
+        <v>Thread Face Lift</v>
+      </c>
+      <c r="C305" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/thread-face-lift-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B306" t="str">
+        <v>Liquid Facelift</v>
+      </c>
+      <c r="C306" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liquid-facelift-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B307" t="str">
+        <v>Non-Surgical Face Lift</v>
+      </c>
+      <c r="C307" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-face-lift/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B308" t="str">
+        <v>Sygma Lift Treatment</v>
+      </c>
+      <c r="C308" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sygma-lift-treatment-in-gurgaon/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B309" t="str">
+        <v>4-D Lift</v>
+      </c>
+      <c r="C309" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/4-d-lift/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B310" t="str">
+        <v>Face Lift Filler</v>
+      </c>
+      <c r="C310" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-lift-filler-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B311" t="str">
+        <v>Square Jaw Treatment</v>
+      </c>
+      <c r="C311" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D311" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/square-jaw-treatment-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>Face Lifting</v>
+      </c>
+      <c r="B312" t="str">
+        <v>Poppy Chin Treatment</v>
+      </c>
+      <c r="C312" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/poppy-chin-treatment-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B313" t="str">
+        <v>BR Facial</v>
+      </c>
+      <c r="C313" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/br-facial/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B314" t="str">
+        <v>Eve Lom Facial</v>
+      </c>
+      <c r="C314" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eve-lom-facial/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B315" t="str">
+        <v>O2Derm Facial</v>
+      </c>
+      <c r="C315" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/o2derm-facial/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B316" t="str">
+        <v>Exo Glow Treatment</v>
+      </c>
+      <c r="C316" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/exo-glow-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B317" t="str">
+        <v>Meso Glow</v>
+      </c>
+      <c r="C317" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D317" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/meso-glow/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B318" t="str">
+        <v>Lumi Face</v>
+      </c>
+      <c r="C318" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-face/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B319" t="str">
+        <v>Lumi Eyes</v>
+      </c>
+      <c r="C319" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-eyes/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B320" t="str">
+        <v>Cryotherapy Facial</v>
+      </c>
+      <c r="C320" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryotherapy-facial/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Vampire Facial</v>
+      </c>
+      <c r="C321" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/vampire-facial/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B322" t="str">
+        <v>Dermabrasion Treatment</v>
+      </c>
+      <c r="C322" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermabrasion-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B323" t="str">
+        <v>Microdermabrasion Treatment</v>
+      </c>
+      <c r="C323" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/microdermabrasion-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B324" t="str">
+        <v>Skin Polishing</v>
+      </c>
+      <c r="C324" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-polishing/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B325" t="str">
+        <v>Dermamelan Treatment</v>
+      </c>
+      <c r="C325" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermamelan-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B326" t="str">
+        <v>Skin Lightening Treatment</v>
+      </c>
+      <c r="C326" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-lightening-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B327" t="str">
+        <v>Tribeam Laser</v>
+      </c>
+      <c r="C327" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D327" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tribeam-laser/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B328" t="str">
+        <v>Fractional Laser Skin</v>
+      </c>
+      <c r="C328" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fractional-laser-skin/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B329" t="str">
+        <v>IPL Therapy</v>
+      </c>
+      <c r="C329" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ipl-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B330" t="str">
+        <v>Face Brightening Treatment</v>
+      </c>
+      <c r="C330" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-brightening-treatments-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B331" t="str">
+        <v>Acne Treatment</v>
+      </c>
+      <c r="C331" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-treatment-in-bangalore/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B332" t="str">
+        <v>Acne Scar Treatment</v>
+      </c>
+      <c r="C332" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D332" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-scar-treatment-in-gurgaon/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B333" t="str">
+        <v>Anti-Ageing Laser Treatment</v>
+      </c>
+      <c r="C333" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-ageing-laser-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B334" t="str">
+        <v>Pink Anti-Aging Treatment</v>
+      </c>
+      <c r="C334" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-anti-aging-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B335" t="str">
+        <v>Wrinkles Treatment</v>
+      </c>
+      <c r="C335" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/wrinkles-treatment-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B336" t="str">
+        <v>Crow's Feet Treatment</v>
+      </c>
+      <c r="C336" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/crows-feet-treatment-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B337" t="str">
+        <v>Dark Circles</v>
+      </c>
+      <c r="C337" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dark-circles/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B338" t="str">
+        <v>Tear Trough Treatment</v>
+      </c>
+      <c r="C338" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tear-trough-treatment-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B339" t="str">
+        <v>Under Eye Fillers Treatment</v>
+      </c>
+      <c r="C339" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/under-eye-fillers-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B340" t="str">
+        <v>Melasma</v>
+      </c>
+      <c r="C340" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/melasma/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B341" t="str">
+        <v>Rosacea</v>
+      </c>
+      <c r="C341" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/rosacea/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B342" t="str">
+        <v>Eczema Treatment</v>
+      </c>
+      <c r="C342" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eczema-treatment-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B343" t="str">
+        <v>Keratosis Pilaris</v>
+      </c>
+      <c r="C343" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D343" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/keratosis-pilaris/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B344" t="str">
+        <v>Sun / Age Spots</v>
+      </c>
+      <c r="C344" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sun-age-spots/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B345" t="str">
+        <v>Underarm Darkening</v>
+      </c>
+      <c r="C345" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D345" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/underarm-darkening/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B346" t="str">
+        <v>Scar Treatment</v>
+      </c>
+      <c r="C346" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/scar-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B347" t="str">
+        <v>Stretch Marks</v>
+      </c>
+      <c r="C347" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D347" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stretch-marks/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B348" t="str">
+        <v>Skin Whitening Treatment</v>
+      </c>
+      <c r="C348" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-whitening-treatment-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B349" t="str">
+        <v>MNRF Treatment</v>
+      </c>
+      <c r="C349" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mnrf-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B350" t="str">
+        <v>Dermarolling / Advanced Microneedling</v>
+      </c>
+      <c r="C350" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B351" t="str">
+        <v>Dermapen Treatment</v>
+      </c>
+      <c r="C351" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermapen-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B352" t="str">
+        <v>Collagen Induction Therapy</v>
+      </c>
+      <c r="C352" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/collagen-induction-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B353" t="str">
+        <v>Electrocautery Treatment</v>
+      </c>
+      <c r="C353" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D353" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/electrocautery-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B354" t="str">
+        <v>Permanent Beard Shaping</v>
+      </c>
+      <c r="C354" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/permanent-beard-shaping-treatment-in-mumbai/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>Facial</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Men's Grooming Treatments</v>
+      </c>
+      <c r="C355" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mens-grooming-treatments/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Lip Fillers</v>
+      </c>
+      <c r="C356" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lip-fillers/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B357" t="str">
+        <v>Anti-Wrinkle Injection (Facelift Filler)</v>
+      </c>
+      <c r="C357" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-wrinkle-injection-for-facelift-filler/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B358" t="str">
+        <v>Fat Lipolysis Injection</v>
+      </c>
+      <c r="C358" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fat-lipolysis-injection/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B359" t="str">
+        <v>Kenacort Injection</v>
+      </c>
+      <c r="C359" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/kenacort-injection/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B360" t="str">
+        <v>Tricort Injection</v>
+      </c>
+      <c r="C360" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tricort-injection/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B361" t="str">
+        <v>Hyaluron Pen (Needle-Free Filler)</v>
+      </c>
+      <c r="C361" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluron-pen-needle-free-filler/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B362" t="str">
+        <v>Hyaluronic Acid Therapy</v>
+      </c>
+      <c r="C362" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluronic-acid-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B363" t="str">
+        <v>Viscoderm Hydrobooster</v>
+      </c>
+      <c r="C363" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D363" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/viscoderm-hydrobooster/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B364" t="str">
+        <v>Dermal Thread Treatment</v>
+      </c>
+      <c r="C364" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D364" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermal-thread-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B365" t="str">
+        <v>Calecim Professional Brand</v>
+      </c>
+      <c r="C365" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D365" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-professional-brand/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B366" t="str">
+        <v>Eyebrow Transplant</v>
+      </c>
+      <c r="C366" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eyebrow-transplant/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B367" t="str">
+        <v>Regenera Activa Hair Treatment</v>
+      </c>
+      <c r="C367" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/regenera-activa-hair-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B368" t="str">
+        <v>Non-Surgical Hair Replacement</v>
+      </c>
+      <c r="C368" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D368" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-hair-replacement/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B369" t="str">
+        <v>Hairgen Booster</v>
+      </c>
+      <c r="C369" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hairgen-booster/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B370" t="str">
+        <v>PRP Hair Treatment</v>
+      </c>
+      <c r="C370" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-hair-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Advanced PRP Growth Factor Concentrate (GFC)</v>
+      </c>
+      <c r="C371" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B372" t="str">
+        <v>PRP Treatment</v>
+      </c>
+      <c r="C372" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D372" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-treatment-in-bangalore/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B373" t="str">
+        <v>Hair Fall Treatment</v>
+      </c>
+      <c r="C373" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hair-fall-treatment-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B374" t="str">
+        <v>Baldness Treatment</v>
+      </c>
+      <c r="C374" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D374" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/baldness-treatment-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B375" t="str">
+        <v>Alopecia Areata</v>
+      </c>
+      <c r="C375" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D375" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/alopecia-areata/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B376" t="str">
+        <v>QR-678 Neo Hair Growth</v>
+      </c>
+      <c r="C376" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D376" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/qr-678-neo-hair-growth-and-hair-qr-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>Hair</v>
+      </c>
+      <c r="B377" t="str">
+        <v>Morphyia Skin and Hair Treatment</v>
+      </c>
+      <c r="C377" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D377" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/morphyia-skin-and-hair-treatment/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>Lasar Hair Reduction</v>
+      </c>
+      <c r="B378" t="str">
+        <v>Soprano Ice Platinum</v>
+      </c>
+      <c r="C378" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D378" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-platinum/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>Lasar Hair Reduction</v>
+      </c>
+      <c r="B379" t="str">
+        <v>Soprano Ice Titanium</v>
+      </c>
+      <c r="C379" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-titanium/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>Drip</v>
+      </c>
+      <c r="B380" t="str">
+        <v>IV Drip Therapy</v>
+      </c>
+      <c r="C380" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D380" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/iv-drip-therapy-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>Drip</v>
+      </c>
+      <c r="B381" t="str">
+        <v>Stem Cell Therapy</v>
+      </c>
+      <c r="C381" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stem-cell-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>Drip</v>
+      </c>
+      <c r="B382" t="str">
+        <v>Hyperbaric Oxygen Therapy</v>
+      </c>
+      <c r="C382" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>Drip</v>
+      </c>
+      <c r="B383" t="str">
+        <v>Colon Hydrotherapy</v>
+      </c>
+      <c r="C383" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/colon-hydrotherapy-in-delhi/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B384" t="str">
+        <v>Pink Himalayan Salt Infrared Sauna</v>
+      </c>
+      <c r="C384" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-himalayan-salt-infrared-sauna/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B385" t="str">
+        <v>Spa Therapy</v>
+      </c>
+      <c r="C385" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D385" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/spa-therapy/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B386" t="str">
+        <v>Forest Essentials Body Spa</v>
+      </c>
+      <c r="C386" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D386" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/forest-essentials-body-spa/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B387" t="str">
+        <v>Deesse Pro LED Mask</v>
+      </c>
+      <c r="C387" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/deesse-pro-led-mask/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B388" t="str">
+        <v>Skin Perfect Oasis</v>
+      </c>
+      <c r="C388" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-perfect-oasis/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B389" t="str">
+        <v>Calecim Product</v>
+      </c>
+      <c r="C389" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-product/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B390" t="str">
+        <v>Bridal Makeover</v>
+      </c>
+      <c r="C390" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D390" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/bridal-makeover/. Not yet built.</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>Wellness (Uncategorized)</v>
+      </c>
+      <c r="B391" t="str">
+        <v>Groom Makeover</v>
+      </c>
+      <c r="C391" t="str">
+        <v>To Build (source available)</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/groom-makeover/. Not yet built.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D285"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D391"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Gynaecomastia, Eyebrow Transplant, Lip Fillers, Non-Surgical Face Lift, Regenera Activa, and Cryolipolysis brochures
Batch 2 of the sitemap-driven build-out, all scraped from their
isaacluxe.co pages (mechanism/technology, what's treated, benefits,
protocol, candidacy). No fabricated photos: Non-Surgical Face Lift and
Cryolipolysis had source images, but they were generic hero/device
shots rather than before/after pairs, so none were used.

Wired into index.html: Lip Fillers under Injectable; Gynaecomastia and
Cryolipolysis under Body Contouring; Non-Surgical Face Lift under Face
Lifting; Eyebrow Transplant and Regenera Activa under Anti Aging --
Hair & Scalp. brochure.xlsx updated with all 6 marked Completed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,10 +402,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D391"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="100.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4420,10 +4420,10 @@
         <v>Gynaecomastia</v>
       </c>
       <c r="C287" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D287" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/gynaecomastia/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html.</v>
       </c>
     </row>
     <row r="288">
@@ -4462,10 +4462,10 @@
         <v>Cryolipolysis</v>
       </c>
       <c r="C290" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D290" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryolipolysis-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html.</v>
       </c>
     </row>
     <row r="291">
@@ -4700,10 +4700,10 @@
         <v>Non-Surgical Face Lift</v>
       </c>
       <c r="C307" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D307" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-face-lift/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html.</v>
       </c>
     </row>
     <row r="308">
@@ -5386,10 +5386,10 @@
         <v>Lip Fillers</v>
       </c>
       <c r="C356" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D356" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lip-fillers/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html.</v>
       </c>
     </row>
     <row r="357">
@@ -5526,10 +5526,10 @@
         <v>Eyebrow Transplant</v>
       </c>
       <c r="C366" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D366" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eyebrow-transplant/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html.</v>
       </c>
     </row>
     <row r="367">
@@ -5540,10 +5540,10 @@
         <v>Regenera Activa Hair Treatment</v>
       </c>
       <c r="C367" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D367" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/regenera-activa-hair-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html.</v>
       </c>
     </row>
     <row r="368">

</xml_diff>

<commit_message>
Add CoolSculpting, Forma, Hair Transplant, GG Glow, Obagi Facial, and Mesotherapy brochures
Batch 3 of the sitemap-driven build-out. All scraped from their
isaacluxe.co pages; no fabricated photos (CoolSculpting's source images
were mechanism diagrams, not before/after, so none were used).

Confirmed "Ulthera Face Lifting" is the same treatment as the existing
Ultherapy brochure (verified via its own page copy) -- no duplicate
built, tracked as Completed against the existing file instead.
"Face Meso Therapy" and "Mesotherapy" point to the same source page --
one brochure covers both.

Wired into index.html: GG Glow, Obagi Facial, and Mesotherapy under
Facial; CoolSculpting under Body Contouring; Forma under Anti Aging;
Hair Transplant under Anti Aging -- Hair & Scalp. brochure.xlsx updated,
55 of 390 rows now Completed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -500,10 +500,10 @@
         <v>Forma</v>
       </c>
       <c r="C7" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D7" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/forma-skin-tightening-treatment-in-mumbai/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html.</v>
       </c>
     </row>
     <row r="8">
@@ -612,10 +612,10 @@
         <v>Cool Sculpt</v>
       </c>
       <c r="C15" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D15" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/coolsculpting/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html.</v>
       </c>
     </row>
     <row r="16">
@@ -906,10 +906,10 @@
         <v>Face Meso Therapy</v>
       </c>
       <c r="C36" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D36" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/mesotherapy/ [fuzzy]. Not yet built.</v>
+        <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built.</v>
       </c>
     </row>
     <row r="37">
@@ -1060,10 +1060,10 @@
         <v>Mesotherapy</v>
       </c>
       <c r="C47" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D47" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/mesotherapy/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html.</v>
       </c>
     </row>
     <row r="48">
@@ -2040,10 +2040,10 @@
         <v>GG Glow</v>
       </c>
       <c r="C117" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D117" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/gg-glow/ [exact]. Not yet built. [Duplicate name also appears at: row 118 (Facial)]</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
       </c>
     </row>
     <row r="118">
@@ -2054,10 +2054,10 @@
         <v>GG-glow</v>
       </c>
       <c r="C118" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D118" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/gg-glow/ [exact]. Not yet built. [Duplicate name also appears at: row 117 (Facial)]</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
       </c>
     </row>
     <row r="119">
@@ -2180,10 +2180,10 @@
         <v>Obagi</v>
       </c>
       <c r="C127" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D127" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/obagi-facial/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html.</v>
       </c>
     </row>
     <row r="128">
@@ -2544,10 +2544,10 @@
         <v>Hair Transplant</v>
       </c>
       <c r="C153" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D153" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/hair-transplant/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html.</v>
       </c>
     </row>
     <row r="154">
@@ -4658,10 +4658,10 @@
         <v>Ulthera Face Lifting</v>
       </c>
       <c r="C304" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D304" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ulthera-face-lifting/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting).</v>
       </c>
     </row>
     <row r="305">

</xml_diff>

<commit_message>
Add Vaginal Fillers, Liposuction Surgery, Non-Surgical Breast Lift, Aptos Thread Lift, Cosmelan Peel, and Skinfill Bacio brochures
Batch 4 of the sitemap-driven build-out. All scraped from their
isaacluxe.co pages; no fabricated photos (Non-Surgical Breast Lift and
Skinfill Bacio had source images, but neither was a before/after pair).

Wired into index.html: Vaginal Fillers, Liposuction Surgery, and
Non-Surgical Breast Lift under Body Contouring; Aptos Thread Lift under
Face Lifting; Cosmelan Peel under Peel; Skinfill Bacio under Injectable.
brochure.xlsx updated, 61 of 390 rows now Completed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -1746,10 +1746,10 @@
         <v>Aptos thread</v>
       </c>
       <c r="C96" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D96" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/aptos-thread-lifting/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html.</v>
       </c>
     </row>
     <row r="97">
@@ -3090,10 +3090,10 @@
         <v>Skinfill</v>
       </c>
       <c r="C192" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D192" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/skinfill-bacio-lip-booster/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html.</v>
       </c>
     </row>
     <row r="193">
@@ -3202,10 +3202,10 @@
         <v>COSMELAN</v>
       </c>
       <c r="C200" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D200" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/cosmelan-peel-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html.</v>
       </c>
     </row>
     <row r="201">
@@ -4434,10 +4434,10 @@
         <v>Liposuction Surgery</v>
       </c>
       <c r="C288" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D288" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liposuction-surgery/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html.</v>
       </c>
     </row>
     <row r="289">
@@ -4448,10 +4448,10 @@
         <v>Non-Surgical Breast Lift</v>
       </c>
       <c r="C289" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D289" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-breast-lift/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html.</v>
       </c>
     </row>
     <row r="290">
@@ -4574,10 +4574,10 @@
         <v>Vaginal Fillers</v>
       </c>
       <c r="C298" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D298" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/vaginal-fillers/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html.</v>
       </c>
     </row>
     <row r="299">

</xml_diff>

<commit_message>
Add Completed Date column to brochure.xlsx
Populated for all 61 Completed rows using each brochure's actual git
add-date (git log --diff-filter=A), not estimated from memory -- so
the dates are verifiable against commit history rather than guessed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -400,12 +400,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D391"/>
+  <dimension ref="A1:E391"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+    <col min="4" max="4" width="100.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,6 +422,9 @@
       <c r="D1" t="str">
         <v>Remarks</v>
       </c>
+      <c r="E1" t="str">
+        <v>Completed Date</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -449,6 +453,9 @@
       <c r="D3" t="str">
         <v>Brochure already exists: DermaFrac (dermafrac-brochure.html) [exact]</v>
       </c>
+      <c r="E3" t="str">
+        <v>2026-07-23</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -463,6 +470,9 @@
       <c r="D4" t="str">
         <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [exact]</v>
       </c>
+      <c r="E4" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -505,6 +515,9 @@
       <c r="D7" t="str">
         <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html.</v>
       </c>
+      <c r="E7" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -519,6 +532,9 @@
       <c r="D8" t="str">
         <v>Brochure already exists: Morpheus 8 (morpheus-8-treatment-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E8" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -547,6 +563,9 @@
       <c r="D10" t="str">
         <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 157 (Hair)]</v>
       </c>
+      <c r="E10" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -603,6 +622,9 @@
       <c r="D14" t="str">
         <v>Brochure already exists: Artiqa (artiqa-brochure.html) [exact]</v>
       </c>
+      <c r="E14" t="str">
+        <v>2026-07-22</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -617,6 +639,9 @@
       <c r="D15" t="str">
         <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html.</v>
       </c>
+      <c r="E15" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -645,6 +670,9 @@
       <c r="D17" t="str">
         <v>Brochure already exists: Emsculpt NEO (emsculpt-neo-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E17" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -659,6 +687,9 @@
       <c r="D18" t="str">
         <v>Brochure already exists: Exilis Elite (exilis-elite-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E18" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -687,6 +718,9 @@
       <c r="D20" t="str">
         <v>Brochure already exists: Lymphatic Drainage (lymphatic-drainage-brochure.html) [exact]</v>
       </c>
+      <c r="E20" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -911,6 +945,9 @@
       <c r="D36" t="str">
         <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built.</v>
       </c>
+      <c r="E36" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1065,6 +1102,9 @@
       <c r="D47" t="str">
         <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html.</v>
       </c>
+      <c r="E47" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1079,6 +1119,9 @@
       <c r="D48" t="str">
         <v>Brochure already exists: Microblading (microblading-brochure.html) [exact]</v>
       </c>
+      <c r="E48" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1191,6 +1234,9 @@
       <c r="D56" t="str">
         <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html.</v>
       </c>
+      <c r="E56" t="str">
+        <v>2026-06-12</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -1219,6 +1265,9 @@
       <c r="D58" t="str">
         <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact]</v>
       </c>
+      <c r="E58" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -1275,6 +1324,9 @@
       <c r="D62" t="str">
         <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact]</v>
       </c>
+      <c r="E62" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1331,6 +1383,9 @@
       <c r="D66" t="str">
         <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact]</v>
       </c>
+      <c r="E66" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -1387,6 +1442,9 @@
       <c r="D70" t="str">
         <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E70" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -1401,6 +1459,9 @@
       <c r="D71" t="str">
         <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact]</v>
       </c>
+      <c r="E71" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -1443,6 +1504,9 @@
       <c r="D74" t="str">
         <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact]</v>
       </c>
+      <c r="E74" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -1681,6 +1745,9 @@
       <c r="D91" t="str">
         <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact]</v>
       </c>
+      <c r="E91" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -1737,6 +1804,9 @@
       <c r="D95" t="str">
         <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact]</v>
       </c>
+      <c r="E95" t="str">
+        <v>2026-07-15</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -1751,6 +1821,9 @@
       <c r="D96" t="str">
         <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html.</v>
       </c>
+      <c r="E96" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -1765,6 +1838,9 @@
       <c r="D97" t="str">
         <v>Brochure already exists: EmFace (emface-treatment-brochure.html) [exact]</v>
       </c>
+      <c r="E97" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -1793,6 +1869,9 @@
       <c r="D99" t="str">
         <v>Brochure already exists: Ultherapy (ultherapy-treatment-brochure.html) [exact]</v>
       </c>
+      <c r="E99" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -1877,6 +1956,9 @@
       <c r="D105" t="str">
         <v>Brochure already exists: Carbon Facial (carbon-facial-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E105" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -1989,6 +2071,9 @@
       <c r="D113" t="str">
         <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html.</v>
       </c>
+      <c r="E113" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -2045,6 +2130,9 @@
       <c r="D117" t="str">
         <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
       </c>
+      <c r="E117" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -2059,6 +2147,9 @@
       <c r="D118" t="str">
         <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
       </c>
+      <c r="E118" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -2115,6 +2206,9 @@
       <c r="D122" t="str">
         <v>Brochure already exists: Laser Toning (laser-toning-brochure.html) [exact]</v>
       </c>
+      <c r="E122" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -2185,6 +2279,9 @@
       <c r="D127" t="str">
         <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html.</v>
       </c>
+      <c r="E127" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -2227,6 +2324,9 @@
       <c r="D130" t="str">
         <v>Brochure already exists: Photo Facial (photo-facial-brochure.html) [exact]</v>
       </c>
+      <c r="E130" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -2283,6 +2383,9 @@
       <c r="D134" t="str">
         <v>Brochure already exists: Retix C (retix-c-brochure.html) [exact]</v>
       </c>
+      <c r="E134" t="str">
+        <v>2026-07-16</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -2352,6 +2455,9 @@
       </c>
       <c r="D139" t="str">
         <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html.</v>
+      </c>
+      <c r="E139" t="str">
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="140">
@@ -2423,6 +2529,9 @@
       <c r="D144" t="str">
         <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E144" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -2549,6 +2658,9 @@
       <c r="D153" t="str">
         <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html.</v>
       </c>
+      <c r="E153" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -2577,6 +2689,9 @@
       <c r="D155" t="str">
         <v>Brochure already exists: Luxe Keravive (keravive-brochure.html) [exact]</v>
       </c>
+      <c r="E155" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -2605,6 +2720,9 @@
       <c r="D157" t="str">
         <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 10 (Anti Aging)]</v>
       </c>
+      <c r="E157" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -2703,6 +2821,9 @@
       <c r="D164" t="str">
         <v>Brochure already exists: HydraFacial MD Elite (hydrafacial-md-elite-brocher.html) [fuzzy]</v>
       </c>
+      <c r="E164" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -2801,6 +2922,9 @@
       <c r="D171" t="str">
         <v>Brochure already exists: Aquagold Fine Touch (aquagold-fine-touch.html) [fuzzy]</v>
       </c>
+      <c r="E171" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -2857,6 +2981,9 @@
       <c r="D175" t="str">
         <v>Brochure already exists: Botox (botox-treatment-brochure.html) [exact]</v>
       </c>
+      <c r="E175" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -2997,6 +3124,9 @@
       <c r="D185" t="str">
         <v>Brochure already exists: Polypeptide (polypeptide-brochure.html) [exact]</v>
       </c>
+      <c r="E185" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -3025,6 +3155,9 @@
       <c r="D187" t="str">
         <v>Brochure already exists: Profhilo (profhilo-brochure.html) [exact]</v>
       </c>
+      <c r="E187" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
@@ -3039,6 +3172,9 @@
       <c r="D188" t="str">
         <v>Brochure already exists: Rejuran (rejuran-brochure.html) [exact]</v>
       </c>
+      <c r="E188" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
@@ -3053,6 +3189,9 @@
       <c r="D189" t="str">
         <v>Brochure already exists: Rejuran (rejuran-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E189" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -3067,6 +3206,9 @@
       <c r="D190" t="str">
         <v>Brochure already exists: Restylane (restylane-brochure.html) [exact]</v>
       </c>
+      <c r="E190" t="str">
+        <v>2026-07-23</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
@@ -3095,6 +3237,9 @@
       <c r="D192" t="str">
         <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html.</v>
       </c>
+      <c r="E192" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -3165,6 +3310,9 @@
       <c r="D197" t="str">
         <v>Built from bioretherapy.pdf (BioRePeelCl3 FND + Body variants, real before/after photos). Brochure: biorepeel-brochure.html.</v>
       </c>
+      <c r="E197" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
@@ -3207,6 +3355,9 @@
       <c r="D200" t="str">
         <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html.</v>
       </c>
+      <c r="E200" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
@@ -3305,6 +3456,9 @@
       <c r="D207" t="str">
         <v>Brochure already exists: House of Peels (house-of-peels-brochure.html) [fuzzy]</v>
       </c>
+      <c r="E207" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -3375,6 +3529,9 @@
       <c r="D212" t="str">
         <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html.</v>
       </c>
+      <c r="E212" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -4425,6 +4582,9 @@
       <c r="D287" t="str">
         <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html.</v>
       </c>
+      <c r="E287" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
@@ -4439,6 +4599,9 @@
       <c r="D288" t="str">
         <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html.</v>
       </c>
+      <c r="E288" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
@@ -4453,6 +4616,9 @@
       <c r="D289" t="str">
         <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html.</v>
       </c>
+      <c r="E289" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
@@ -4467,6 +4633,9 @@
       <c r="D290" t="str">
         <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html.</v>
       </c>
+      <c r="E290" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
@@ -4579,6 +4748,9 @@
       <c r="D298" t="str">
         <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html.</v>
       </c>
+      <c r="E298" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
@@ -4663,6 +4835,9 @@
       <c r="D304" t="str">
         <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting).</v>
       </c>
+      <c r="E304" t="str">
+        <v>2026-06-26</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
@@ -4705,6 +4880,9 @@
       <c r="D307" t="str">
         <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html.</v>
       </c>
+      <c r="E307" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
@@ -5391,6 +5569,9 @@
       <c r="D356" t="str">
         <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html.</v>
       </c>
+      <c r="E356" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
@@ -5531,6 +5712,9 @@
       <c r="D366" t="str">
         <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html.</v>
       </c>
+      <c r="E366" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
@@ -5545,6 +5729,9 @@
       <c r="D367" t="str">
         <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html.</v>
       </c>
+      <c r="E367" t="str">
+        <v>2026-07-24</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
@@ -5884,7 +6071,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E391"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add X-Wave, Med Contour, Derma Roller, Hyperbaric Oxygen Chamber, Cryo Facial, Valmont Facial, and Vampire Facial brochures
Batch 5 of the sitemap-driven build-out. All scraped from their
isaacluxe.co pages; no fabricated photos (Med Contour had banner/
diagram images only, not before/after, so none were used).

Wired into index.html: Derma Roller, Cryo Facial, Valmont Facial, and
Vampire Facial under Facial; X-Wave and Med Contour under Body
Contouring; Hyperbaric Oxygen Chamber under Drip Therapy as the
closest fit for a general wellness/recovery treatment (flagged in
brochure.xlsx remarks). brochure.xlsx updated, both "X WAve" and
"X-Wave" duplicate rows marked against the same file.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,11 +402,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E391"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="100.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,6 +438,9 @@
       <c r="D2" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content. [Duplicate name also appears at: row 159 (Hair)]</v>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -487,6 +489,9 @@
       <c r="D5" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -501,6 +506,9 @@
       <c r="D6" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -549,6 +557,9 @@
       <c r="D9" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -580,6 +591,9 @@
       <c r="D11" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -594,6 +608,9 @@
       <c r="D12" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -608,6 +625,9 @@
       <c r="D13" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -656,6 +676,9 @@
       <c r="D16" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -704,6 +727,9 @@
       <c r="D19" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/intragen-skin-tightening-treatment/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -730,10 +756,13 @@
         <v>Medcontour</v>
       </c>
       <c r="C21" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D21" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/medcontour-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html.</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -749,6 +778,9 @@
       <c r="D22" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -763,6 +795,9 @@
       <c r="D23" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -777,6 +812,9 @@
       <c r="D24" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -791,6 +829,9 @@
       <c r="D25" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -805,6 +846,9 @@
       <c r="D26" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -819,6 +863,9 @@
       <c r="D27" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -833,6 +880,9 @@
       <c r="D28" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -842,10 +892,13 @@
         <v>X WAve</v>
       </c>
       <c r="C29" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D29" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/x-wave/ [exact]. Not yet built. [Duplicate name also appears at: row 30 (Body Contouring)]</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -856,10 +909,13 @@
         <v>X-Wave</v>
       </c>
       <c r="C30" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D30" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/x-wave/ [exact]. Not yet built. [Duplicate name also appears at: row 29 (Body Contouring)]</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -875,6 +931,9 @@
       <c r="D31" t="str">
         <v>Generic spa/personal-care service (not a documented clinical treatment) — flagging as out of scope, let me know if this should be treated differently.</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -889,6 +948,9 @@
       <c r="D32" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -903,6 +965,9 @@
       <c r="D33" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -917,6 +982,9 @@
       <c r="D34" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -926,10 +994,13 @@
         <v>Dermaroller</v>
       </c>
       <c r="C35" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D35" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/derma-roller-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html.</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -962,6 +1033,9 @@
       <c r="D37" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -976,6 +1050,9 @@
       <c r="D38" t="str">
         <v>Booking/administrative line item, not a treatment — no brochure appropriate.</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -990,6 +1067,9 @@
       <c r="D39" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1004,6 +1084,9 @@
       <c r="D40" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1018,6 +1101,9 @@
       <c r="D41" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1032,6 +1118,9 @@
       <c r="D42" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1046,6 +1135,9 @@
       <c r="D43" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1060,6 +1152,9 @@
       <c r="D44" t="str">
         <v>Generic spa/personal-care service (not a documented clinical treatment) — flagging as out of scope, let me know if this should be treated differently.</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1074,6 +1169,9 @@
       <c r="D45" t="str">
         <v>Booking/administrative line item, not a treatment — no brochure appropriate.</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1088,6 +1186,9 @@
       <c r="D46" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1136,6 +1237,9 @@
       <c r="D49" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1150,6 +1254,9 @@
       <c r="D50" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1159,10 +1266,13 @@
         <v>Oxygen Chamber</v>
       </c>
       <c r="C51" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D51" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/hyperbaric-oxygen-chamber/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html.</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -1178,6 +1288,9 @@
       <c r="D52" t="str">
         <v>Booking/administrative line item, not a treatment — no brochure appropriate.</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1192,6 +1305,9 @@
       <c r="D53" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/get-hair-free-smooth-skin-with-laser-hair-removal-technology/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1206,6 +1322,9 @@
       <c r="D54" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content. [Duplicate name also appears at: row 193 (Lasar Hair Reduction)]</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1220,6 +1339,9 @@
       <c r="D55" t="str">
         <v>Booking/administrative line item, not a treatment — no brochure appropriate.</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -1251,6 +1373,9 @@
       <c r="D57" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1282,6 +1407,9 @@
       <c r="D59" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -1296,6 +1424,9 @@
       <c r="D60" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1310,6 +1441,9 @@
       <c r="D61" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -1341,6 +1475,9 @@
       <c r="D63" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1355,6 +1492,9 @@
       <c r="D64" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1369,6 +1509,9 @@
       <c r="D65" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1400,6 +1543,9 @@
       <c r="D67" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -1414,6 +1560,9 @@
       <c r="D68" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -1428,6 +1577,9 @@
       <c r="D69" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -1476,6 +1628,9 @@
       <c r="D72" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -1490,6 +1645,9 @@
       <c r="D73" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -1521,6 +1679,9 @@
       <c r="D75" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -1535,6 +1696,9 @@
       <c r="D76" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -1549,6 +1713,9 @@
       <c r="D77" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -1563,6 +1730,9 @@
       <c r="D78" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -1577,6 +1747,9 @@
       <c r="D79" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -1591,6 +1764,9 @@
       <c r="D80" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -1605,6 +1781,9 @@
       <c r="D81" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -1619,6 +1798,9 @@
       <c r="D82" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -1633,6 +1815,9 @@
       <c r="D83" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -1647,6 +1832,9 @@
       <c r="D84" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -1661,6 +1849,9 @@
       <c r="D85" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -1675,6 +1866,9 @@
       <c r="D86" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -1689,6 +1883,9 @@
       <c r="D87" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -1703,6 +1900,9 @@
       <c r="D88" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -1717,6 +1917,9 @@
       <c r="D89" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -1731,6 +1934,9 @@
       <c r="D90" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -1762,6 +1968,9 @@
       <c r="D92" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -1776,6 +1985,9 @@
       <c r="D93" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -1790,6 +2002,9 @@
       <c r="D94" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -1855,6 +2070,9 @@
       <c r="D98" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -1886,6 +2104,9 @@
       <c r="D100" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -1900,6 +2121,9 @@
       <c r="D101" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -1914,6 +2138,9 @@
       <c r="D102" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -1928,6 +2155,9 @@
       <c r="D103" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/biologique/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -1942,6 +2172,9 @@
       <c r="D104" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -1973,6 +2206,9 @@
       <c r="D106" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -1987,6 +2223,9 @@
       <c r="D107" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -2001,6 +2240,9 @@
       <c r="D108" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -2010,10 +2252,13 @@
         <v>Cryo Facial</v>
       </c>
       <c r="C109" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D109" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/cryo-facial-in-mumbai/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html.</v>
+      </c>
+      <c r="E109" t="str">
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -2029,6 +2274,9 @@
       <c r="D110" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -2043,6 +2291,9 @@
       <c r="D111" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/jet-peel-facial-or-dolphin-facial/ [fuzzy]. Not yet built. [Duplicate name also appears at: row 145 (Hair)]</v>
       </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -2057,6 +2308,9 @@
       <c r="D112" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -2088,6 +2342,9 @@
       <c r="D114" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -2102,6 +2359,9 @@
       <c r="D115" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -2116,6 +2376,9 @@
       <c r="D116" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -2164,6 +2427,9 @@
       <c r="D119" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -2178,6 +2444,9 @@
       <c r="D120" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/ice-facial-treatment/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -2192,6 +2461,9 @@
       <c r="D121" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -2223,6 +2495,9 @@
       <c r="D123" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/love-light-fusion-facial/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E123" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -2237,6 +2512,9 @@
       <c r="D124" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -2251,6 +2529,9 @@
       <c r="D125" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -2265,6 +2546,9 @@
       <c r="D126" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/oasis-facial-treatment/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -2296,6 +2580,9 @@
       <c r="D128" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/oxygeneo-facial-best-oxygen-facial/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -2310,6 +2597,9 @@
       <c r="D129" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E129" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -2341,6 +2631,9 @@
       <c r="D131" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E131" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -2355,6 +2648,9 @@
       <c r="D132" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E132" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -2369,6 +2665,9 @@
       <c r="D133" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E133" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -2400,6 +2699,9 @@
       <c r="D135" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/salmon-dna-pdrn-facial/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E135" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -2414,6 +2716,9 @@
       <c r="D136" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E136" t="str">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -2428,6 +2733,9 @@
       <c r="D137" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/signature-facial-treatment-3/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E137" t="str">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -2442,6 +2750,9 @@
       <c r="D138" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E138" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -2473,6 +2784,9 @@
       <c r="D140" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/v-bianco-skin-lightening-treatment/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E140" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -2487,6 +2801,9 @@
       <c r="D141" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/v-carbon-treatment/ [fuzzy]. Not yet built.</v>
       </c>
+      <c r="E141" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -2496,10 +2813,13 @@
         <v>Valmont Facial</v>
       </c>
       <c r="C142" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D142" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/valmont-facial/ [exact]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html.</v>
+      </c>
+      <c r="E142" t="str">
+        <v/>
       </c>
     </row>
     <row r="143">
@@ -2515,6 +2835,9 @@
       <c r="D143" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E143" t="str">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -2546,6 +2869,9 @@
       <c r="D145" t="str">
         <v>Live site page found for scraping: https://www.isaacluxe.co/jet-peel-facial-or-dolphin-facial/ [fuzzy]. Not yet built. [Duplicate name also appears at: row 111 (Facial)]</v>
       </c>
+      <c r="E145" t="str">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -2560,6 +2886,9 @@
       <c r="D146" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E146" t="str">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -2574,6 +2903,9 @@
       <c r="D147" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E147" t="str">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -2588,6 +2920,9 @@
       <c r="D148" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E148" t="str">
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -2602,6 +2937,9 @@
       <c r="D149" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E149" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -2616,6 +2954,9 @@
       <c r="D150" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E150" t="str">
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -2630,6 +2971,9 @@
       <c r="D151" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E151" t="str">
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -2644,6 +2988,9 @@
       <c r="D152" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E152" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -2675,6 +3022,9 @@
       <c r="D154" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -2706,6 +3056,9 @@
       <c r="D156" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E156" t="str">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -2737,6 +3090,9 @@
       <c r="D158" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E158" t="str">
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -2751,6 +3107,9 @@
       <c r="D159" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content. [Duplicate name also appears at: row 2 (Anti Aging)]</v>
       </c>
+      <c r="E159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -2765,6 +3124,9 @@
       <c r="D160" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E160" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -2779,6 +3141,9 @@
       <c r="D161" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E161" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -2793,6 +3158,9 @@
       <c r="D162" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E162" t="str">
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -2807,6 +3175,9 @@
       <c r="D163" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E163" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -2838,6 +3209,9 @@
       <c r="D165" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E165" t="str">
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -2852,6 +3226,9 @@
       <c r="D166" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E166" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -2866,6 +3243,9 @@
       <c r="D167" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E167" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -2880,6 +3260,9 @@
       <c r="D168" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E168" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -2894,6 +3277,9 @@
       <c r="D169" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E169" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -2908,6 +3294,9 @@
       <c r="D170" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E170" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -2939,6 +3328,9 @@
       <c r="D172" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -2953,6 +3345,9 @@
       <c r="D173" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E173" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -2967,6 +3362,9 @@
       <c r="D174" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E174" t="str">
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -2998,6 +3396,9 @@
       <c r="D176" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E176" t="str">
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -3012,6 +3413,9 @@
       <c r="D177" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E177" t="str">
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -3026,6 +3430,9 @@
       <c r="D178" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E178" t="str">
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
@@ -3040,6 +3447,9 @@
       <c r="D179" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E179" t="str">
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -3054,6 +3464,9 @@
       <c r="D180" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E180" t="str">
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
@@ -3068,6 +3481,9 @@
       <c r="D181" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E181" t="str">
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -3082,6 +3498,9 @@
       <c r="D182" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E182" t="str">
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -3096,6 +3515,9 @@
       <c r="D183" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E183" t="str">
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -3110,6 +3532,9 @@
       <c r="D184" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E184" t="str">
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -3141,6 +3566,9 @@
       <c r="D186" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E186" t="str">
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
@@ -3223,6 +3651,9 @@
       <c r="D191" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E191" t="str">
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -3254,6 +3685,9 @@
       <c r="D193" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content. [Duplicate name also appears at: row 54 (Common)]</v>
       </c>
+      <c r="E193" t="str">
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
@@ -3268,6 +3702,9 @@
       <c r="D194" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E194" t="str">
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -3282,6 +3719,9 @@
       <c r="D195" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E195" t="str">
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -3296,6 +3736,9 @@
       <c r="D196" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E196" t="str">
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -3327,6 +3770,9 @@
       <c r="D198" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E198" t="str">
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -3341,6 +3787,9 @@
       <c r="D199" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E199" t="str">
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
@@ -3372,6 +3821,9 @@
       <c r="D201" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E201" t="str">
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
@@ -3386,6 +3838,9 @@
       <c r="D202" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E202" t="str">
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -3400,6 +3855,9 @@
       <c r="D203" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E203" t="str">
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
@@ -3414,6 +3872,9 @@
       <c r="D204" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E204" t="str">
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -3428,6 +3889,9 @@
       <c r="D205" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E205" t="str">
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -3442,6 +3906,9 @@
       <c r="D206" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E206" t="str">
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -3473,6 +3940,9 @@
       <c r="D208" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E208" t="str">
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -3487,6 +3957,9 @@
       <c r="D209" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E209" t="str">
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -3501,6 +3974,9 @@
       <c r="D210" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E210" t="str">
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -3515,6 +3991,9 @@
       <c r="D211" t="str">
         <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
       </c>
+      <c r="E211" t="str">
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -3546,6 +4025,9 @@
       <c r="D213" t="str">
         <v>Blank row.</v>
       </c>
+      <c r="E213" t="str">
+        <v/>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -3560,6 +4042,9 @@
       <c r="D214" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E214" t="str">
+        <v/>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -3574,6 +4059,9 @@
       <c r="D215" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E215" t="str">
+        <v/>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -3588,6 +4076,9 @@
       <c r="D216" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E216" t="str">
+        <v/>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -3602,6 +4093,9 @@
       <c r="D217" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E217" t="str">
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -3616,6 +4110,9 @@
       <c r="D218" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E218" t="str">
+        <v/>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -3630,6 +4127,9 @@
       <c r="D219" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E219" t="str">
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -3644,6 +4144,9 @@
       <c r="D220" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E220" t="str">
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -3658,6 +4161,9 @@
       <c r="D221" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E221" t="str">
+        <v/>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -3672,6 +4178,9 @@
       <c r="D222" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E222" t="str">
+        <v/>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -3686,6 +4195,9 @@
       <c r="D223" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E223" t="str">
+        <v/>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -3700,6 +4212,9 @@
       <c r="D224" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E224" t="str">
+        <v/>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -3714,6 +4229,9 @@
       <c r="D225" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E225" t="str">
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -3728,6 +4246,9 @@
       <c r="D226" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E226" t="str">
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -3742,6 +4263,9 @@
       <c r="D227" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E227" t="str">
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -3756,6 +4280,9 @@
       <c r="D228" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E228" t="str">
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -3770,6 +4297,9 @@
       <c r="D229" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E229" t="str">
+        <v/>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -3784,6 +4314,9 @@
       <c r="D230" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E230" t="str">
+        <v/>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -3798,6 +4331,9 @@
       <c r="D231" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E231" t="str">
+        <v/>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -3812,6 +4348,9 @@
       <c r="D232" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E232" t="str">
+        <v/>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -3826,6 +4365,9 @@
       <c r="D233" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E233" t="str">
+        <v/>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -3840,6 +4382,9 @@
       <c r="D234" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E234" t="str">
+        <v/>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -3854,6 +4399,9 @@
       <c r="D235" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E235" t="str">
+        <v/>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -3868,6 +4416,9 @@
       <c r="D236" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E236" t="str">
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -3882,6 +4433,9 @@
       <c r="D237" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E237" t="str">
+        <v/>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -3896,6 +4450,9 @@
       <c r="D238" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E238" t="str">
+        <v/>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -3910,6 +4467,9 @@
       <c r="D239" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E239" t="str">
+        <v/>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -3924,6 +4484,9 @@
       <c r="D240" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E240" t="str">
+        <v/>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -3938,6 +4501,9 @@
       <c r="D241" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E241" t="str">
+        <v/>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -3952,6 +4518,9 @@
       <c r="D242" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E242" t="str">
+        <v/>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -3966,6 +4535,9 @@
       <c r="D243" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E243" t="str">
+        <v/>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
@@ -3980,6 +4552,9 @@
       <c r="D244" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E244" t="str">
+        <v/>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
@@ -3994,6 +4569,9 @@
       <c r="D245" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E245" t="str">
+        <v/>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
@@ -4008,6 +4586,9 @@
       <c r="D246" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E246" t="str">
+        <v/>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
@@ -4022,6 +4603,9 @@
       <c r="D247" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E247" t="str">
+        <v/>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
@@ -4036,6 +4620,9 @@
       <c r="D248" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E248" t="str">
+        <v/>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
@@ -4050,6 +4637,9 @@
       <c r="D249" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E249" t="str">
+        <v/>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
@@ -4064,6 +4654,9 @@
       <c r="D250" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E250" t="str">
+        <v/>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
@@ -4078,6 +4671,9 @@
       <c r="D251" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E251" t="str">
+        <v/>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
@@ -4092,6 +4688,9 @@
       <c r="D252" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E252" t="str">
+        <v/>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
@@ -4106,6 +4705,9 @@
       <c r="D253" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E253" t="str">
+        <v/>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
@@ -4120,6 +4722,9 @@
       <c r="D254" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E254" t="str">
+        <v/>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
@@ -4134,6 +4739,9 @@
       <c r="D255" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E255" t="str">
+        <v/>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
@@ -4148,6 +4756,9 @@
       <c r="D256" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E256" t="str">
+        <v/>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
@@ -4162,6 +4773,9 @@
       <c r="D257" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E257" t="str">
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
@@ -4176,6 +4790,9 @@
       <c r="D258" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E258" t="str">
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
@@ -4190,6 +4807,9 @@
       <c r="D259" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E259" t="str">
+        <v/>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
@@ -4204,6 +4824,9 @@
       <c r="D260" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E260" t="str">
+        <v/>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
@@ -4218,6 +4841,9 @@
       <c r="D261" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E261" t="str">
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
@@ -4232,6 +4858,9 @@
       <c r="D262" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E262" t="str">
+        <v/>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
@@ -4246,6 +4875,9 @@
       <c r="D263" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E263" t="str">
+        <v/>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
@@ -4260,6 +4892,9 @@
       <c r="D264" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E264" t="str">
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
@@ -4274,6 +4909,9 @@
       <c r="D265" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E265" t="str">
+        <v/>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
@@ -4288,6 +4926,9 @@
       <c r="D266" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E266" t="str">
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
@@ -4302,6 +4943,9 @@
       <c r="D267" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E267" t="str">
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
@@ -4316,6 +4960,9 @@
       <c r="D268" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E268" t="str">
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
@@ -4330,6 +4977,9 @@
       <c r="D269" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E269" t="str">
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
@@ -4344,6 +4994,9 @@
       <c r="D270" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E270" t="str">
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
@@ -4358,6 +5011,9 @@
       <c r="D271" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E271" t="str">
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
@@ -4372,6 +5028,9 @@
       <c r="D272" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E272" t="str">
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
@@ -4386,6 +5045,9 @@
       <c r="D273" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E273" t="str">
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
@@ -4400,6 +5062,9 @@
       <c r="D274" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E274" t="str">
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
@@ -4414,6 +5079,9 @@
       <c r="D275" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E275" t="str">
+        <v/>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
@@ -4428,6 +5096,9 @@
       <c r="D276" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E276" t="str">
+        <v/>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
@@ -4442,6 +5113,9 @@
       <c r="D277" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E277" t="str">
+        <v/>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
@@ -4456,6 +5130,9 @@
       <c r="D278" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate. [Duplicate name also appears at: row 279 (Salon)]</v>
       </c>
+      <c r="E278" t="str">
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
@@ -4470,6 +5147,9 @@
       <c r="D279" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate. [Duplicate name also appears at: row 278 (Salon)]</v>
       </c>
+      <c r="E279" t="str">
+        <v/>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
@@ -4484,6 +5164,9 @@
       <c r="D280" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E280" t="str">
+        <v/>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
@@ -4498,6 +5181,9 @@
       <c r="D281" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E281" t="str">
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
@@ -4512,6 +5198,9 @@
       <c r="D282" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E282" t="str">
+        <v/>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
@@ -4526,6 +5215,9 @@
       <c r="D283" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E283" t="str">
+        <v/>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
@@ -4540,6 +5232,9 @@
       <c r="D284" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E284" t="str">
+        <v/>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
@@ -4554,6 +5249,9 @@
       <c r="D285" t="str">
         <v>Salon/personal-care service, not a clinical aesthetic treatment — no brochure appropriate.</v>
       </c>
+      <c r="E285" t="str">
+        <v/>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
@@ -4566,6 +5264,9 @@
         <v/>
       </c>
       <c r="D286" t="str">
+        <v/>
+      </c>
+      <c r="E286" t="str">
         <v/>
       </c>
     </row>
@@ -4650,6 +5351,9 @@
       <c r="D291" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/instasculpt/. Not yet built.</v>
       </c>
+      <c r="E291" t="str">
+        <v/>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
@@ -4664,6 +5368,9 @@
       <c r="D292" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-sculpt/. Not yet built.</v>
       </c>
+      <c r="E292" t="str">
+        <v/>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
@@ -4678,6 +5385,9 @@
       <c r="D293" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-proportion/. Not yet built.</v>
       </c>
+      <c r="E293" t="str">
+        <v/>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
@@ -4692,6 +5402,9 @@
       <c r="D294" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tummy-tightening/. Not yet built.</v>
       </c>
+      <c r="E294" t="str">
+        <v/>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
@@ -4706,6 +5419,9 @@
       <c r="D295" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tight-pro/. Not yet built.</v>
       </c>
+      <c r="E295" t="str">
+        <v/>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
@@ -4720,6 +5436,9 @@
       <c r="D296" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ballancer-pro-treatment/. Not yet built.</v>
       </c>
+      <c r="E296" t="str">
+        <v/>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
@@ -4734,6 +5453,9 @@
       <c r="D297" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/femme-360-vaginal-tightening/. Not yet built.</v>
       </c>
+      <c r="E297" t="str">
+        <v/>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
@@ -4765,6 +5487,9 @@
       <c r="D299" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/multipolar-radio-frequency-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E299" t="str">
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
@@ -4779,6 +5504,9 @@
       <c r="D300" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3/. Not yet built.</v>
       </c>
+      <c r="E300" t="str">
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
@@ -4793,6 +5521,9 @@
       <c r="D301" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-tightening-treatment-in-vasant-vihar/. Not yet built.</v>
       </c>
+      <c r="E301" t="str">
+        <v/>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
@@ -4807,6 +5538,9 @@
       <c r="D302" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sculptone-plus/. Not yet built.</v>
       </c>
+      <c r="E302" t="str">
+        <v/>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
@@ -4821,6 +5555,9 @@
       <c r="D303" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cool-tech/. Not yet built.</v>
       </c>
+      <c r="E303" t="str">
+        <v/>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
@@ -4852,6 +5589,9 @@
       <c r="D305" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/thread-face-lift-treatment/. Not yet built.</v>
       </c>
+      <c r="E305" t="str">
+        <v/>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
@@ -4866,6 +5606,9 @@
       <c r="D306" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liquid-facelift-treatment/. Not yet built.</v>
       </c>
+      <c r="E306" t="str">
+        <v/>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
@@ -4897,6 +5640,9 @@
       <c r="D308" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sygma-lift-treatment-in-gurgaon/. Not yet built.</v>
       </c>
+      <c r="E308" t="str">
+        <v/>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
@@ -4911,6 +5657,9 @@
       <c r="D309" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/4-d-lift/. Not yet built.</v>
       </c>
+      <c r="E309" t="str">
+        <v/>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
@@ -4925,6 +5674,9 @@
       <c r="D310" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-lift-filler-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E310" t="str">
+        <v/>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
@@ -4939,6 +5691,9 @@
       <c r="D311" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/square-jaw-treatment-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E311" t="str">
+        <v/>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
@@ -4953,6 +5708,9 @@
       <c r="D312" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/poppy-chin-treatment-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E312" t="str">
+        <v/>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
@@ -4967,6 +5725,9 @@
       <c r="D313" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/br-facial/. Not yet built.</v>
       </c>
+      <c r="E313" t="str">
+        <v/>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
@@ -4981,6 +5742,9 @@
       <c r="D314" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eve-lom-facial/. Not yet built.</v>
       </c>
+      <c r="E314" t="str">
+        <v/>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
@@ -4995,6 +5759,9 @@
       <c r="D315" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/o2derm-facial/. Not yet built.</v>
       </c>
+      <c r="E315" t="str">
+        <v/>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
@@ -5009,6 +5776,9 @@
       <c r="D316" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/exo-glow-treatment/. Not yet built.</v>
       </c>
+      <c r="E316" t="str">
+        <v/>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
@@ -5023,6 +5793,9 @@
       <c r="D317" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/meso-glow/. Not yet built.</v>
       </c>
+      <c r="E317" t="str">
+        <v/>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
@@ -5037,6 +5810,9 @@
       <c r="D318" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-face/. Not yet built.</v>
       </c>
+      <c r="E318" t="str">
+        <v/>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
@@ -5051,6 +5827,9 @@
       <c r="D319" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-eyes/. Not yet built.</v>
       </c>
+      <c r="E319" t="str">
+        <v/>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
@@ -5065,6 +5844,9 @@
       <c r="D320" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryotherapy-facial/. Not yet built.</v>
       </c>
+      <c r="E320" t="str">
+        <v/>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
@@ -5074,10 +5856,13 @@
         <v>Vampire Facial</v>
       </c>
       <c r="C321" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D321" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/vampire-facial/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html.</v>
+      </c>
+      <c r="E321" t="str">
+        <v/>
       </c>
     </row>
     <row r="322">
@@ -5093,6 +5878,9 @@
       <c r="D322" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermabrasion-treatment/. Not yet built.</v>
       </c>
+      <c r="E322" t="str">
+        <v/>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
@@ -5107,6 +5895,9 @@
       <c r="D323" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/microdermabrasion-treatment/. Not yet built.</v>
       </c>
+      <c r="E323" t="str">
+        <v/>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
@@ -5121,6 +5912,9 @@
       <c r="D324" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-polishing/. Not yet built.</v>
       </c>
+      <c r="E324" t="str">
+        <v/>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
@@ -5135,6 +5929,9 @@
       <c r="D325" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermamelan-treatment/. Not yet built.</v>
       </c>
+      <c r="E325" t="str">
+        <v/>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
@@ -5149,6 +5946,9 @@
       <c r="D326" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-lightening-treatment/. Not yet built.</v>
       </c>
+      <c r="E326" t="str">
+        <v/>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
@@ -5163,6 +5963,9 @@
       <c r="D327" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tribeam-laser/. Not yet built.</v>
       </c>
+      <c r="E327" t="str">
+        <v/>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
@@ -5177,6 +5980,9 @@
       <c r="D328" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fractional-laser-skin/. Not yet built.</v>
       </c>
+      <c r="E328" t="str">
+        <v/>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
@@ -5191,6 +5997,9 @@
       <c r="D329" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ipl-therapy/. Not yet built.</v>
       </c>
+      <c r="E329" t="str">
+        <v/>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
@@ -5205,6 +6014,9 @@
       <c r="D330" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-brightening-treatments-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E330" t="str">
+        <v/>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
@@ -5219,6 +6031,9 @@
       <c r="D331" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-treatment-in-bangalore/. Not yet built.</v>
       </c>
+      <c r="E331" t="str">
+        <v/>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
@@ -5233,6 +6048,9 @@
       <c r="D332" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-scar-treatment-in-gurgaon/. Not yet built.</v>
       </c>
+      <c r="E332" t="str">
+        <v/>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
@@ -5247,6 +6065,9 @@
       <c r="D333" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-ageing-laser-treatment/. Not yet built.</v>
       </c>
+      <c r="E333" t="str">
+        <v/>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
@@ -5261,6 +6082,9 @@
       <c r="D334" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-anti-aging-treatment/. Not yet built.</v>
       </c>
+      <c r="E334" t="str">
+        <v/>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
@@ -5275,6 +6099,9 @@
       <c r="D335" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/wrinkles-treatment-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E335" t="str">
+        <v/>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
@@ -5289,6 +6116,9 @@
       <c r="D336" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/crows-feet-treatment-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E336" t="str">
+        <v/>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
@@ -5303,6 +6133,9 @@
       <c r="D337" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dark-circles/. Not yet built.</v>
       </c>
+      <c r="E337" t="str">
+        <v/>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
@@ -5317,6 +6150,9 @@
       <c r="D338" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tear-trough-treatment-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E338" t="str">
+        <v/>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
@@ -5331,6 +6167,9 @@
       <c r="D339" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/under-eye-fillers-treatment/. Not yet built.</v>
       </c>
+      <c r="E339" t="str">
+        <v/>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
@@ -5345,6 +6184,9 @@
       <c r="D340" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/melasma/. Not yet built.</v>
       </c>
+      <c r="E340" t="str">
+        <v/>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
@@ -5359,6 +6201,9 @@
       <c r="D341" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/rosacea/. Not yet built.</v>
       </c>
+      <c r="E341" t="str">
+        <v/>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
@@ -5373,6 +6218,9 @@
       <c r="D342" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eczema-treatment-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E342" t="str">
+        <v/>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
@@ -5387,6 +6235,9 @@
       <c r="D343" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/keratosis-pilaris/. Not yet built.</v>
       </c>
+      <c r="E343" t="str">
+        <v/>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
@@ -5401,6 +6252,9 @@
       <c r="D344" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sun-age-spots/. Not yet built.</v>
       </c>
+      <c r="E344" t="str">
+        <v/>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
@@ -5415,6 +6269,9 @@
       <c r="D345" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/underarm-darkening/. Not yet built.</v>
       </c>
+      <c r="E345" t="str">
+        <v/>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
@@ -5429,6 +6286,9 @@
       <c r="D346" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/scar-treatment/. Not yet built.</v>
       </c>
+      <c r="E346" t="str">
+        <v/>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
@@ -5443,6 +6303,9 @@
       <c r="D347" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stretch-marks/. Not yet built.</v>
       </c>
+      <c r="E347" t="str">
+        <v/>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
@@ -5457,6 +6320,9 @@
       <c r="D348" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-whitening-treatment-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E348" t="str">
+        <v/>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
@@ -5471,6 +6337,9 @@
       <c r="D349" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mnrf-treatment/. Not yet built.</v>
       </c>
+      <c r="E349" t="str">
+        <v/>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
@@ -5485,6 +6354,9 @@
       <c r="D350" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy/. Not yet built.</v>
       </c>
+      <c r="E350" t="str">
+        <v/>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
@@ -5499,6 +6371,9 @@
       <c r="D351" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermapen-treatment/. Not yet built.</v>
       </c>
+      <c r="E351" t="str">
+        <v/>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
@@ -5513,6 +6388,9 @@
       <c r="D352" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/collagen-induction-therapy/. Not yet built.</v>
       </c>
+      <c r="E352" t="str">
+        <v/>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
@@ -5527,6 +6405,9 @@
       <c r="D353" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/electrocautery-treatment/. Not yet built.</v>
       </c>
+      <c r="E353" t="str">
+        <v/>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
@@ -5541,6 +6422,9 @@
       <c r="D354" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/permanent-beard-shaping-treatment-in-mumbai/. Not yet built.</v>
       </c>
+      <c r="E354" t="str">
+        <v/>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
@@ -5554,6 +6438,9 @@
       </c>
       <c r="D355" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mens-grooming-treatments/. Not yet built.</v>
+      </c>
+      <c r="E355" t="str">
+        <v/>
       </c>
     </row>
     <row r="356">
@@ -5586,6 +6473,9 @@
       <c r="D357" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-wrinkle-injection-for-facelift-filler/. Not yet built.</v>
       </c>
+      <c r="E357" t="str">
+        <v/>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
@@ -5600,6 +6490,9 @@
       <c r="D358" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fat-lipolysis-injection/. Not yet built.</v>
       </c>
+      <c r="E358" t="str">
+        <v/>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
@@ -5614,6 +6507,9 @@
       <c r="D359" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/kenacort-injection/. Not yet built.</v>
       </c>
+      <c r="E359" t="str">
+        <v/>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
@@ -5628,6 +6524,9 @@
       <c r="D360" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tricort-injection/. Not yet built.</v>
       </c>
+      <c r="E360" t="str">
+        <v/>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
@@ -5642,6 +6541,9 @@
       <c r="D361" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluron-pen-needle-free-filler/. Not yet built.</v>
       </c>
+      <c r="E361" t="str">
+        <v/>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
@@ -5656,6 +6558,9 @@
       <c r="D362" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluronic-acid-therapy/. Not yet built.</v>
       </c>
+      <c r="E362" t="str">
+        <v/>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
@@ -5670,6 +6575,9 @@
       <c r="D363" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/viscoderm-hydrobooster/. Not yet built.</v>
       </c>
+      <c r="E363" t="str">
+        <v/>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
@@ -5684,6 +6592,9 @@
       <c r="D364" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermal-thread-treatment/. Not yet built.</v>
       </c>
+      <c r="E364" t="str">
+        <v/>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
@@ -5698,6 +6609,9 @@
       <c r="D365" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-professional-brand/. Not yet built.</v>
       </c>
+      <c r="E365" t="str">
+        <v/>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
@@ -5746,6 +6660,9 @@
       <c r="D368" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-hair-replacement/. Not yet built.</v>
       </c>
+      <c r="E368" t="str">
+        <v/>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
@@ -5760,6 +6677,9 @@
       <c r="D369" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hairgen-booster/. Not yet built.</v>
       </c>
+      <c r="E369" t="str">
+        <v/>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
@@ -5774,6 +6694,9 @@
       <c r="D370" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-hair-treatment/. Not yet built.</v>
       </c>
+      <c r="E370" t="str">
+        <v/>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
@@ -5788,6 +6711,9 @@
       <c r="D371" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc/. Not yet built.</v>
       </c>
+      <c r="E371" t="str">
+        <v/>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
@@ -5802,6 +6728,9 @@
       <c r="D372" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-treatment-in-bangalore/. Not yet built.</v>
       </c>
+      <c r="E372" t="str">
+        <v/>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
@@ -5816,6 +6745,9 @@
       <c r="D373" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hair-fall-treatment-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E373" t="str">
+        <v/>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
@@ -5830,6 +6762,9 @@
       <c r="D374" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/baldness-treatment-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E374" t="str">
+        <v/>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
@@ -5844,6 +6779,9 @@
       <c r="D375" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/alopecia-areata/. Not yet built.</v>
       </c>
+      <c r="E375" t="str">
+        <v/>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
@@ -5858,6 +6796,9 @@
       <c r="D376" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/qr-678-neo-hair-growth-and-hair-qr-treatment/. Not yet built.</v>
       </c>
+      <c r="E376" t="str">
+        <v/>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
@@ -5872,6 +6813,9 @@
       <c r="D377" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/morphyia-skin-and-hair-treatment/. Not yet built.</v>
       </c>
+      <c r="E377" t="str">
+        <v/>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
@@ -5886,6 +6830,9 @@
       <c r="D378" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-platinum/. Not yet built.</v>
       </c>
+      <c r="E378" t="str">
+        <v/>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
@@ -5900,6 +6847,9 @@
       <c r="D379" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-titanium/. Not yet built.</v>
       </c>
+      <c r="E379" t="str">
+        <v/>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
@@ -5914,6 +6864,9 @@
       <c r="D380" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/iv-drip-therapy-delhi/. Not yet built.</v>
       </c>
+      <c r="E380" t="str">
+        <v/>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
@@ -5928,6 +6881,9 @@
       <c r="D381" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stem-cell-therapy/. Not yet built.</v>
       </c>
+      <c r="E381" t="str">
+        <v/>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
@@ -5942,6 +6898,9 @@
       <c r="D382" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E382" t="str">
+        <v/>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
@@ -5956,6 +6915,9 @@
       <c r="D383" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/colon-hydrotherapy-in-delhi/. Not yet built.</v>
       </c>
+      <c r="E383" t="str">
+        <v/>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
@@ -5970,6 +6932,9 @@
       <c r="D384" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-himalayan-salt-infrared-sauna/. Not yet built.</v>
       </c>
+      <c r="E384" t="str">
+        <v/>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
@@ -5984,6 +6949,9 @@
       <c r="D385" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/spa-therapy/. Not yet built.</v>
       </c>
+      <c r="E385" t="str">
+        <v/>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
@@ -5998,6 +6966,9 @@
       <c r="D386" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/forest-essentials-body-spa/. Not yet built.</v>
       </c>
+      <c r="E386" t="str">
+        <v/>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
@@ -6012,6 +6983,9 @@
       <c r="D387" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/deesse-pro-led-mask/. Not yet built.</v>
       </c>
+      <c r="E387" t="str">
+        <v/>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
@@ -6026,6 +7000,9 @@
       <c r="D388" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-perfect-oasis/. Not yet built.</v>
       </c>
+      <c r="E388" t="str">
+        <v/>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
@@ -6040,6 +7017,9 @@
       <c r="D389" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-product/. Not yet built.</v>
       </c>
+      <c r="E389" t="str">
+        <v/>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
@@ -6054,6 +7034,9 @@
       <c r="D390" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/bridal-makeover/. Not yet built.</v>
       </c>
+      <c r="E390" t="str">
+        <v/>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
@@ -6067,6 +7050,9 @@
       </c>
       <c r="D391" t="str">
         <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/groom-makeover/. Not yet built.</v>
+      </c>
+      <c r="E391" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fill Completed Date for batch 5 rows in brochure.xlsx
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,10 +402,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E391"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+    <col min="4" max="4" width="100.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -762,7 +763,7 @@
         <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html.</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +899,7 @@
         <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="30">
@@ -915,7 +916,7 @@
         <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="31">
@@ -1000,7 +1001,7 @@
         <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html.</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="36">
@@ -1272,7 +1273,7 @@
         <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html.</v>
       </c>
       <c r="E51" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="52">
@@ -2258,7 +2259,7 @@
         <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html.</v>
       </c>
       <c r="E109" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="110">
@@ -2819,7 +2820,7 @@
         <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html.</v>
       </c>
       <c r="E142" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="143">
@@ -5862,7 +5863,7 @@
         <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html.</v>
       </c>
       <c r="E321" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="322">

</xml_diff>

<commit_message>
Fully reconcile brochure.xlsx against index.html (83/83 matched)
Applies the batch 6 completions and reconciliation fixes that failed
to save earlier due to the file being locked, adds batch 7 completions,
and adds final rows for Dermal Fillers and Laser Hair Reduction (two
pre-existing brochures with no matching row in the original service-menu
export). Every one of the 83 brochures currently linked from index.html
now has a corresponding Completed row with a source note and date.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$285</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$390</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E395"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
@@ -1403,13 +1403,13 @@
         <v>Celestrial Drip</v>
       </c>
       <c r="C59" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D59" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial").</v>
       </c>
       <c r="E59" t="str">
-        <v/>
+        <v>2026-07-15</v>
       </c>
     </row>
     <row r="60">
@@ -2066,13 +2066,13 @@
         <v>Threads</v>
       </c>
       <c r="C98" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D98" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Existing brochure: Thread Lift (thread-lift-brochure.html). Missed in the original cross-reference due to naming difference ("Threads" vs "Thread Lift").</v>
       </c>
       <c r="E98" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="99">
@@ -2151,13 +2151,13 @@
         <v>Biologique Recherche Double Booster Facial</v>
       </c>
       <c r="C103" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D103" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/biologique/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/biologique. No before/after images on source page. Placed under Facial. Brochure: biologique-recherche-facial-brochure.html.</v>
       </c>
       <c r="E103" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="104">
@@ -2440,13 +2440,13 @@
         <v>Ice Facial</v>
       </c>
       <c r="C120" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D120" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/ice-facial-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/ice-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: ice-facial-brochure.html.</v>
       </c>
       <c r="E120" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="121">
@@ -2491,13 +2491,13 @@
         <v>Love Light</v>
       </c>
       <c r="C123" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D123" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/love-light-fusion-facial/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/love-light-fusion-facial. No before/after images on source page. Placed under Facial. Brochure: love-light-fusion-facial-brochure.html.</v>
       </c>
       <c r="E123" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="124">
@@ -2542,13 +2542,13 @@
         <v>Oasis Facial</v>
       </c>
       <c r="C126" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D126" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/oasis-facial-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/oasis-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: oasis-facial-brochure.html.</v>
       </c>
       <c r="E126" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="127">
@@ -2576,13 +2576,13 @@
         <v>Oxygeneo</v>
       </c>
       <c r="C128" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D128" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/oxygeneo-facial-best-oxygen-facial/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/oxygeneo-facial-best-oxygen-facial. No before/after images on source page. Placed under Facial. Brochure: oxygeneo-facial-brochure.html.</v>
       </c>
       <c r="E128" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="129">
@@ -2695,13 +2695,13 @@
         <v>Salmon DNA</v>
       </c>
       <c r="C135" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D135" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/salmon-dna-pdrn-facial/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/salmon-dna-pdrn-facial. Only banner/decorative images found, not before/after. Placed under Facial. Brochure: salmon-dna-facial-brochure.html.</v>
       </c>
       <c r="E135" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="136">
@@ -2899,13 +2899,13 @@
         <v>Exosome- Hair</v>
       </c>
       <c r="C147" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D147" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Existing brochure: Exosome Scalp Treatment (exosome-scalp-treatment-brochure.html). Missed in the original cross-reference due to naming difference ("Exosome- Hair" vs "Exosome Scalp Treatment").</v>
       </c>
       <c r="E147" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="148">
@@ -2984,13 +2984,13 @@
         <v>Hair science- QR678</v>
       </c>
       <c r="C152" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D152" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Existing brochure: QR678 Hair Science (QR678-hair-science-brochure.html). Missed in the original cross-reference due to word order ("Hair science- QR678" vs "QR678 Hair Science").</v>
       </c>
       <c r="E152" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="153">
@@ -5256,19 +5256,19 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v/>
+        <v>Body Contouring</v>
       </c>
       <c r="B286" t="str">
-        <v/>
+        <v>Gynaecomastia</v>
       </c>
       <c r="C286" t="str">
-        <v/>
+        <v>Completed</v>
       </c>
       <c r="D286" t="str">
-        <v/>
+        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html.</v>
       </c>
       <c r="E286" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="287">
@@ -5276,13 +5276,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B287" t="str">
-        <v>Gynaecomastia</v>
+        <v>Liposuction Surgery</v>
       </c>
       <c r="C287" t="str">
         <v>Completed</v>
       </c>
       <c r="D287" t="str">
-        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html.</v>
       </c>
       <c r="E287" t="str">
         <v>2026-07-24</v>
@@ -5293,13 +5293,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B288" t="str">
-        <v>Liposuction Surgery</v>
+        <v>Non-Surgical Breast Lift</v>
       </c>
       <c r="C288" t="str">
         <v>Completed</v>
       </c>
       <c r="D288" t="str">
-        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html.</v>
       </c>
       <c r="E288" t="str">
         <v>2026-07-24</v>
@@ -5310,13 +5310,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B289" t="str">
-        <v>Non-Surgical Breast Lift</v>
+        <v>Cryolipolysis</v>
       </c>
       <c r="C289" t="str">
         <v>Completed</v>
       </c>
       <c r="D289" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html.</v>
       </c>
       <c r="E289" t="str">
         <v>2026-07-24</v>
@@ -5327,16 +5327,16 @@
         <v>Body Contouring</v>
       </c>
       <c r="B290" t="str">
-        <v>Cryolipolysis</v>
+        <v>Instasculpt</v>
       </c>
       <c r="C290" t="str">
         <v>Completed</v>
       </c>
       <c r="D290" t="str">
-        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/instasculpt. No before/after images on source page. Placed under Body Contouring. Brochure: instasculpt-brochure.html.</v>
       </c>
       <c r="E290" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="291">
@@ -5344,13 +5344,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B291" t="str">
-        <v>Instasculpt</v>
+        <v>House of Sculpt</v>
       </c>
       <c r="C291" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D291" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/instasculpt/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-sculpt/. Not yet built.</v>
       </c>
       <c r="E291" t="str">
         <v/>
@@ -5361,13 +5361,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B292" t="str">
-        <v>House of Sculpt</v>
+        <v>House of Proportion</v>
       </c>
       <c r="C292" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D292" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-sculpt/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-proportion/. Not yet built.</v>
       </c>
       <c r="E292" t="str">
         <v/>
@@ -5378,16 +5378,16 @@
         <v>Body Contouring</v>
       </c>
       <c r="B293" t="str">
-        <v>House of Proportion</v>
+        <v>Tummy Tightening</v>
       </c>
       <c r="C293" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D293" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-proportion/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/tummy-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: tummy-tightening-brochure.html.</v>
       </c>
       <c r="E293" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="294">
@@ -5395,13 +5395,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B294" t="str">
-        <v>Tummy Tightening</v>
+        <v>Tight Pro</v>
       </c>
       <c r="C294" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D294" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tummy-tightening/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tight-pro/. Not yet built.</v>
       </c>
       <c r="E294" t="str">
         <v/>
@@ -5412,13 +5412,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B295" t="str">
-        <v>Tight Pro</v>
+        <v>Ballancer Pro</v>
       </c>
       <c r="C295" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D295" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tight-pro/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ballancer-pro-treatment/. Not yet built.</v>
       </c>
       <c r="E295" t="str">
         <v/>
@@ -5429,13 +5429,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B296" t="str">
-        <v>Ballancer Pro</v>
+        <v>Femme 360 Vaginal Tightening</v>
       </c>
       <c r="C296" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D296" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ballancer-pro-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/femme-360-vaginal-tightening/. Not yet built.</v>
       </c>
       <c r="E296" t="str">
         <v/>
@@ -5446,16 +5446,16 @@
         <v>Body Contouring</v>
       </c>
       <c r="B297" t="str">
-        <v>Femme 360 Vaginal Tightening</v>
+        <v>Vaginal Fillers</v>
       </c>
       <c r="C297" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D297" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/femme-360-vaginal-tightening/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html.</v>
       </c>
       <c r="E297" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="298">
@@ -5463,16 +5463,16 @@
         <v>Body Contouring</v>
       </c>
       <c r="B298" t="str">
-        <v>Vaginal Fillers</v>
+        <v>Multipolar Radio Frequency</v>
       </c>
       <c r="C298" t="str">
-        <v>Completed</v>
+        <v>To Build (source available)</v>
       </c>
       <c r="D298" t="str">
-        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/multipolar-radio-frequency-in-delhi/. Not yet built.</v>
       </c>
       <c r="E298" t="str">
-        <v>2026-07-24</v>
+        <v/>
       </c>
     </row>
     <row r="299">
@@ -5480,13 +5480,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B299" t="str">
-        <v>Multipolar Radio Frequency</v>
+        <v>HIFU Skin Tightening</v>
       </c>
       <c r="C299" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D299" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/multipolar-radio-frequency-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3/. Not yet built.</v>
       </c>
       <c r="E299" t="str">
         <v/>
@@ -5497,13 +5497,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B300" t="str">
-        <v>HIFU Skin Tightening</v>
+        <v>Skin Tightening Treatment</v>
       </c>
       <c r="C300" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D300" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-tightening-treatment-in-vasant-vihar/. Not yet built.</v>
       </c>
       <c r="E300" t="str">
         <v/>
@@ -5514,13 +5514,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B301" t="str">
-        <v>Skin Tightening Treatment</v>
+        <v>Sculpt Tone Plus</v>
       </c>
       <c r="C301" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D301" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-tightening-treatment-in-vasant-vihar/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sculptone-plus/. Not yet built.</v>
       </c>
       <c r="E301" t="str">
         <v/>
@@ -5531,13 +5531,13 @@
         <v>Body Contouring</v>
       </c>
       <c r="B302" t="str">
-        <v>Sculpt Tone Plus</v>
+        <v>Cool Tech</v>
       </c>
       <c r="C302" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D302" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sculptone-plus/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cool-tech/. Not yet built.</v>
       </c>
       <c r="E302" t="str">
         <v/>
@@ -5545,19 +5545,19 @@
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>Body Contouring</v>
+        <v>Face Lifting</v>
       </c>
       <c r="B303" t="str">
-        <v>Cool Tech</v>
+        <v>Ulthera Face Lifting</v>
       </c>
       <c r="C303" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D303" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cool-tech/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting).</v>
       </c>
       <c r="E303" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="304">
@@ -5565,16 +5565,16 @@
         <v>Face Lifting</v>
       </c>
       <c r="B304" t="str">
-        <v>Ulthera Face Lifting</v>
+        <v>Thread Face Lift</v>
       </c>
       <c r="C304" t="str">
         <v>Completed</v>
       </c>
       <c r="D304" t="str">
-        <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting).</v>
+        <v>Scraped from isaacluxe.co/thread-face-lift-treatment. Note: conceptually overlaps with the existing "Thread Lift" and "Aptos Thread Lift" brochures (all use PDO/PLLA-style threads), but is its own distinct catalog line item, so built separately -- flag if you want these consolidated. No before/after photos (only hero images). Placed under Face Lifting. Brochure: thread-face-lift-brochure.html.</v>
       </c>
       <c r="E304" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="305">
@@ -5582,13 +5582,13 @@
         <v>Face Lifting</v>
       </c>
       <c r="B305" t="str">
-        <v>Thread Face Lift</v>
+        <v>Liquid Facelift</v>
       </c>
       <c r="C305" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D305" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/thread-face-lift-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liquid-facelift-treatment/. Not yet built.</v>
       </c>
       <c r="E305" t="str">
         <v/>
@@ -5599,16 +5599,16 @@
         <v>Face Lifting</v>
       </c>
       <c r="B306" t="str">
-        <v>Liquid Facelift</v>
+        <v>Non-Surgical Face Lift</v>
       </c>
       <c r="C306" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D306" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liquid-facelift-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html.</v>
       </c>
       <c r="E306" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="307">
@@ -5616,16 +5616,16 @@
         <v>Face Lifting</v>
       </c>
       <c r="B307" t="str">
-        <v>Non-Surgical Face Lift</v>
+        <v>Sygma Lift Treatment</v>
       </c>
       <c r="C307" t="str">
-        <v>Completed</v>
+        <v>To Build (source available)</v>
       </c>
       <c r="D307" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sygma-lift-treatment-in-gurgaon/. Not yet built.</v>
       </c>
       <c r="E307" t="str">
-        <v>2026-07-24</v>
+        <v/>
       </c>
     </row>
     <row r="308">
@@ -5633,16 +5633,16 @@
         <v>Face Lifting</v>
       </c>
       <c r="B308" t="str">
-        <v>Sygma Lift Treatment</v>
+        <v>4-D Lift</v>
       </c>
       <c r="C308" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D308" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sygma-lift-treatment-in-gurgaon/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/4-d-lift. No before/after images on source page. Placed under Face Lifting. Brochure: 4d-lift-brochure.html.</v>
       </c>
       <c r="E308" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="309">
@@ -5650,13 +5650,13 @@
         <v>Face Lifting</v>
       </c>
       <c r="B309" t="str">
-        <v>4-D Lift</v>
+        <v>Face Lift Filler</v>
       </c>
       <c r="C309" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D309" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/4-d-lift/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-lift-filler-in-delhi/. Not yet built.</v>
       </c>
       <c r="E309" t="str">
         <v/>
@@ -5667,13 +5667,13 @@
         <v>Face Lifting</v>
       </c>
       <c r="B310" t="str">
-        <v>Face Lift Filler</v>
+        <v>Square Jaw Treatment</v>
       </c>
       <c r="C310" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D310" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-lift-filler-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/square-jaw-treatment-in-delhi/. Not yet built.</v>
       </c>
       <c r="E310" t="str">
         <v/>
@@ -5684,13 +5684,13 @@
         <v>Face Lifting</v>
       </c>
       <c r="B311" t="str">
-        <v>Square Jaw Treatment</v>
+        <v>Poppy Chin Treatment</v>
       </c>
       <c r="C311" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D311" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/square-jaw-treatment-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/poppy-chin-treatment-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E311" t="str">
         <v/>
@@ -5698,16 +5698,16 @@
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>Face Lifting</v>
+        <v>Facial</v>
       </c>
       <c r="B312" t="str">
-        <v>Poppy Chin Treatment</v>
+        <v>BR Facial</v>
       </c>
       <c r="C312" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D312" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/poppy-chin-treatment-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/br-facial/. Not yet built.</v>
       </c>
       <c r="E312" t="str">
         <v/>
@@ -5718,13 +5718,13 @@
         <v>Facial</v>
       </c>
       <c r="B313" t="str">
-        <v>BR Facial</v>
+        <v>Eve Lom Facial</v>
       </c>
       <c r="C313" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D313" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/br-facial/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eve-lom-facial/. Not yet built.</v>
       </c>
       <c r="E313" t="str">
         <v/>
@@ -5735,13 +5735,13 @@
         <v>Facial</v>
       </c>
       <c r="B314" t="str">
-        <v>Eve Lom Facial</v>
+        <v>O2Derm Facial</v>
       </c>
       <c r="C314" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D314" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eve-lom-facial/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/o2derm-facial/. Not yet built.</v>
       </c>
       <c r="E314" t="str">
         <v/>
@@ -5752,13 +5752,13 @@
         <v>Facial</v>
       </c>
       <c r="B315" t="str">
-        <v>O2Derm Facial</v>
+        <v>Exo Glow Treatment</v>
       </c>
       <c r="C315" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D315" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/o2derm-facial/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/exo-glow-treatment/. Not yet built.</v>
       </c>
       <c r="E315" t="str">
         <v/>
@@ -5769,13 +5769,13 @@
         <v>Facial</v>
       </c>
       <c r="B316" t="str">
-        <v>Exo Glow Treatment</v>
+        <v>Meso Glow</v>
       </c>
       <c r="C316" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D316" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/exo-glow-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/meso-glow/. Not yet built.</v>
       </c>
       <c r="E316" t="str">
         <v/>
@@ -5786,13 +5786,13 @@
         <v>Facial</v>
       </c>
       <c r="B317" t="str">
-        <v>Meso Glow</v>
+        <v>Lumi Face</v>
       </c>
       <c r="C317" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D317" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/meso-glow/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-face/. Not yet built.</v>
       </c>
       <c r="E317" t="str">
         <v/>
@@ -5803,13 +5803,13 @@
         <v>Facial</v>
       </c>
       <c r="B318" t="str">
-        <v>Lumi Face</v>
+        <v>Lumi Eyes</v>
       </c>
       <c r="C318" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D318" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-face/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-eyes/. Not yet built.</v>
       </c>
       <c r="E318" t="str">
         <v/>
@@ -5820,13 +5820,13 @@
         <v>Facial</v>
       </c>
       <c r="B319" t="str">
-        <v>Lumi Eyes</v>
+        <v>Cryotherapy Facial</v>
       </c>
       <c r="C319" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D319" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-eyes/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryotherapy-facial/. Not yet built.</v>
       </c>
       <c r="E319" t="str">
         <v/>
@@ -5837,16 +5837,16 @@
         <v>Facial</v>
       </c>
       <c r="B320" t="str">
-        <v>Cryotherapy Facial</v>
+        <v>Vampire Facial</v>
       </c>
       <c r="C320" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D320" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryotherapy-facial/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html.</v>
       </c>
       <c r="E320" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="321">
@@ -5854,16 +5854,16 @@
         <v>Facial</v>
       </c>
       <c r="B321" t="str">
-        <v>Vampire Facial</v>
+        <v>Dermabrasion Treatment</v>
       </c>
       <c r="C321" t="str">
-        <v>Completed</v>
+        <v>To Build (source available)</v>
       </c>
       <c r="D321" t="str">
-        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermabrasion-treatment/. Not yet built.</v>
       </c>
       <c r="E321" t="str">
-        <v>2026-07-25</v>
+        <v/>
       </c>
     </row>
     <row r="322">
@@ -5871,13 +5871,13 @@
         <v>Facial</v>
       </c>
       <c r="B322" t="str">
-        <v>Dermabrasion Treatment</v>
+        <v>Microdermabrasion Treatment</v>
       </c>
       <c r="C322" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D322" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermabrasion-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/microdermabrasion-treatment/. Not yet built.</v>
       </c>
       <c r="E322" t="str">
         <v/>
@@ -5888,16 +5888,16 @@
         <v>Facial</v>
       </c>
       <c r="B323" t="str">
-        <v>Microdermabrasion Treatment</v>
+        <v>Skin Polishing</v>
       </c>
       <c r="C323" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D323" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/microdermabrasion-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/skin-polishing (a body-wide treatment; titled "Body Polishing" in the brochure). No before/after images on source page. Placed under Facial as closest fit. Brochure: skin-polishing-brochure.html.</v>
       </c>
       <c r="E323" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="324">
@@ -5905,16 +5905,16 @@
         <v>Facial</v>
       </c>
       <c r="B324" t="str">
-        <v>Skin Polishing</v>
+        <v>Dermamelan Treatment</v>
       </c>
       <c r="C324" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D324" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-polishing/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/dermamelan-treatment. Only a process-diagram image found, not before/after. Placed under Facial. Brochure: dermamelan-brochure.html.</v>
       </c>
       <c r="E324" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="325">
@@ -5922,13 +5922,13 @@
         <v>Facial</v>
       </c>
       <c r="B325" t="str">
-        <v>Dermamelan Treatment</v>
+        <v>Skin Lightening Treatment</v>
       </c>
       <c r="C325" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D325" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermamelan-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-lightening-treatment/. Not yet built.</v>
       </c>
       <c r="E325" t="str">
         <v/>
@@ -5939,13 +5939,13 @@
         <v>Facial</v>
       </c>
       <c r="B326" t="str">
-        <v>Skin Lightening Treatment</v>
+        <v>Tribeam Laser</v>
       </c>
       <c r="C326" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D326" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-lightening-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tribeam-laser/. Not yet built.</v>
       </c>
       <c r="E326" t="str">
         <v/>
@@ -5956,13 +5956,13 @@
         <v>Facial</v>
       </c>
       <c r="B327" t="str">
-        <v>Tribeam Laser</v>
+        <v>Fractional Laser Skin</v>
       </c>
       <c r="C327" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D327" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tribeam-laser/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fractional-laser-skin/. Not yet built.</v>
       </c>
       <c r="E327" t="str">
         <v/>
@@ -5973,13 +5973,13 @@
         <v>Facial</v>
       </c>
       <c r="B328" t="str">
-        <v>Fractional Laser Skin</v>
+        <v>IPL Therapy</v>
       </c>
       <c r="C328" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D328" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fractional-laser-skin/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ipl-therapy/. Not yet built.</v>
       </c>
       <c r="E328" t="str">
         <v/>
@@ -5990,13 +5990,13 @@
         <v>Facial</v>
       </c>
       <c r="B329" t="str">
-        <v>IPL Therapy</v>
+        <v>Face Brightening Treatment</v>
       </c>
       <c r="C329" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D329" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ipl-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-brightening-treatments-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E329" t="str">
         <v/>
@@ -6007,13 +6007,13 @@
         <v>Facial</v>
       </c>
       <c r="B330" t="str">
-        <v>Face Brightening Treatment</v>
+        <v>Acne Treatment</v>
       </c>
       <c r="C330" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D330" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-brightening-treatments-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-treatment-in-bangalore/. Not yet built.</v>
       </c>
       <c r="E330" t="str">
         <v/>
@@ -6024,13 +6024,13 @@
         <v>Facial</v>
       </c>
       <c r="B331" t="str">
-        <v>Acne Treatment</v>
+        <v>Acne Scar Treatment</v>
       </c>
       <c r="C331" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D331" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-treatment-in-bangalore/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-scar-treatment-in-gurgaon/. Not yet built.</v>
       </c>
       <c r="E331" t="str">
         <v/>
@@ -6041,13 +6041,13 @@
         <v>Facial</v>
       </c>
       <c r="B332" t="str">
-        <v>Acne Scar Treatment</v>
+        <v>Anti-Ageing Laser Treatment</v>
       </c>
       <c r="C332" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D332" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-scar-treatment-in-gurgaon/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-ageing-laser-treatment/. Not yet built.</v>
       </c>
       <c r="E332" t="str">
         <v/>
@@ -6058,13 +6058,13 @@
         <v>Facial</v>
       </c>
       <c r="B333" t="str">
-        <v>Anti-Ageing Laser Treatment</v>
+        <v>Pink Anti-Aging Treatment</v>
       </c>
       <c r="C333" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D333" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-ageing-laser-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-anti-aging-treatment/. Not yet built.</v>
       </c>
       <c r="E333" t="str">
         <v/>
@@ -6075,13 +6075,13 @@
         <v>Facial</v>
       </c>
       <c r="B334" t="str">
-        <v>Pink Anti-Aging Treatment</v>
+        <v>Wrinkles Treatment</v>
       </c>
       <c r="C334" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D334" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-anti-aging-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/wrinkles-treatment-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E334" t="str">
         <v/>
@@ -6092,13 +6092,13 @@
         <v>Facial</v>
       </c>
       <c r="B335" t="str">
-        <v>Wrinkles Treatment</v>
+        <v>Crow's Feet Treatment</v>
       </c>
       <c r="C335" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D335" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/wrinkles-treatment-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/crows-feet-treatment-in-delhi/. Not yet built.</v>
       </c>
       <c r="E335" t="str">
         <v/>
@@ -6109,13 +6109,13 @@
         <v>Facial</v>
       </c>
       <c r="B336" t="str">
-        <v>Crow's Feet Treatment</v>
+        <v>Dark Circles</v>
       </c>
       <c r="C336" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D336" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/crows-feet-treatment-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dark-circles/. Not yet built.</v>
       </c>
       <c r="E336" t="str">
         <v/>
@@ -6126,13 +6126,13 @@
         <v>Facial</v>
       </c>
       <c r="B337" t="str">
-        <v>Dark Circles</v>
+        <v>Tear Trough Treatment</v>
       </c>
       <c r="C337" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D337" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dark-circles/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tear-trough-treatment-in-delhi/. Not yet built.</v>
       </c>
       <c r="E337" t="str">
         <v/>
@@ -6143,13 +6143,13 @@
         <v>Facial</v>
       </c>
       <c r="B338" t="str">
-        <v>Tear Trough Treatment</v>
+        <v>Under Eye Fillers Treatment</v>
       </c>
       <c r="C338" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D338" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tear-trough-treatment-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/under-eye-fillers-treatment/. Not yet built.</v>
       </c>
       <c r="E338" t="str">
         <v/>
@@ -6160,13 +6160,13 @@
         <v>Facial</v>
       </c>
       <c r="B339" t="str">
-        <v>Under Eye Fillers Treatment</v>
+        <v>Melasma</v>
       </c>
       <c r="C339" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D339" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/under-eye-fillers-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/melasma/. Not yet built.</v>
       </c>
       <c r="E339" t="str">
         <v/>
@@ -6177,13 +6177,13 @@
         <v>Facial</v>
       </c>
       <c r="B340" t="str">
-        <v>Melasma</v>
+        <v>Rosacea</v>
       </c>
       <c r="C340" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D340" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/melasma/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/rosacea/. Not yet built.</v>
       </c>
       <c r="E340" t="str">
         <v/>
@@ -6194,13 +6194,13 @@
         <v>Facial</v>
       </c>
       <c r="B341" t="str">
-        <v>Rosacea</v>
+        <v>Eczema Treatment</v>
       </c>
       <c r="C341" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D341" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/rosacea/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eczema-treatment-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E341" t="str">
         <v/>
@@ -6211,13 +6211,13 @@
         <v>Facial</v>
       </c>
       <c r="B342" t="str">
-        <v>Eczema Treatment</v>
+        <v>Keratosis Pilaris</v>
       </c>
       <c r="C342" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D342" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eczema-treatment-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/keratosis-pilaris/. Not yet built.</v>
       </c>
       <c r="E342" t="str">
         <v/>
@@ -6228,13 +6228,13 @@
         <v>Facial</v>
       </c>
       <c r="B343" t="str">
-        <v>Keratosis Pilaris</v>
+        <v>Sun / Age Spots</v>
       </c>
       <c r="C343" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D343" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/keratosis-pilaris/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sun-age-spots/. Not yet built.</v>
       </c>
       <c r="E343" t="str">
         <v/>
@@ -6245,13 +6245,13 @@
         <v>Facial</v>
       </c>
       <c r="B344" t="str">
-        <v>Sun / Age Spots</v>
+        <v>Underarm Darkening</v>
       </c>
       <c r="C344" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D344" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sun-age-spots/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/underarm-darkening/. Not yet built.</v>
       </c>
       <c r="E344" t="str">
         <v/>
@@ -6262,13 +6262,13 @@
         <v>Facial</v>
       </c>
       <c r="B345" t="str">
-        <v>Underarm Darkening</v>
+        <v>Scar Treatment</v>
       </c>
       <c r="C345" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D345" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/underarm-darkening/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/scar-treatment/. Not yet built.</v>
       </c>
       <c r="E345" t="str">
         <v/>
@@ -6279,13 +6279,13 @@
         <v>Facial</v>
       </c>
       <c r="B346" t="str">
-        <v>Scar Treatment</v>
+        <v>Stretch Marks</v>
       </c>
       <c r="C346" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D346" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/scar-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stretch-marks/. Not yet built.</v>
       </c>
       <c r="E346" t="str">
         <v/>
@@ -6296,13 +6296,13 @@
         <v>Facial</v>
       </c>
       <c r="B347" t="str">
-        <v>Stretch Marks</v>
+        <v>Skin Whitening Treatment</v>
       </c>
       <c r="C347" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D347" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stretch-marks/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-whitening-treatment-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E347" t="str">
         <v/>
@@ -6313,13 +6313,13 @@
         <v>Facial</v>
       </c>
       <c r="B348" t="str">
-        <v>Skin Whitening Treatment</v>
+        <v>MNRF Treatment</v>
       </c>
       <c r="C348" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D348" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-whitening-treatment-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mnrf-treatment/. Not yet built.</v>
       </c>
       <c r="E348" t="str">
         <v/>
@@ -6330,13 +6330,13 @@
         <v>Facial</v>
       </c>
       <c r="B349" t="str">
-        <v>MNRF Treatment</v>
+        <v>Dermarolling / Advanced Microneedling</v>
       </c>
       <c r="C349" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D349" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mnrf-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy/. Not yet built.</v>
       </c>
       <c r="E349" t="str">
         <v/>
@@ -6347,13 +6347,13 @@
         <v>Facial</v>
       </c>
       <c r="B350" t="str">
-        <v>Dermarolling / Advanced Microneedling</v>
+        <v>Dermapen Treatment</v>
       </c>
       <c r="C350" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D350" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermapen-treatment/. Not yet built.</v>
       </c>
       <c r="E350" t="str">
         <v/>
@@ -6364,13 +6364,13 @@
         <v>Facial</v>
       </c>
       <c r="B351" t="str">
-        <v>Dermapen Treatment</v>
+        <v>Collagen Induction Therapy</v>
       </c>
       <c r="C351" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D351" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermapen-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/collagen-induction-therapy/. Not yet built.</v>
       </c>
       <c r="E351" t="str">
         <v/>
@@ -6381,13 +6381,13 @@
         <v>Facial</v>
       </c>
       <c r="B352" t="str">
-        <v>Collagen Induction Therapy</v>
+        <v>Electrocautery Treatment</v>
       </c>
       <c r="C352" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D352" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/collagen-induction-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/electrocautery-treatment/. Not yet built.</v>
       </c>
       <c r="E352" t="str">
         <v/>
@@ -6398,13 +6398,13 @@
         <v>Facial</v>
       </c>
       <c r="B353" t="str">
-        <v>Electrocautery Treatment</v>
+        <v>Permanent Beard Shaping</v>
       </c>
       <c r="C353" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D353" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/electrocautery-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/permanent-beard-shaping-treatment-in-mumbai/. Not yet built.</v>
       </c>
       <c r="E353" t="str">
         <v/>
@@ -6415,13 +6415,13 @@
         <v>Facial</v>
       </c>
       <c r="B354" t="str">
-        <v>Permanent Beard Shaping</v>
+        <v>Men's Grooming Treatments</v>
       </c>
       <c r="C354" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D354" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/permanent-beard-shaping-treatment-in-mumbai/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mens-grooming-treatments/. Not yet built.</v>
       </c>
       <c r="E354" t="str">
         <v/>
@@ -6429,19 +6429,19 @@
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>Facial</v>
+        <v>Injectable</v>
       </c>
       <c r="B355" t="str">
-        <v>Men's Grooming Treatments</v>
+        <v>Lip Fillers</v>
       </c>
       <c r="C355" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D355" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mens-grooming-treatments/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html.</v>
       </c>
       <c r="E355" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="356">
@@ -6449,16 +6449,16 @@
         <v>Injectable</v>
       </c>
       <c r="B356" t="str">
-        <v>Lip Fillers</v>
+        <v>Anti-Wrinkle Injection (Facelift Filler)</v>
       </c>
       <c r="C356" t="str">
-        <v>Completed</v>
+        <v>To Build (source available)</v>
       </c>
       <c r="D356" t="str">
-        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-wrinkle-injection-for-facelift-filler/. Not yet built.</v>
       </c>
       <c r="E356" t="str">
-        <v>2026-07-24</v>
+        <v/>
       </c>
     </row>
     <row r="357">
@@ -6466,13 +6466,13 @@
         <v>Injectable</v>
       </c>
       <c r="B357" t="str">
-        <v>Anti-Wrinkle Injection (Facelift Filler)</v>
+        <v>Fat Lipolysis Injection</v>
       </c>
       <c r="C357" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D357" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-wrinkle-injection-for-facelift-filler/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fat-lipolysis-injection/. Not yet built.</v>
       </c>
       <c r="E357" t="str">
         <v/>
@@ -6483,13 +6483,13 @@
         <v>Injectable</v>
       </c>
       <c r="B358" t="str">
-        <v>Fat Lipolysis Injection</v>
+        <v>Kenacort Injection</v>
       </c>
       <c r="C358" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D358" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fat-lipolysis-injection/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/kenacort-injection/. Not yet built.</v>
       </c>
       <c r="E358" t="str">
         <v/>
@@ -6500,13 +6500,13 @@
         <v>Injectable</v>
       </c>
       <c r="B359" t="str">
-        <v>Kenacort Injection</v>
+        <v>Tricort Injection</v>
       </c>
       <c r="C359" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D359" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/kenacort-injection/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tricort-injection/. Not yet built.</v>
       </c>
       <c r="E359" t="str">
         <v/>
@@ -6517,13 +6517,13 @@
         <v>Injectable</v>
       </c>
       <c r="B360" t="str">
-        <v>Tricort Injection</v>
+        <v>Hyaluron Pen (Needle-Free Filler)</v>
       </c>
       <c r="C360" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D360" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tricort-injection/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluron-pen-needle-free-filler/. Not yet built.</v>
       </c>
       <c r="E360" t="str">
         <v/>
@@ -6534,13 +6534,13 @@
         <v>Injectable</v>
       </c>
       <c r="B361" t="str">
-        <v>Hyaluron Pen (Needle-Free Filler)</v>
+        <v>Hyaluronic Acid Therapy</v>
       </c>
       <c r="C361" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D361" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluron-pen-needle-free-filler/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluronic-acid-therapy/. Not yet built.</v>
       </c>
       <c r="E361" t="str">
         <v/>
@@ -6551,13 +6551,13 @@
         <v>Injectable</v>
       </c>
       <c r="B362" t="str">
-        <v>Hyaluronic Acid Therapy</v>
+        <v>Viscoderm Hydrobooster</v>
       </c>
       <c r="C362" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D362" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluronic-acid-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/viscoderm-hydrobooster/. Not yet built.</v>
       </c>
       <c r="E362" t="str">
         <v/>
@@ -6568,13 +6568,13 @@
         <v>Injectable</v>
       </c>
       <c r="B363" t="str">
-        <v>Viscoderm Hydrobooster</v>
+        <v>Dermal Thread Treatment</v>
       </c>
       <c r="C363" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D363" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/viscoderm-hydrobooster/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermal-thread-treatment/. Not yet built.</v>
       </c>
       <c r="E363" t="str">
         <v/>
@@ -6585,13 +6585,13 @@
         <v>Injectable</v>
       </c>
       <c r="B364" t="str">
-        <v>Dermal Thread Treatment</v>
+        <v>Calecim Professional Brand</v>
       </c>
       <c r="C364" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D364" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermal-thread-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-professional-brand/. Not yet built.</v>
       </c>
       <c r="E364" t="str">
         <v/>
@@ -6599,19 +6599,19 @@
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>Injectable</v>
+        <v>Hair</v>
       </c>
       <c r="B365" t="str">
-        <v>Calecim Professional Brand</v>
+        <v>Eyebrow Transplant</v>
       </c>
       <c r="C365" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D365" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-professional-brand/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html.</v>
       </c>
       <c r="E365" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="366">
@@ -6619,13 +6619,13 @@
         <v>Hair</v>
       </c>
       <c r="B366" t="str">
-        <v>Eyebrow Transplant</v>
+        <v>Regenera Activa Hair Treatment</v>
       </c>
       <c r="C366" t="str">
         <v>Completed</v>
       </c>
       <c r="D366" t="str">
-        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html.</v>
       </c>
       <c r="E366" t="str">
         <v>2026-07-24</v>
@@ -6636,16 +6636,16 @@
         <v>Hair</v>
       </c>
       <c r="B367" t="str">
-        <v>Regenera Activa Hair Treatment</v>
+        <v>Non-Surgical Hair Replacement</v>
       </c>
       <c r="C367" t="str">
-        <v>Completed</v>
+        <v>To Build (source available)</v>
       </c>
       <c r="D367" t="str">
-        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-hair-replacement/. Not yet built.</v>
       </c>
       <c r="E367" t="str">
-        <v>2026-07-24</v>
+        <v/>
       </c>
     </row>
     <row r="368">
@@ -6653,13 +6653,13 @@
         <v>Hair</v>
       </c>
       <c r="B368" t="str">
-        <v>Non-Surgical Hair Replacement</v>
+        <v>Hairgen Booster</v>
       </c>
       <c r="C368" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D368" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-hair-replacement/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hairgen-booster/. Not yet built.</v>
       </c>
       <c r="E368" t="str">
         <v/>
@@ -6670,13 +6670,13 @@
         <v>Hair</v>
       </c>
       <c r="B369" t="str">
-        <v>Hairgen Booster</v>
+        <v>PRP Hair Treatment</v>
       </c>
       <c r="C369" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D369" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hairgen-booster/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-hair-treatment/. Not yet built.</v>
       </c>
       <c r="E369" t="str">
         <v/>
@@ -6687,13 +6687,13 @@
         <v>Hair</v>
       </c>
       <c r="B370" t="str">
-        <v>PRP Hair Treatment</v>
+        <v>Advanced PRP Growth Factor Concentrate (GFC)</v>
       </c>
       <c r="C370" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D370" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-hair-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc/. Not yet built.</v>
       </c>
       <c r="E370" t="str">
         <v/>
@@ -6704,13 +6704,13 @@
         <v>Hair</v>
       </c>
       <c r="B371" t="str">
-        <v>Advanced PRP Growth Factor Concentrate (GFC)</v>
+        <v>PRP Treatment</v>
       </c>
       <c r="C371" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D371" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-treatment-in-bangalore/. Not yet built.</v>
       </c>
       <c r="E371" t="str">
         <v/>
@@ -6721,13 +6721,13 @@
         <v>Hair</v>
       </c>
       <c r="B372" t="str">
-        <v>PRP Treatment</v>
+        <v>Hair Fall Treatment</v>
       </c>
       <c r="C372" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D372" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-treatment-in-bangalore/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hair-fall-treatment-in-delhi/. Not yet built.</v>
       </c>
       <c r="E372" t="str">
         <v/>
@@ -6738,13 +6738,13 @@
         <v>Hair</v>
       </c>
       <c r="B373" t="str">
-        <v>Hair Fall Treatment</v>
+        <v>Baldness Treatment</v>
       </c>
       <c r="C373" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D373" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hair-fall-treatment-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/baldness-treatment-in-delhi/. Not yet built.</v>
       </c>
       <c r="E373" t="str">
         <v/>
@@ -6755,13 +6755,13 @@
         <v>Hair</v>
       </c>
       <c r="B374" t="str">
-        <v>Baldness Treatment</v>
+        <v>Alopecia Areata</v>
       </c>
       <c r="C374" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D374" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/baldness-treatment-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/alopecia-areata/. Not yet built.</v>
       </c>
       <c r="E374" t="str">
         <v/>
@@ -6772,13 +6772,13 @@
         <v>Hair</v>
       </c>
       <c r="B375" t="str">
-        <v>Alopecia Areata</v>
+        <v>QR-678 Neo Hair Growth</v>
       </c>
       <c r="C375" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D375" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/alopecia-areata/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/qr-678-neo-hair-growth-and-hair-qr-treatment/. Not yet built.</v>
       </c>
       <c r="E375" t="str">
         <v/>
@@ -6789,13 +6789,13 @@
         <v>Hair</v>
       </c>
       <c r="B376" t="str">
-        <v>QR-678 Neo Hair Growth</v>
+        <v>Morphyia Skin and Hair Treatment</v>
       </c>
       <c r="C376" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D376" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/qr-678-neo-hair-growth-and-hair-qr-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/morphyia-skin-and-hair-treatment/. Not yet built.</v>
       </c>
       <c r="E376" t="str">
         <v/>
@@ -6803,16 +6803,16 @@
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>Hair</v>
+        <v>Lasar Hair Reduction</v>
       </c>
       <c r="B377" t="str">
-        <v>Morphyia Skin and Hair Treatment</v>
+        <v>Soprano Ice Platinum</v>
       </c>
       <c r="C377" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D377" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/morphyia-skin-and-hair-treatment/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-platinum/. Not yet built.</v>
       </c>
       <c r="E377" t="str">
         <v/>
@@ -6823,13 +6823,13 @@
         <v>Lasar Hair Reduction</v>
       </c>
       <c r="B378" t="str">
-        <v>Soprano Ice Platinum</v>
+        <v>Soprano Ice Titanium</v>
       </c>
       <c r="C378" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D378" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-platinum/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-titanium/. Not yet built.</v>
       </c>
       <c r="E378" t="str">
         <v/>
@@ -6837,16 +6837,16 @@
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>Lasar Hair Reduction</v>
+        <v>Drip</v>
       </c>
       <c r="B379" t="str">
-        <v>Soprano Ice Titanium</v>
+        <v>IV Drip Therapy</v>
       </c>
       <c r="C379" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D379" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-titanium/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/iv-drip-therapy-delhi/. Not yet built.</v>
       </c>
       <c r="E379" t="str">
         <v/>
@@ -6857,13 +6857,13 @@
         <v>Drip</v>
       </c>
       <c r="B380" t="str">
-        <v>IV Drip Therapy</v>
+        <v>Stem Cell Therapy</v>
       </c>
       <c r="C380" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D380" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/iv-drip-therapy-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stem-cell-therapy/. Not yet built.</v>
       </c>
       <c r="E380" t="str">
         <v/>
@@ -6874,13 +6874,13 @@
         <v>Drip</v>
       </c>
       <c r="B381" t="str">
-        <v>Stem Cell Therapy</v>
+        <v>Hyperbaric Oxygen Therapy</v>
       </c>
       <c r="C381" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D381" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stem-cell-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi/. Not yet built.</v>
       </c>
       <c r="E381" t="str">
         <v/>
@@ -6891,13 +6891,13 @@
         <v>Drip</v>
       </c>
       <c r="B382" t="str">
-        <v>Hyperbaric Oxygen Therapy</v>
+        <v>Colon Hydrotherapy</v>
       </c>
       <c r="C382" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D382" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/colon-hydrotherapy-in-delhi/. Not yet built.</v>
       </c>
       <c r="E382" t="str">
         <v/>
@@ -6905,16 +6905,16 @@
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>Drip</v>
+        <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B383" t="str">
-        <v>Colon Hydrotherapy</v>
+        <v>Pink Himalayan Salt Infrared Sauna</v>
       </c>
       <c r="C383" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D383" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/colon-hydrotherapy-in-delhi/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-himalayan-salt-infrared-sauna/. Not yet built.</v>
       </c>
       <c r="E383" t="str">
         <v/>
@@ -6925,13 +6925,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B384" t="str">
-        <v>Pink Himalayan Salt Infrared Sauna</v>
+        <v>Spa Therapy</v>
       </c>
       <c r="C384" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D384" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-himalayan-salt-infrared-sauna/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/spa-therapy/. Not yet built.</v>
       </c>
       <c r="E384" t="str">
         <v/>
@@ -6942,13 +6942,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B385" t="str">
-        <v>Spa Therapy</v>
+        <v>Forest Essentials Body Spa</v>
       </c>
       <c r="C385" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D385" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/spa-therapy/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/forest-essentials-body-spa/. Not yet built.</v>
       </c>
       <c r="E385" t="str">
         <v/>
@@ -6959,13 +6959,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B386" t="str">
-        <v>Forest Essentials Body Spa</v>
+        <v>Deesse Pro LED Mask</v>
       </c>
       <c r="C386" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D386" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/forest-essentials-body-spa/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/deesse-pro-led-mask/. Not yet built.</v>
       </c>
       <c r="E386" t="str">
         <v/>
@@ -6976,13 +6976,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B387" t="str">
-        <v>Deesse Pro LED Mask</v>
+        <v>Skin Perfect Oasis</v>
       </c>
       <c r="C387" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D387" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/deesse-pro-led-mask/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-perfect-oasis/. Not yet built.</v>
       </c>
       <c r="E387" t="str">
         <v/>
@@ -6993,13 +6993,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B388" t="str">
-        <v>Skin Perfect Oasis</v>
+        <v>Calecim Product</v>
       </c>
       <c r="C388" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D388" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-perfect-oasis/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-product/. Not yet built.</v>
       </c>
       <c r="E388" t="str">
         <v/>
@@ -7010,13 +7010,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B389" t="str">
-        <v>Calecim Product</v>
+        <v>Bridal Makeover</v>
       </c>
       <c r="C389" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D389" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-product/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/bridal-makeover/. Not yet built.</v>
       </c>
       <c r="E389" t="str">
         <v/>
@@ -7027,13 +7027,13 @@
         <v>Wellness (Uncategorized)</v>
       </c>
       <c r="B390" t="str">
-        <v>Bridal Makeover</v>
+        <v>Groom Makeover</v>
       </c>
       <c r="C390" t="str">
         <v>To Build (source available)</v>
       </c>
       <c r="D390" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/bridal-makeover/. Not yet built.</v>
+        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/groom-makeover/. Not yet built.</v>
       </c>
       <c r="E390" t="str">
         <v/>
@@ -7041,24 +7041,92 @@
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>Wellness (Uncategorized)</v>
+        <v>ISAAC Luxe</v>
       </c>
       <c r="B391" t="str">
-        <v>Groom Makeover</v>
+        <v>ISAAC Luxe (Company Brochure)</v>
       </c>
       <c r="C391" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D391" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/groom-makeover/. Not yet built.</v>
+        <v>Brand/company overview page, not an individual treatment -- no row existed in the original 285-row service-menu export. Brochure: company-brochure.html.</v>
       </c>
       <c r="E391" t="str">
-        <v/>
+        <v>2026-06-12</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>Drip</v>
+      </c>
+      <c r="B392" t="str">
+        <v>House of Drips</v>
+      </c>
+      <c r="C392" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Category-level umbrella brochure covering the full drip menu, not an individual treatment line item -- no row existed in the original 285-row export. Brochure: house-of-drips-brochure.html.</v>
+      </c>
+      <c r="E392" t="str">
+        <v>2026-06-26</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>Qlara</v>
+      </c>
+      <c r="B393" t="str">
+        <v>Qlara</v>
+      </c>
+      <c r="C393" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="D393" t="str">
+        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html.</v>
+      </c>
+      <c r="E393" t="str">
+        <v>2026-07-16</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>Injectable</v>
+      </c>
+      <c r="B394" t="str">
+        <v>Dermal Fillers</v>
+      </c>
+      <c r="C394" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Existing brochure covering dermal fillers generally (closest Excel row was "Juvederm-Filler", a specific brand, not a match) -- no row existed for the generic treatment. Brochure: dermal-fillers-brochure.html.</v>
+      </c>
+      <c r="E394" t="str">
+        <v>2026-06-26</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>Lasar Hair Reduction</v>
+      </c>
+      <c r="B395" t="str">
+        <v>Laser Hair Reduction</v>
+      </c>
+      <c r="C395" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Existing brochure covering laser hair reduction generally -- the Excel only had specific device variants (Soprano Platinum/Titanium, Triton), no generic row. Brochure: laser-hair-reduction-brochure.html.</v>
+      </c>
+      <c r="E395" t="str">
+        <v>2026-06-27</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E395"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mark batch 8 brochures Completed in brochure.xlsx
Jet Peel Facial, Dermabrasion, Microdermabrasion, Acne Treatment, Acne
Scar Treatment, and Face Lift Filler all marked Completed with source
notes and dates. Fully reconciled again: all 89 brochures currently on
index.html have a matching Completed row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -2287,13 +2287,13 @@
         <v>Dolphin</v>
       </c>
       <c r="C111" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D111" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/jet-peel-facial-or-dolphin-facial/ [fuzzy]. Not yet built. [Duplicate name also appears at: row 145 (Hair)]</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html.</v>
       </c>
       <c r="E111" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="112">
@@ -2865,13 +2865,13 @@
         <v>Dolphin</v>
       </c>
       <c r="C145" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D145" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/jet-peel-facial-or-dolphin-facial/ [fuzzy]. Not yet built. [Duplicate name also appears at: row 111 (Facial)]</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html.</v>
       </c>
       <c r="E145" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="146">
@@ -5653,13 +5653,13 @@
         <v>Face Lift Filler</v>
       </c>
       <c r="C309" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D309" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-lift-filler-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/face-lift-filler-in-delhi. No before/after images on source page. Placed under Face Lifting. Brochure: face-lift-filler-brochure.html.</v>
       </c>
       <c r="E309" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="310">
@@ -5857,13 +5857,13 @@
         <v>Dermabrasion Treatment</v>
       </c>
       <c r="C321" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D321" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermabrasion-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html.</v>
       </c>
       <c r="E321" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="322">
@@ -5874,13 +5874,13 @@
         <v>Microdermabrasion Treatment</v>
       </c>
       <c r="C322" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D322" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/microdermabrasion-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/microdermabrasion-treatment. Real before/after composite image found and used. Placed under Facial. Brochure: microdermabrasion-treatment-brochure.html.</v>
       </c>
       <c r="E322" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="323">
@@ -6010,13 +6010,13 @@
         <v>Acne Treatment</v>
       </c>
       <c r="C330" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D330" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-treatment-in-bangalore/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/acne-treatment-in-bangalore. Hero/treatment photos only, not before/after. Placed under Facial. Brochure: acne-treatment-brochure.html.</v>
       </c>
       <c r="E330" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="331">
@@ -6027,13 +6027,13 @@
         <v>Acne Scar Treatment</v>
       </c>
       <c r="C331" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D331" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/acne-scar-treatment-in-gurgaon/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/acne-scar-treatment-in-gurgaon. Stock portrait photos only, not before/after. Placed under Facial. Brochure: acne-scar-treatment-brochure.html.</v>
       </c>
       <c r="E331" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="332">

</xml_diff>

<commit_message>
Mark batch 9 brochures Completed in brochure.xlsx
IntraGen, Ballancer Pro, Femme 360, Liquid Facelift, Sygma Lift, and
Under Eye Fillers all marked Completed with source notes and dates.
Fully reconciled again: all 95 brochures currently on index.html have
a matching Completed row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -723,13 +723,13 @@
         <v>Intragen</v>
       </c>
       <c r="C19" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D19" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/intragen-skin-tightening-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/intragen-skin-tightening-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: intragen-skin-tightening-brochure.html.</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="20">
@@ -5415,13 +5415,13 @@
         <v>Ballancer Pro</v>
       </c>
       <c r="C295" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D295" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ballancer-pro-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/ballancer-pro-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: ballancer-pro-brochure.html.</v>
       </c>
       <c r="E295" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="296">
@@ -5432,13 +5432,13 @@
         <v>Femme 360 Vaginal Tightening</v>
       </c>
       <c r="C296" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D296" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/femme-360-vaginal-tightening/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/femme-360-vaginal-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: femme-360-vaginal-tightening-brochure.html.</v>
       </c>
       <c r="E296" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="297">
@@ -5585,13 +5585,13 @@
         <v>Liquid Facelift</v>
       </c>
       <c r="C305" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D305" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/liquid-facelift-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/liquid-facelift-treatment. No before/after images on source page. Placed under Face Lifting. Brochure: liquid-facelift-brochure.html.</v>
       </c>
       <c r="E305" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="306">
@@ -5619,13 +5619,13 @@
         <v>Sygma Lift Treatment</v>
       </c>
       <c r="C307" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D307" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sygma-lift-treatment-in-gurgaon/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/sygma-lift-treatment-in-gurgaon. No before/after images on source page. Placed under Face Lifting. Brochure: sygma-lift-brochure.html.</v>
       </c>
       <c r="E307" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="308">
@@ -6146,13 +6146,13 @@
         <v>Under Eye Fillers Treatment</v>
       </c>
       <c r="C338" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D338" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/under-eye-fillers-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/under-eye-fillers-treatment. No before/after images on source page. Placed under Injectable. Brochure: under-eye-fillers-brochure.html.</v>
       </c>
       <c r="E338" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="339">

</xml_diff>

<commit_message>
Mark batch 10 brochures Completed in brochure.xlsx
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -5483,13 +5483,13 @@
         <v>HIFU Skin Tightening</v>
       </c>
       <c r="C299" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D299" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html.</v>
       </c>
       <c r="E299" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="300">
@@ -5670,13 +5670,13 @@
         <v>Square Jaw Treatment</v>
       </c>
       <c r="C310" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D310" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/square-jaw-treatment-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/square-jaw-treatment-in-delhi. Source images were generic treatment photos, not before/after -- none used. Note: this is a surgical jawline-implant procedure (general anesthesia), distinct in mechanism from the mostly non-surgical treatments elsewhere in Face Lifting -- kept in Face Lifting per its category match. Brochure: square-jaw-treatment-brochure.html.</v>
       </c>
       <c r="E310" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="311">
@@ -6163,13 +6163,13 @@
         <v>Melasma</v>
       </c>
       <c r="C339" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D339" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/melasma/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/melasma. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: melasma-treatment-brochure.html.</v>
       </c>
       <c r="E339" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="340">
@@ -6180,13 +6180,13 @@
         <v>Rosacea</v>
       </c>
       <c r="C340" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D340" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/rosacea/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/rosacea. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: rosacea-treatment-brochure.html.</v>
       </c>
       <c r="E340" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="341">
@@ -6214,13 +6214,13 @@
         <v>Keratosis Pilaris</v>
       </c>
       <c r="C342" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D342" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/keratosis-pilaris/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html.</v>
       </c>
       <c r="E342" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="343">
@@ -6282,13 +6282,13 @@
         <v>Stretch Marks</v>
       </c>
       <c r="C346" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D346" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stretch-marks/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/stretch-marks. Source had a banner image and one treatment image, not a before/after pair -- none used. Note: conceptually overlaps with the existing Derma Roller brochure, which lists stretch marks as one of its uses, but this dedicated page covers the fuller multi-modality approach (laser, MNRF, PRP/exosomes, peels) -- kept separate per its own sitemap URL/Excel row, flag if you want these consolidated. Placed under Facial. Brochure: stretch-marks-treatment-brochure.html.</v>
       </c>
       <c r="E346" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="347">

</xml_diff>

<commit_message>
Mark batch 11 brochures Completed in brochure.xlsx
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -5347,13 +5347,13 @@
         <v>House of Sculpt</v>
       </c>
       <c r="C291" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D291" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-sculpt/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html.</v>
       </c>
       <c r="E291" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="292">
@@ -5364,13 +5364,13 @@
         <v>House of Proportion</v>
       </c>
       <c r="C292" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D292" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/house-of-proportion/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html.</v>
       </c>
       <c r="E292" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="293">
@@ -5398,13 +5398,13 @@
         <v>Tight Pro</v>
       </c>
       <c r="C294" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D294" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tight-pro/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html.</v>
       </c>
       <c r="E294" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="295">
@@ -5466,13 +5466,13 @@
         <v>Multipolar Radio Frequency</v>
       </c>
       <c r="C298" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D298" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/multipolar-radio-frequency-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html.</v>
       </c>
       <c r="E298" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="299">
@@ -5687,13 +5687,13 @@
         <v>Poppy Chin Treatment</v>
       </c>
       <c r="C311" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D311" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/poppy-chin-treatment-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html.</v>
       </c>
       <c r="E311" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="312">
@@ -5704,13 +5704,13 @@
         <v>BR Facial</v>
       </c>
       <c r="C312" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D312" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/br-facial/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/br-facial that "BR Facial" is the same Biologique Recherche treatment (same brand, same Lotion P50 cleanser/mechanism) as the existing biologique-recherche-facial-brochure.html -- no new brochure built, this row is covered by that existing file (Facial category).</v>
       </c>
       <c r="E312" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="313">
@@ -5721,13 +5721,13 @@
         <v>Eve Lom Facial</v>
       </c>
       <c r="C313" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D313" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eve-lom-facial/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html.</v>
       </c>
       <c r="E313" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="314">

</xml_diff>

<commit_message>
Mark batch 12/13 brochures Completed in brochure.xlsx; merge QR678 Neo, Injection Kenacort, Calecim Product, and Soprano Ice Platinum/Titanium into existing brochures
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$395</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3460,13 +3460,13 @@
         <v>Injection Kenacort</v>
       </c>
       <c r="C180" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D180" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Previously "Missing - No Source" -- this is the same treatment as the "Kenacort Injection" row (reversed word order), which was built this session from isaacluxe.co/kenacort-injection. Brochure: kenacort-injection-brochure.html.</v>
       </c>
       <c r="E180" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="181">
@@ -5517,13 +5517,13 @@
         <v>Sculpt Tone Plus</v>
       </c>
       <c r="C301" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D301" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sculptone-plus/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/sculptone-plus. No before/after images on source page; source page also gave no explicit session count/frequency. Note: conceptually similar in goal (fat reduction + muscle building) to the existing Emsculpt NEO brochure. Placed under Body Contouring. Brochure: sculpt-tone-plus-brochure.html.</v>
       </c>
       <c r="E301" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="302">
@@ -5534,13 +5534,13 @@
         <v>Cool Tech</v>
       </c>
       <c r="C302" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D302" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cool-tech/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/cool-tech. One banner image found, not a before/after pair. Note: this is a cooling/cryolipolysis-based fat-freezing technology, likely the same core mechanism as the existing Cryolipolysis and CoolSculpting brochures (three separate branded fat-freezing entries now) -- kept as its own distinct catalog item per its own sitemap page, flag if you would like these consolidated or cross-referenced. Placed under Body Contouring. Brochure: cool-tech-brochure.html.</v>
       </c>
       <c r="E302" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="303">
@@ -6469,13 +6469,13 @@
         <v>Fat Lipolysis Injection</v>
       </c>
       <c r="C357" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D357" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fat-lipolysis-injection/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/fat-lipolysis-injection. No before/after images on source page. Placed under Injectable. Brochure: fat-lipolysis-injection-brochure.html.</v>
       </c>
       <c r="E357" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="358">
@@ -6486,13 +6486,13 @@
         <v>Kenacort Injection</v>
       </c>
       <c r="C358" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D358" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/kenacort-injection/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/kenacort-injection. No before/after images on source page. Placed under Injectable. Brochure: kenacort-injection-brochure.html.</v>
       </c>
       <c r="E358" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="359">
@@ -6520,13 +6520,13 @@
         <v>Hyaluron Pen (Needle-Free Filler)</v>
       </c>
       <c r="C360" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D360" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluron-pen-needle-free-filler/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html.</v>
       </c>
       <c r="E360" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="361">
@@ -6554,13 +6554,13 @@
         <v>Viscoderm Hydrobooster</v>
       </c>
       <c r="C362" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D362" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/viscoderm-hydrobooster/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html.</v>
       </c>
       <c r="E362" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="363">
@@ -6588,13 +6588,13 @@
         <v>Calecim Professional Brand</v>
       </c>
       <c r="C364" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D364" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-professional-brand/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/calecim-professional-brand. One product image found, not before/after. Placed under Injectable. Brochure: calecim-professional-brochure.html.</v>
       </c>
       <c r="E364" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="365">
@@ -6639,13 +6639,13 @@
         <v>Non-Surgical Hair Replacement</v>
       </c>
       <c r="C367" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D367" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/non-surgical-hair-replacement/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-hair-replacement. One product image found, not before/after. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: non-surgical-hair-replacement-brochure.html.</v>
       </c>
       <c r="E367" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="368">
@@ -6656,13 +6656,13 @@
         <v>Hairgen Booster</v>
       </c>
       <c r="C368" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D368" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hairgen-booster/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html.</v>
       </c>
       <c r="E368" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="369">
@@ -6673,13 +6673,13 @@
         <v>PRP Hair Treatment</v>
       </c>
       <c r="C369" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D369" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-hair-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html.</v>
       </c>
       <c r="E369" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="370">
@@ -6758,13 +6758,13 @@
         <v>Alopecia Areata</v>
       </c>
       <c r="C374" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D374" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/alopecia-areata/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html.</v>
       </c>
       <c r="E374" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="375">
@@ -6775,13 +6775,13 @@
         <v>QR-678 Neo Hair Growth</v>
       </c>
       <c r="C375" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D375" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/qr-678-neo-hair-growth-and-hair-qr-treatment/. Not yet built.</v>
+        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category).</v>
       </c>
       <c r="E375" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="376">
@@ -6809,13 +6809,13 @@
         <v>Soprano Ice Platinum</v>
       </c>
       <c r="C377" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D377" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-platinum/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/soprano-ice-platinum that this Alma Soprano ICE Platinum device uses the same triple-wavelength (755nm Alexandrite / 810nm Diode / 1064nm Nd:YAG) technology already documented in the existing laser-hair-reduction-brochure.html (built around Soprano Titanium). Per user decision, treated as the same core device -- no new brochure built, this row is covered by the existing Laser Hair Reduction brochure.</v>
       </c>
       <c r="E377" t="str">
-        <v/>
+        <v>2026-06-27</v>
       </c>
     </row>
     <row r="378">
@@ -6826,13 +6826,13 @@
         <v>Soprano Ice Titanium</v>
       </c>
       <c r="C378" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D378" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/soprano-ice-titanium/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/soprano-ice-titanium that this device has essentially identical specs (same 3 wavelengths, ICE cooling, ~30-min sessions) to the existing laser-hair-reduction-brochure.html, which is already built around Soprano Titanium. No new brochure built, this row is covered by the existing Laser Hair Reduction brochure.</v>
       </c>
       <c r="E378" t="str">
-        <v/>
+        <v>2026-06-27</v>
       </c>
     </row>
     <row r="379">
@@ -6996,13 +6996,13 @@
         <v>Calecim Product</v>
       </c>
       <c r="C388" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D388" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/calecim-product/. Not yet built.</v>
+        <v>Source URL isaacluxe.co/calecim-product/ returns an HTTP 301 redirect, landing on the same content already scraped as "Calecim Professional Brand". Same product, old URL slug. Brochure: calecim-professional-brochure.html.</v>
       </c>
       <c r="E388" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="389">

</xml_diff>

<commit_message>
Document photo additions and gaps in brochure.xlsx
Notes which of the 117 treatment brochures received a real isaacluxe.co
photo this pass (69 rows / 62 unique files) and which of the 23
remaining have no photo, with the specific reason for each (no
compliant source page, zero images on the source page, or mismatched
image content).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,8 +402,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="100.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
@@ -522,7 +522,7 @@
         <v>Completed</v>
       </c>
       <c r="D7" t="str">
-        <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E7" t="str">
         <v>2026-07-24</v>
@@ -658,7 +658,7 @@
         <v>Completed</v>
       </c>
       <c r="D15" t="str">
-        <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E15" t="str">
         <v>2026-07-24</v>
@@ -726,7 +726,7 @@
         <v>Completed</v>
       </c>
       <c r="D19" t="str">
-        <v>Scraped from isaacluxe.co/intragen-skin-tightening-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: intragen-skin-tightening-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/intragen-skin-tightening-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: intragen-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E19" t="str">
         <v>2026-07-25</v>
@@ -760,7 +760,7 @@
         <v>Completed</v>
       </c>
       <c r="D21" t="str">
-        <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E21" t="str">
         <v>2026-07-25</v>
@@ -896,7 +896,7 @@
         <v>Completed</v>
       </c>
       <c r="D29" t="str">
-        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E29" t="str">
         <v>2026-07-25</v>
@@ -913,7 +913,7 @@
         <v>Completed</v>
       </c>
       <c r="D30" t="str">
-        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E30" t="str">
         <v>2026-07-25</v>
@@ -998,7 +998,7 @@
         <v>Completed</v>
       </c>
       <c r="D35" t="str">
-        <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E35" t="str">
         <v>2026-07-25</v>
@@ -1015,7 +1015,7 @@
         <v>Completed</v>
       </c>
       <c r="D36" t="str">
-        <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built.</v>
+        <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E36" t="str">
         <v>2026-07-24</v>
@@ -1202,7 +1202,7 @@
         <v>Completed</v>
       </c>
       <c r="D47" t="str">
-        <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E47" t="str">
         <v>2026-07-24</v>
@@ -1270,7 +1270,7 @@
         <v>Completed</v>
       </c>
       <c r="D51" t="str">
-        <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E51" t="str">
         <v>2026-07-25</v>
@@ -1355,7 +1355,7 @@
         <v>Completed</v>
       </c>
       <c r="D56" t="str">
-        <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E56" t="str">
         <v>2026-06-12</v>
@@ -1389,7 +1389,7 @@
         <v>Completed</v>
       </c>
       <c r="D58" t="str">
-        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact]</v>
+        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added.</v>
       </c>
       <c r="E58" t="str">
         <v>2026-07-15</v>
@@ -1406,7 +1406,7 @@
         <v>Completed</v>
       </c>
       <c r="D59" t="str">
-        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial").</v>
+        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E59" t="str">
         <v>2026-07-15</v>
@@ -1457,7 +1457,7 @@
         <v>Completed</v>
       </c>
       <c r="D62" t="str">
-        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact]</v>
+        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E62" t="str">
         <v>2026-07-15</v>
@@ -1525,7 +1525,7 @@
         <v>Completed</v>
       </c>
       <c r="D66" t="str">
-        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact]</v>
+        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E66" t="str">
         <v>2026-07-15</v>
@@ -1593,7 +1593,7 @@
         <v>Completed</v>
       </c>
       <c r="D70" t="str">
-        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E70" t="str">
         <v>2026-07-15</v>
@@ -1610,7 +1610,7 @@
         <v>Completed</v>
       </c>
       <c r="D71" t="str">
-        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact]</v>
+        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E71" t="str">
         <v>2026-07-15</v>
@@ -1661,7 +1661,7 @@
         <v>Completed</v>
       </c>
       <c r="D74" t="str">
-        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact]</v>
+        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E74" t="str">
         <v>2026-07-15</v>
@@ -1950,7 +1950,7 @@
         <v>Completed</v>
       </c>
       <c r="D91" t="str">
-        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact]</v>
+        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E91" t="str">
         <v>2026-07-15</v>
@@ -2018,7 +2018,7 @@
         <v>Completed</v>
       </c>
       <c r="D95" t="str">
-        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact]</v>
+        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E95" t="str">
         <v>2026-07-15</v>
@@ -2035,7 +2035,7 @@
         <v>Completed</v>
       </c>
       <c r="D96" t="str">
-        <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E96" t="str">
         <v>2026-07-24</v>
@@ -2154,7 +2154,7 @@
         <v>Completed</v>
       </c>
       <c r="D103" t="str">
-        <v>Scraped from isaacluxe.co/biologique. No before/after images on source page. Placed under Facial. Brochure: biologique-recherche-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/biologique. No before/after images on source page. Placed under Facial. Brochure: biologique-recherche-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E103" t="str">
         <v>2026-07-25</v>
@@ -2256,7 +2256,7 @@
         <v>Completed</v>
       </c>
       <c r="D109" t="str">
-        <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E109" t="str">
         <v>2026-07-25</v>
@@ -2290,7 +2290,7 @@
         <v>Completed</v>
       </c>
       <c r="D111" t="str">
-        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E111" t="str">
         <v>2026-07-25</v>
@@ -2324,7 +2324,7 @@
         <v>Completed</v>
       </c>
       <c r="D113" t="str">
-        <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E113" t="str">
         <v>2026-07-24</v>
@@ -2392,7 +2392,7 @@
         <v>Completed</v>
       </c>
       <c r="D117" t="str">
-        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E117" t="str">
         <v>2026-07-24</v>
@@ -2409,7 +2409,7 @@
         <v>Completed</v>
       </c>
       <c r="D118" t="str">
-        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E118" t="str">
         <v>2026-07-24</v>
@@ -2443,7 +2443,7 @@
         <v>Completed</v>
       </c>
       <c r="D120" t="str">
-        <v>Scraped from isaacluxe.co/ice-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: ice-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/ice-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: ice-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E120" t="str">
         <v>2026-07-25</v>
@@ -2494,7 +2494,7 @@
         <v>Completed</v>
       </c>
       <c r="D123" t="str">
-        <v>Scraped from isaacluxe.co/love-light-fusion-facial. No before/after images on source page. Placed under Facial. Brochure: love-light-fusion-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/love-light-fusion-facial. No before/after images on source page. Placed under Facial. Brochure: love-light-fusion-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E123" t="str">
         <v>2026-07-25</v>
@@ -2545,7 +2545,7 @@
         <v>Completed</v>
       </c>
       <c r="D126" t="str">
-        <v>Scraped from isaacluxe.co/oasis-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: oasis-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/oasis-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: oasis-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E126" t="str">
         <v>2026-07-25</v>
@@ -2562,7 +2562,7 @@
         <v>Completed</v>
       </c>
       <c r="D127" t="str">
-        <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E127" t="str">
         <v>2026-07-24</v>
@@ -2579,7 +2579,7 @@
         <v>Completed</v>
       </c>
       <c r="D128" t="str">
-        <v>Scraped from isaacluxe.co/oxygeneo-facial-best-oxygen-facial. No before/after images on source page. Placed under Facial. Brochure: oxygeneo-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/oxygeneo-facial-best-oxygen-facial. No before/after images on source page. Placed under Facial. Brochure: oxygeneo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E128" t="str">
         <v>2026-07-25</v>
@@ -2698,7 +2698,7 @@
         <v>Completed</v>
       </c>
       <c r="D135" t="str">
-        <v>Scraped from isaacluxe.co/salmon-dna-pdrn-facial. Only banner/decorative images found, not before/after. Placed under Facial. Brochure: salmon-dna-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/salmon-dna-pdrn-facial. Only banner/decorative images found, not before/after. Placed under Facial. Brochure: salmon-dna-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E135" t="str">
         <v>2026-07-25</v>
@@ -2766,7 +2766,7 @@
         <v>Completed</v>
       </c>
       <c r="D139" t="str">
-        <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E139" t="str">
         <v>2026-07-24</v>
@@ -2817,7 +2817,7 @@
         <v>Completed</v>
       </c>
       <c r="D142" t="str">
-        <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E142" t="str">
         <v>2026-07-25</v>
@@ -2868,7 +2868,7 @@
         <v>Completed</v>
       </c>
       <c r="D145" t="str">
-        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E145" t="str">
         <v>2026-07-25</v>
@@ -3004,7 +3004,7 @@
         <v>Completed</v>
       </c>
       <c r="D153" t="str">
-        <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E153" t="str">
         <v>2026-07-24</v>
@@ -3463,7 +3463,7 @@
         <v>Completed</v>
       </c>
       <c r="D180" t="str">
-        <v>Previously "Missing - No Source" -- this is the same treatment as the "Kenacort Injection" row (reversed word order), which was built this session from isaacluxe.co/kenacort-injection. Brochure: kenacort-injection-brochure.html.</v>
+        <v>Previously "Missing - No Source" -- this is the same treatment as the "Kenacort Injection" row (reversed word order), which was built this session from isaacluxe.co/kenacort-injection. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E180" t="str">
         <v>2026-07-25</v>
@@ -3667,7 +3667,7 @@
         <v>Completed</v>
       </c>
       <c r="D192" t="str">
-        <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E192" t="str">
         <v>2026-07-24</v>
@@ -3803,7 +3803,7 @@
         <v>Completed</v>
       </c>
       <c r="D200" t="str">
-        <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E200" t="str">
         <v>2026-07-24</v>
@@ -4007,7 +4007,7 @@
         <v>Completed</v>
       </c>
       <c r="D212" t="str">
-        <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E212" t="str">
         <v>2026-07-24</v>
@@ -5265,7 +5265,7 @@
         <v>Completed</v>
       </c>
       <c r="D286" t="str">
-        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E286" t="str">
         <v>2026-07-24</v>
@@ -5282,7 +5282,7 @@
         <v>Completed</v>
       </c>
       <c r="D287" t="str">
-        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E287" t="str">
         <v>2026-07-24</v>
@@ -5299,7 +5299,7 @@
         <v>Completed</v>
       </c>
       <c r="D288" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E288" t="str">
         <v>2026-07-24</v>
@@ -5316,7 +5316,7 @@
         <v>Completed</v>
       </c>
       <c r="D289" t="str">
-        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E289" t="str">
         <v>2026-07-24</v>
@@ -5333,7 +5333,7 @@
         <v>Completed</v>
       </c>
       <c r="D290" t="str">
-        <v>Scraped from isaacluxe.co/instasculpt. No before/after images on source page. Placed under Body Contouring. Brochure: instasculpt-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/instasculpt. No before/after images on source page. Placed under Body Contouring. Brochure: instasculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E290" t="str">
         <v>2026-07-25</v>
@@ -5350,7 +5350,7 @@
         <v>Completed</v>
       </c>
       <c r="D291" t="str">
-        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E291" t="str">
         <v>2026-07-25</v>
@@ -5367,7 +5367,7 @@
         <v>Completed</v>
       </c>
       <c r="D292" t="str">
-        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E292" t="str">
         <v>2026-07-25</v>
@@ -5384,7 +5384,7 @@
         <v>Completed</v>
       </c>
       <c r="D293" t="str">
-        <v>Scraped from isaacluxe.co/tummy-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: tummy-tightening-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/tummy-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: tummy-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E293" t="str">
         <v>2026-07-25</v>
@@ -5401,7 +5401,7 @@
         <v>Completed</v>
       </c>
       <c r="D294" t="str">
-        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E294" t="str">
         <v>2026-07-25</v>
@@ -5418,7 +5418,7 @@
         <v>Completed</v>
       </c>
       <c r="D295" t="str">
-        <v>Scraped from isaacluxe.co/ballancer-pro-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: ballancer-pro-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/ballancer-pro-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: ballancer-pro-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E295" t="str">
         <v>2026-07-25</v>
@@ -5435,7 +5435,7 @@
         <v>Completed</v>
       </c>
       <c r="D296" t="str">
-        <v>Scraped from isaacluxe.co/femme-360-vaginal-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: femme-360-vaginal-tightening-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/femme-360-vaginal-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: femme-360-vaginal-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E296" t="str">
         <v>2026-07-25</v>
@@ -5452,7 +5452,7 @@
         <v>Completed</v>
       </c>
       <c r="D297" t="str">
-        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E297" t="str">
         <v>2026-07-24</v>
@@ -5469,7 +5469,7 @@
         <v>Completed</v>
       </c>
       <c r="D298" t="str">
-        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E298" t="str">
         <v>2026-07-25</v>
@@ -5486,7 +5486,7 @@
         <v>Completed</v>
       </c>
       <c r="D299" t="str">
-        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E299" t="str">
         <v>2026-07-25</v>
@@ -5520,7 +5520,7 @@
         <v>Completed</v>
       </c>
       <c r="D301" t="str">
-        <v>Scraped from isaacluxe.co/sculptone-plus. No before/after images on source page; source page also gave no explicit session count/frequency. Note: conceptually similar in goal (fat reduction + muscle building) to the existing Emsculpt NEO brochure. Placed under Body Contouring. Brochure: sculpt-tone-plus-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/sculptone-plus. No before/after images on source page; source page also gave no explicit session count/frequency. Note: conceptually similar in goal (fat reduction + muscle building) to the existing Emsculpt NEO brochure. Placed under Body Contouring. Brochure: sculpt-tone-plus-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E301" t="str">
         <v>2026-07-25</v>
@@ -5537,7 +5537,7 @@
         <v>Completed</v>
       </c>
       <c r="D302" t="str">
-        <v>Scraped from isaacluxe.co/cool-tech. One banner image found, not a before/after pair. Note: this is a cooling/cryolipolysis-based fat-freezing technology, likely the same core mechanism as the existing Cryolipolysis and CoolSculpting brochures (three separate branded fat-freezing entries now) -- kept as its own distinct catalog item per its own sitemap page, flag if you would like these consolidated or cross-referenced. Placed under Body Contouring. Brochure: cool-tech-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/cool-tech. One banner image found, not a before/after pair. Note: this is a cooling/cryolipolysis-based fat-freezing technology, likely the same core mechanism as the existing Cryolipolysis and CoolSculpting brochures (three separate branded fat-freezing entries now) -- kept as its own distinct catalog item per its own sitemap page, flag if you would like these consolidated or cross-referenced. Placed under Body Contouring. Brochure: cool-tech-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E302" t="str">
         <v>2026-07-25</v>
@@ -5571,7 +5571,7 @@
         <v>Completed</v>
       </c>
       <c r="D304" t="str">
-        <v>Scraped from isaacluxe.co/thread-face-lift-treatment. Note: conceptually overlaps with the existing "Thread Lift" and "Aptos Thread Lift" brochures (all use PDO/PLLA-style threads), but is its own distinct catalog line item, so built separately -- flag if you want these consolidated. No before/after photos (only hero images). Placed under Face Lifting. Brochure: thread-face-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/thread-face-lift-treatment. Note: conceptually overlaps with the existing "Thread Lift" and "Aptos Thread Lift" brochures (all use PDO/PLLA-style threads), but is its own distinct catalog line item, so built separately -- flag if you want these consolidated. No before/after photos (only hero images). Placed under Face Lifting. Brochure: thread-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E304" t="str">
         <v>2026-07-25</v>
@@ -5588,7 +5588,7 @@
         <v>Completed</v>
       </c>
       <c r="D305" t="str">
-        <v>Scraped from isaacluxe.co/liquid-facelift-treatment. No before/after images on source page. Placed under Face Lifting. Brochure: liquid-facelift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/liquid-facelift-treatment. No before/after images on source page. Placed under Face Lifting. Brochure: liquid-facelift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E305" t="str">
         <v>2026-07-25</v>
@@ -5605,7 +5605,7 @@
         <v>Completed</v>
       </c>
       <c r="D306" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E306" t="str">
         <v>2026-07-24</v>
@@ -5622,7 +5622,7 @@
         <v>Completed</v>
       </c>
       <c r="D307" t="str">
-        <v>Scraped from isaacluxe.co/sygma-lift-treatment-in-gurgaon. No before/after images on source page. Placed under Face Lifting. Brochure: sygma-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/sygma-lift-treatment-in-gurgaon. No before/after images on source page. Placed under Face Lifting. Brochure: sygma-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E307" t="str">
         <v>2026-07-25</v>
@@ -5639,7 +5639,7 @@
         <v>Completed</v>
       </c>
       <c r="D308" t="str">
-        <v>Scraped from isaacluxe.co/4-d-lift. No before/after images on source page. Placed under Face Lifting. Brochure: 4d-lift-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/4-d-lift. No before/after images on source page. Placed under Face Lifting. Brochure: 4d-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E308" t="str">
         <v>2026-07-25</v>
@@ -5656,7 +5656,7 @@
         <v>Completed</v>
       </c>
       <c r="D309" t="str">
-        <v>Scraped from isaacluxe.co/face-lift-filler-in-delhi. No before/after images on source page. Placed under Face Lifting. Brochure: face-lift-filler-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/face-lift-filler-in-delhi. No before/after images on source page. Placed under Face Lifting. Brochure: face-lift-filler-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E309" t="str">
         <v>2026-07-25</v>
@@ -5673,7 +5673,7 @@
         <v>Completed</v>
       </c>
       <c r="D310" t="str">
-        <v>Scraped from isaacluxe.co/square-jaw-treatment-in-delhi. Source images were generic treatment photos, not before/after -- none used. Note: this is a surgical jawline-implant procedure (general anesthesia), distinct in mechanism from the mostly non-surgical treatments elsewhere in Face Lifting -- kept in Face Lifting per its category match. Brochure: square-jaw-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/square-jaw-treatment-in-delhi. Source images were generic treatment photos, not before/after -- none used. Note: this is a surgical jawline-implant procedure (general anesthesia), distinct in mechanism from the mostly non-surgical treatments elsewhere in Face Lifting -- kept in Face Lifting per its category match. Brochure: square-jaw-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E310" t="str">
         <v>2026-07-25</v>
@@ -5690,7 +5690,7 @@
         <v>Completed</v>
       </c>
       <c r="D311" t="str">
-        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E311" t="str">
         <v>2026-07-25</v>
@@ -5707,7 +5707,7 @@
         <v>Completed</v>
       </c>
       <c r="D312" t="str">
-        <v>Confirmed via isaacluxe.co/br-facial that "BR Facial" is the same Biologique Recherche treatment (same brand, same Lotion P50 cleanser/mechanism) as the existing biologique-recherche-facial-brochure.html -- no new brochure built, this row is covered by that existing file (Facial category).</v>
+        <v>Confirmed via isaacluxe.co/br-facial that "BR Facial" is the same Biologique Recherche treatment (same brand, same Lotion P50 cleanser/mechanism) as the existing biologique-recherche-facial-brochure.html -- no new brochure built, this row is covered by that existing file (Facial category). Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E312" t="str">
         <v>2026-07-25</v>
@@ -5724,7 +5724,7 @@
         <v>Completed</v>
       </c>
       <c r="D313" t="str">
-        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E313" t="str">
         <v>2026-07-25</v>
@@ -5843,7 +5843,7 @@
         <v>Completed</v>
       </c>
       <c r="D320" t="str">
-        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E320" t="str">
         <v>2026-07-25</v>
@@ -5860,7 +5860,7 @@
         <v>Completed</v>
       </c>
       <c r="D321" t="str">
-        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html. PHOTO CHECK: source page's only non-logo image was mislabeled/mismatched (a photo captioned "Ultherapy" appearing on the Dermabrasion page) -- not used to avoid misrepresenting the treatment. No photo added.</v>
       </c>
       <c r="E321" t="str">
         <v>2026-07-25</v>
@@ -5894,7 +5894,7 @@
         <v>Completed</v>
       </c>
       <c r="D323" t="str">
-        <v>Scraped from isaacluxe.co/skin-polishing (a body-wide treatment; titled "Body Polishing" in the brochure). No before/after images on source page. Placed under Facial as closest fit. Brochure: skin-polishing-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/skin-polishing (a body-wide treatment; titled "Body Polishing" in the brochure). No before/after images on source page. Placed under Facial as closest fit. Brochure: skin-polishing-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E323" t="str">
         <v>2026-07-25</v>
@@ -5911,7 +5911,7 @@
         <v>Completed</v>
       </c>
       <c r="D324" t="str">
-        <v>Scraped from isaacluxe.co/dermamelan-treatment. Only a process-diagram image found, not before/after. Placed under Facial. Brochure: dermamelan-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/dermamelan-treatment. Only a process-diagram image found, not before/after. Placed under Facial. Brochure: dermamelan-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E324" t="str">
         <v>2026-07-25</v>
@@ -6013,7 +6013,7 @@
         <v>Completed</v>
       </c>
       <c r="D330" t="str">
-        <v>Scraped from isaacluxe.co/acne-treatment-in-bangalore. Hero/treatment photos only, not before/after. Placed under Facial. Brochure: acne-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/acne-treatment-in-bangalore. Hero/treatment photos only, not before/after. Placed under Facial. Brochure: acne-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E330" t="str">
         <v>2026-07-25</v>
@@ -6030,7 +6030,7 @@
         <v>Completed</v>
       </c>
       <c r="D331" t="str">
-        <v>Scraped from isaacluxe.co/acne-scar-treatment-in-gurgaon. Stock portrait photos only, not before/after. Placed under Facial. Brochure: acne-scar-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/acne-scar-treatment-in-gurgaon. Stock portrait photos only, not before/after. Placed under Facial. Brochure: acne-scar-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E331" t="str">
         <v>2026-07-25</v>
@@ -6149,7 +6149,7 @@
         <v>Completed</v>
       </c>
       <c r="D338" t="str">
-        <v>Scraped from isaacluxe.co/under-eye-fillers-treatment. No before/after images on source page. Placed under Injectable. Brochure: under-eye-fillers-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/under-eye-fillers-treatment. No before/after images on source page. Placed under Injectable. Brochure: under-eye-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E338" t="str">
         <v>2026-07-25</v>
@@ -6166,7 +6166,7 @@
         <v>Completed</v>
       </c>
       <c r="D339" t="str">
-        <v>Scraped from isaacluxe.co/melasma. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: melasma-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/melasma. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: melasma-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E339" t="str">
         <v>2026-07-25</v>
@@ -6183,7 +6183,7 @@
         <v>Completed</v>
       </c>
       <c r="D340" t="str">
-        <v>Scraped from isaacluxe.co/rosacea. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: rosacea-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/rosacea. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: rosacea-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E340" t="str">
         <v>2026-07-25</v>
@@ -6217,7 +6217,7 @@
         <v>Completed</v>
       </c>
       <c r="D342" t="str">
-        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E342" t="str">
         <v>2026-07-25</v>
@@ -6285,7 +6285,7 @@
         <v>Completed</v>
       </c>
       <c r="D346" t="str">
-        <v>Scraped from isaacluxe.co/stretch-marks. Source had a banner image and one treatment image, not a before/after pair -- none used. Note: conceptually overlaps with the existing Derma Roller brochure, which lists stretch marks as one of its uses, but this dedicated page covers the fuller multi-modality approach (laser, MNRF, PRP/exosomes, peels) -- kept separate per its own sitemap URL/Excel row, flag if you want these consolidated. Placed under Facial. Brochure: stretch-marks-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/stretch-marks. Source had a banner image and one treatment image, not a before/after pair -- none used. Note: conceptually overlaps with the existing Derma Roller brochure, which lists stretch marks as one of its uses, but this dedicated page covers the fuller multi-modality approach (laser, MNRF, PRP/exosomes, peels) -- kept separate per its own sitemap URL/Excel row, flag if you want these consolidated. Placed under Facial. Brochure: stretch-marks-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E346" t="str">
         <v>2026-07-25</v>
@@ -6438,7 +6438,7 @@
         <v>Completed</v>
       </c>
       <c r="D355" t="str">
-        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E355" t="str">
         <v>2026-07-24</v>
@@ -6472,7 +6472,7 @@
         <v>Completed</v>
       </c>
       <c r="D357" t="str">
-        <v>Scraped from isaacluxe.co/fat-lipolysis-injection. No before/after images on source page. Placed under Injectable. Brochure: fat-lipolysis-injection-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/fat-lipolysis-injection. No before/after images on source page. Placed under Injectable. Brochure: fat-lipolysis-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E357" t="str">
         <v>2026-07-25</v>
@@ -6489,7 +6489,7 @@
         <v>Completed</v>
       </c>
       <c r="D358" t="str">
-        <v>Scraped from isaacluxe.co/kenacort-injection. No before/after images on source page. Placed under Injectable. Brochure: kenacort-injection-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/kenacort-injection. No before/after images on source page. Placed under Injectable. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E358" t="str">
         <v>2026-07-25</v>
@@ -6523,7 +6523,7 @@
         <v>Completed</v>
       </c>
       <c r="D360" t="str">
-        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E360" t="str">
         <v>2026-07-25</v>
@@ -6557,7 +6557,7 @@
         <v>Completed</v>
       </c>
       <c r="D362" t="str">
-        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E362" t="str">
         <v>2026-07-25</v>
@@ -6591,7 +6591,7 @@
         <v>Completed</v>
       </c>
       <c r="D364" t="str">
-        <v>Scraped from isaacluxe.co/calecim-professional-brand. One product image found, not before/after. Placed under Injectable. Brochure: calecim-professional-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/calecim-professional-brand. One product image found, not before/after. Placed under Injectable. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E364" t="str">
         <v>2026-07-25</v>
@@ -6608,7 +6608,7 @@
         <v>Completed</v>
       </c>
       <c r="D365" t="str">
-        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html. PHOTO CHECK: source page has only the generic site logo and footer photo, no treatment-specific image. No photo added.</v>
       </c>
       <c r="E365" t="str">
         <v>2026-07-24</v>
@@ -6625,7 +6625,7 @@
         <v>Completed</v>
       </c>
       <c r="D366" t="str">
-        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E366" t="str">
         <v>2026-07-24</v>
@@ -6642,7 +6642,7 @@
         <v>Completed</v>
       </c>
       <c r="D367" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-hair-replacement. One product image found, not before/after. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: non-surgical-hair-replacement-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/non-surgical-hair-replacement. One product image found, not before/after. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: non-surgical-hair-replacement-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E367" t="str">
         <v>2026-07-25</v>
@@ -6659,7 +6659,7 @@
         <v>Completed</v>
       </c>
       <c r="D368" t="str">
-        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E368" t="str">
         <v>2026-07-25</v>
@@ -6676,7 +6676,7 @@
         <v>Completed</v>
       </c>
       <c r="D369" t="str">
-        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E369" t="str">
         <v>2026-07-25</v>
@@ -6761,7 +6761,7 @@
         <v>Completed</v>
       </c>
       <c r="D374" t="str">
-        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
       </c>
       <c r="E374" t="str">
         <v>2026-07-25</v>
@@ -6999,7 +6999,7 @@
         <v>Completed</v>
       </c>
       <c r="D388" t="str">
-        <v>Source URL isaacluxe.co/calecim-product/ returns an HTTP 301 redirect, landing on the same content already scraped as "Calecim Professional Brand". Same product, old URL slug. Brochure: calecim-professional-brochure.html.</v>
+        <v>Source URL isaacluxe.co/calecim-product/ returns an HTTP 301 redirect, landing on the same content already scraped as "Calecim Professional Brand". Same product, old URL slug. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
       </c>
       <c r="E388" t="str">
         <v>2026-07-25</v>
@@ -7084,7 +7084,7 @@
         <v>Completed</v>
       </c>
       <c r="D393" t="str">
-        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html.</v>
+        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html. PHOTO CHECK: no corresponding live isaacluxe.co page exists for Qlara (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
       </c>
       <c r="E393" t="str">
         <v>2026-07-16</v>

</xml_diff>

<commit_message>
Mark batch 14 brochures Completed in brochure.xlsx; merge Tear Trough Treatment and Hyperbaric Oxygen Therapy into existing brochures
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,8 +402,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="100.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
@@ -2780,13 +2780,13 @@
         <v>V BIANCO</v>
       </c>
       <c r="C140" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D140" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/v-bianco-skin-lightening-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/v-bianco-skin-lightening-treatment. Real treatment banner image found and used. Placed under Facial. Brochure: v-bianco-brochure.html.</v>
       </c>
       <c r="E140" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="141">
@@ -2797,13 +2797,13 @@
         <v>V Carbon</v>
       </c>
       <c r="C141" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D141" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/v-carbon-treatment/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/v-carbon-treatment (also called "Erase Treatment"). Note: conceptually adjacent to the existing Carbon Facial brochure, but a distinct mechanism -- V Carbon is a topical film/spray system (no laser), while Carbon Facial is laser-based -- kept separate, flag if you disagree. Source page images were generic/mismatched stock photos of facial masks, not clearly specific to this treatment -- none used. Placed under Facial. Brochure: v-carbon-brochure.html.</v>
       </c>
       <c r="E141" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="142">
@@ -5772,13 +5772,13 @@
         <v>Meso Glow</v>
       </c>
       <c r="C316" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D316" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/meso-glow/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/meso-glow. Real treatment image found and used. Note: conceptually overlaps with the existing Mesotherapy brochure (both are micro-injected vitamin/nutrient infusions), but MesoGlow is its own named protocol with a distinct ingredient profile (HA/vitamin C/E) and timeline -- kept separate, flag if you want these consolidated. Placed under Facial. Brochure: meso-glow-brochure.html.</v>
       </c>
       <c r="E316" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="317">
@@ -6112,13 +6112,13 @@
         <v>Dark Circles</v>
       </c>
       <c r="C336" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D336" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dark-circles/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/dark-circles. This is a condition/menu page listing multiple approaches (fillers, Eye Light, peels, laser) similar in structure to the Melasma/Rosacea/Square Jaw pattern -- two of its named modalities (Eye Light, Under Eye/Tear Trough Fillers) already have their own dedicated brochures, referenced here as part of the combined protocol rather than duplicated. No images found on the source page. Placed under Facial. Brochure: dark-circles-treatment-brochure.html.</v>
       </c>
       <c r="E336" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="337">
@@ -6129,13 +6129,13 @@
         <v>Tear Trough Treatment</v>
       </c>
       <c r="C337" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D337" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tear-trough-treatment-in-delhi/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/tear-trough-treatment-in-delhi that this is the same hyaluronic-acid tear trough filler treatment already covered by the existing Under Eye Fillers brochure (which explicitly describes itself as "also known as tear trough fillers"). No new brochure built, this row is covered by under-eye-fillers-brochure.html (Injectable category).</v>
       </c>
       <c r="E337" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="338">
@@ -6877,13 +6877,13 @@
         <v>Hyperbaric Oxygen Therapy</v>
       </c>
       <c r="C381" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D381" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi that this describes the same pressurised-oxygen-chamber treatment already covered by the existing Hyperbaric Oxygen Chamber brochure (same mechanism, chamber types, and benefit list, just a city-specific page). No new brochure built, this row is covered by hyperbaric-oxygen-chamber-brochure.html (Drip Therapy category).</v>
       </c>
       <c r="E381" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="382">
@@ -6894,13 +6894,13 @@
         <v>Colon Hydrotherapy</v>
       </c>
       <c r="C382" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D382" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/colon-hydrotherapy-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/colon-hydrotherapy-in-delhi. Real treatment image found and used. Placed under Drip Therapy as closest fit (a wellness treatment, not a literal IV drip) -- flag if a dedicated category is preferred. Brochure: colon-hydrotherapy-brochure.html.</v>
       </c>
       <c r="E382" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="383">
@@ -6911,13 +6911,13 @@
         <v>Pink Himalayan Salt Infrared Sauna</v>
       </c>
       <c r="C383" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D383" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-himalayan-salt-infrared-sauna/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/pink-himalayan-salt-infrared-sauna. Real treatment banner image found and used. This fulfills the item flagged as "mentioned but not yet built" during the House of Sculpt brochure (batch 11). Placed under Drip Therapy as closest fit (same convention as Hyperbaric Oxygen Chamber) -- flag if a dedicated Wellness category is preferred. Brochure: pink-himalayan-salt-infrared-sauna-brochure.html.</v>
       </c>
       <c r="E383" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="384">

</xml_diff>

<commit_message>
Document "Your Treatment Journey" page rollout in brochure.xlsx
Logs which of the 122 treatment brochures got a new Journey page (80
files / 89 rows), which were intentionally skipped with a reason (12
files / 13 rows: 9 drips, Artiqa, Retix C, and the two bundle-programme
pages), and which already had equivalent content on the older, richer
template and needed no change (29 files / 36 rows).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,8 +402,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="100.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
@@ -454,7 +454,7 @@
         <v>Completed</v>
       </c>
       <c r="D3" t="str">
-        <v>Brochure already exists: DermaFrac (dermafrac-brochure.html) [exact]</v>
+        <v>Brochure already exists: DermaFrac (dermafrac-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E3" t="str">
         <v>2026-07-23</v>
@@ -471,7 +471,7 @@
         <v>Completed</v>
       </c>
       <c r="D4" t="str">
-        <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [exact]</v>
+        <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E4" t="str">
         <v>2026-06-26</v>
@@ -522,7 +522,7 @@
         <v>Completed</v>
       </c>
       <c r="D7" t="str">
-        <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/forma-skin-tightening-treatment-in-mumbai. Hero image only, no before/after. Placed under Anti Aging. Brochure: forma-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E7" t="str">
         <v>2026-07-24</v>
@@ -539,7 +539,7 @@
         <v>Completed</v>
       </c>
       <c r="D8" t="str">
-        <v>Brochure already exists: Morpheus 8 (morpheus-8-treatment-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Morpheus 8 (morpheus-8-treatment-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E8" t="str">
         <v>2026-06-26</v>
@@ -573,7 +573,7 @@
         <v>Completed</v>
       </c>
       <c r="D10" t="str">
-        <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 157 (Hair)]</v>
+        <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 157 (Hair)] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E10" t="str">
         <v>2026-06-26</v>
@@ -641,7 +641,7 @@
         <v>Completed</v>
       </c>
       <c r="D14" t="str">
-        <v>Brochure already exists: Artiqa (artiqa-brochure.html) [exact]</v>
+        <v>Brochure already exists: Artiqa (artiqa-brochure.html) [exact] JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment (pre-dates the sitemap cross-reference) -- no additional source to draw genuine new content from, so no Journey page added.</v>
       </c>
       <c r="E14" t="str">
         <v>2026-07-22</v>
@@ -658,7 +658,7 @@
         <v>Completed</v>
       </c>
       <c r="D15" t="str">
-        <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/coolsculpting. Note: same underlying cryolipolysis technology as the separate "Cryolipolysis" row/brochure, but kept as its own brochure since it is a distinct branded service on the booking menu. Placed under Body Contouring. Brochure: coolsculpting-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E15" t="str">
         <v>2026-07-24</v>
@@ -692,7 +692,7 @@
         <v>Completed</v>
       </c>
       <c r="D17" t="str">
-        <v>Brochure already exists: Emsculpt NEO (emsculpt-neo-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Emsculpt NEO (emsculpt-neo-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E17" t="str">
         <v>2026-06-26</v>
@@ -709,7 +709,7 @@
         <v>Completed</v>
       </c>
       <c r="D18" t="str">
-        <v>Brochure already exists: Exilis Elite (exilis-elite-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Exilis Elite (exilis-elite-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E18" t="str">
         <v>2026-06-26</v>
@@ -726,7 +726,7 @@
         <v>Completed</v>
       </c>
       <c r="D19" t="str">
-        <v>Scraped from isaacluxe.co/intragen-skin-tightening-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: intragen-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/intragen-skin-tightening-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: intragen-skin-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E19" t="str">
         <v>2026-07-25</v>
@@ -743,7 +743,7 @@
         <v>Completed</v>
       </c>
       <c r="D20" t="str">
-        <v>Brochure already exists: Lymphatic Drainage (lymphatic-drainage-brochure.html) [exact]</v>
+        <v>Brochure already exists: Lymphatic Drainage (lymphatic-drainage-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E20" t="str">
         <v>2026-06-26</v>
@@ -760,7 +760,7 @@
         <v>Completed</v>
       </c>
       <c r="D21" t="str">
-        <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/medcontour-treatment. Banner + diagram images only, not before/after. Placed under Body Contouring. Brochure: medcontour-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E21" t="str">
         <v>2026-07-25</v>
@@ -896,7 +896,7 @@
         <v>Completed</v>
       </c>
       <c r="D29" t="str">
-        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E29" t="str">
         <v>2026-07-25</v>
@@ -913,7 +913,7 @@
         <v>Completed</v>
       </c>
       <c r="D30" t="str">
-        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/x-wave. No before/after images on source page. Placed under Body Contouring. Brochure: x-wave-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E30" t="str">
         <v>2026-07-25</v>
@@ -998,7 +998,7 @@
         <v>Completed</v>
       </c>
       <c r="D35" t="str">
-        <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/derma-roller-treatment. No before/after images on source page. Placed under Facial. Brochure: dermaroller-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E35" t="str">
         <v>2026-07-25</v>
@@ -1015,7 +1015,7 @@
         <v>Completed</v>
       </c>
       <c r="D36" t="str">
-        <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Same underlying page/treatment as the "Mesotherapy" row -- covered by mesotherapy-brochure.html, no separate brochure built. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E36" t="str">
         <v>2026-07-24</v>
@@ -1202,7 +1202,7 @@
         <v>Completed</v>
       </c>
       <c r="D47" t="str">
-        <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/mesotherapy. Covers both skin and hair application; placed under Facial as closest fit. No before/after images on source page. Brochure: mesotherapy-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E47" t="str">
         <v>2026-07-24</v>
@@ -1219,7 +1219,7 @@
         <v>Completed</v>
       </c>
       <c r="D48" t="str">
-        <v>Brochure already exists: Microblading (microblading-brochure.html) [exact]</v>
+        <v>Brochure already exists: Microblading (microblading-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E48" t="str">
         <v>2026-06-26</v>
@@ -1270,7 +1270,7 @@
         <v>Completed</v>
       </c>
       <c r="D51" t="str">
-        <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/hyperbaric-oxygen-chamber. No before/after images on source page. General wellness/recovery treatment -- placed under Drip Therapy as closest fit (flag if a dedicated category is preferred). Brochure: hyperbaric-oxygen-chamber-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E51" t="str">
         <v>2026-07-25</v>
@@ -1355,7 +1355,7 @@
         <v>Completed</v>
       </c>
       <c r="D56" t="str">
-        <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/tattoo-removal. No before/after images on source page. Placed under "Facial" category on index.html as a closest fit -- flag if you want a dedicated category instead. Brochure: tattoo-removal-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E56" t="str">
         <v>2026-06-12</v>
@@ -1389,7 +1389,7 @@
         <v>Completed</v>
       </c>
       <c r="D58" t="str">
-        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added.</v>
+        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E58" t="str">
         <v>2026-07-15</v>
@@ -1406,7 +1406,7 @@
         <v>Completed</v>
       </c>
       <c r="D59" t="str">
-        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E59" t="str">
         <v>2026-07-15</v>
@@ -1457,7 +1457,7 @@
         <v>Completed</v>
       </c>
       <c r="D62" t="str">
-        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E62" t="str">
         <v>2026-07-15</v>
@@ -1525,7 +1525,7 @@
         <v>Completed</v>
       </c>
       <c r="D66" t="str">
-        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E66" t="str">
         <v>2026-07-15</v>
@@ -1593,7 +1593,7 @@
         <v>Completed</v>
       </c>
       <c r="D70" t="str">
-        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E70" t="str">
         <v>2026-07-15</v>
@@ -1610,7 +1610,7 @@
         <v>Completed</v>
       </c>
       <c r="D71" t="str">
-        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E71" t="str">
         <v>2026-07-15</v>
@@ -1661,7 +1661,7 @@
         <v>Completed</v>
       </c>
       <c r="D74" t="str">
-        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E74" t="str">
         <v>2026-07-15</v>
@@ -1950,7 +1950,7 @@
         <v>Completed</v>
       </c>
       <c r="D91" t="str">
-        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E91" t="str">
         <v>2026-07-15</v>
@@ -2018,7 +2018,7 @@
         <v>Completed</v>
       </c>
       <c r="D95" t="str">
-        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added.</v>
       </c>
       <c r="E95" t="str">
         <v>2026-07-15</v>
@@ -2035,7 +2035,7 @@
         <v>Completed</v>
       </c>
       <c r="D96" t="str">
-        <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/aptos-thread-lifting. No before/after images on source page. Placed under Face Lifting. Brochure: aptos-thread-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E96" t="str">
         <v>2026-07-24</v>
@@ -2052,7 +2052,7 @@
         <v>Completed</v>
       </c>
       <c r="D97" t="str">
-        <v>Brochure already exists: EmFace (emface-treatment-brochure.html) [exact]</v>
+        <v>Brochure already exists: EmFace (emface-treatment-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E97" t="str">
         <v>2026-06-26</v>
@@ -2069,7 +2069,7 @@
         <v>Completed</v>
       </c>
       <c r="D98" t="str">
-        <v>Existing brochure: Thread Lift (thread-lift-brochure.html). Missed in the original cross-reference due to naming difference ("Threads" vs "Thread Lift").</v>
+        <v>Existing brochure: Thread Lift (thread-lift-brochure.html). Missed in the original cross-reference due to naming difference ("Threads" vs "Thread Lift"). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E98" t="str">
         <v>2026-06-26</v>
@@ -2086,7 +2086,7 @@
         <v>Completed</v>
       </c>
       <c r="D99" t="str">
-        <v>Brochure already exists: Ultherapy (ultherapy-treatment-brochure.html) [exact]</v>
+        <v>Brochure already exists: Ultherapy (ultherapy-treatment-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E99" t="str">
         <v>2026-06-26</v>
@@ -2154,7 +2154,7 @@
         <v>Completed</v>
       </c>
       <c r="D103" t="str">
-        <v>Scraped from isaacluxe.co/biologique. No before/after images on source page. Placed under Facial. Brochure: biologique-recherche-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/biologique. No before/after images on source page. Placed under Facial. Brochure: biologique-recherche-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E103" t="str">
         <v>2026-07-25</v>
@@ -2188,7 +2188,7 @@
         <v>Completed</v>
       </c>
       <c r="D105" t="str">
-        <v>Brochure already exists: Carbon Facial (carbon-facial-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Carbon Facial (carbon-facial-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E105" t="str">
         <v>2026-06-26</v>
@@ -2256,7 +2256,7 @@
         <v>Completed</v>
       </c>
       <c r="D109" t="str">
-        <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/cryo-facial-in-mumbai. No before/after images on source page. Placed under Facial. Brochure: cryo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E109" t="str">
         <v>2026-07-25</v>
@@ -2290,7 +2290,7 @@
         <v>Completed</v>
       </c>
       <c r="D111" t="str">
-        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E111" t="str">
         <v>2026-07-25</v>
@@ -2324,7 +2324,7 @@
         <v>Completed</v>
       </c>
       <c r="D113" t="str">
-        <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/eye-light. No before/after images on source page. Brochure: eye-light-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E113" t="str">
         <v>2026-07-24</v>
@@ -2392,7 +2392,7 @@
         <v>Completed</v>
       </c>
       <c r="D117" t="str">
-        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E117" t="str">
         <v>2026-07-24</v>
@@ -2409,7 +2409,7 @@
         <v>Completed</v>
       </c>
       <c r="D118" t="str">
-        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/gg-glow. No before/after images on source page. Placed under Facial. Brochure: gg-glow-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E118" t="str">
         <v>2026-07-24</v>
@@ -2443,7 +2443,7 @@
         <v>Completed</v>
       </c>
       <c r="D120" t="str">
-        <v>Scraped from isaacluxe.co/ice-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: ice-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/ice-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: ice-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E120" t="str">
         <v>2026-07-25</v>
@@ -2477,7 +2477,7 @@
         <v>Completed</v>
       </c>
       <c r="D122" t="str">
-        <v>Brochure already exists: Laser Toning (laser-toning-brochure.html) [exact]</v>
+        <v>Brochure already exists: Laser Toning (laser-toning-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E122" t="str">
         <v>2026-06-26</v>
@@ -2494,7 +2494,7 @@
         <v>Completed</v>
       </c>
       <c r="D123" t="str">
-        <v>Scraped from isaacluxe.co/love-light-fusion-facial. No before/after images on source page. Placed under Facial. Brochure: love-light-fusion-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/love-light-fusion-facial. No before/after images on source page. Placed under Facial. Brochure: love-light-fusion-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E123" t="str">
         <v>2026-07-25</v>
@@ -2545,7 +2545,7 @@
         <v>Completed</v>
       </c>
       <c r="D126" t="str">
-        <v>Scraped from isaacluxe.co/oasis-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: oasis-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/oasis-facial-treatment. No before/after images on source page. Placed under Facial. Brochure: oasis-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E126" t="str">
         <v>2026-07-25</v>
@@ -2562,7 +2562,7 @@
         <v>Completed</v>
       </c>
       <c r="D127" t="str">
-        <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/obagi-facial. No before/after images on source page. Placed under Facial. Brochure: obagi-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E127" t="str">
         <v>2026-07-24</v>
@@ -2579,7 +2579,7 @@
         <v>Completed</v>
       </c>
       <c r="D128" t="str">
-        <v>Scraped from isaacluxe.co/oxygeneo-facial-best-oxygen-facial. No before/after images on source page. Placed under Facial. Brochure: oxygeneo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/oxygeneo-facial-best-oxygen-facial. No before/after images on source page. Placed under Facial. Brochure: oxygeneo-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E128" t="str">
         <v>2026-07-25</v>
@@ -2613,7 +2613,7 @@
         <v>Completed</v>
       </c>
       <c r="D130" t="str">
-        <v>Brochure already exists: Photo Facial (photo-facial-brochure.html) [exact]</v>
+        <v>Brochure already exists: Photo Facial (photo-facial-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E130" t="str">
         <v>2026-06-26</v>
@@ -2681,7 +2681,7 @@
         <v>Completed</v>
       </c>
       <c r="D134" t="str">
-        <v>Brochure already exists: Retix C (retix-c-brochure.html) [exact]</v>
+        <v>Brochure already exists: Retix C (retix-c-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure was originally built from retixc.com (manufacturer site), not an isaacluxe.co page -- no Journey page added in this pass, flag if you want it sourced from retixc.com.</v>
       </c>
       <c r="E134" t="str">
         <v>2026-07-16</v>
@@ -2698,7 +2698,7 @@
         <v>Completed</v>
       </c>
       <c r="D135" t="str">
-        <v>Scraped from isaacluxe.co/salmon-dna-pdrn-facial. Only banner/decorative images found, not before/after. Placed under Facial. Brochure: salmon-dna-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/salmon-dna-pdrn-facial. Only banner/decorative images found, not before/after. Placed under Facial. Brochure: salmon-dna-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E135" t="str">
         <v>2026-07-25</v>
@@ -2766,7 +2766,7 @@
         <v>Completed</v>
       </c>
       <c r="D139" t="str">
-        <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/snow-white-facial. No before/after images on source page. Brochure: snow-white-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E139" t="str">
         <v>2026-07-24</v>
@@ -2783,7 +2783,7 @@
         <v>Completed</v>
       </c>
       <c r="D140" t="str">
-        <v>Scraped from isaacluxe.co/v-bianco-skin-lightening-treatment. Real treatment banner image found and used. Placed under Facial. Brochure: v-bianco-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/v-bianco-skin-lightening-treatment. Real treatment banner image found and used. Placed under Facial. Brochure: v-bianco-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E140" t="str">
         <v>2026-07-25</v>
@@ -2800,7 +2800,7 @@
         <v>Completed</v>
       </c>
       <c r="D141" t="str">
-        <v>Scraped from isaacluxe.co/v-carbon-treatment (also called "Erase Treatment"). Note: conceptually adjacent to the existing Carbon Facial brochure, but a distinct mechanism -- V Carbon is a topical film/spray system (no laser), while Carbon Facial is laser-based -- kept separate, flag if you disagree. Source page images were generic/mismatched stock photos of facial masks, not clearly specific to this treatment -- none used. Placed under Facial. Brochure: v-carbon-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/v-carbon-treatment (also called "Erase Treatment"). Note: conceptually adjacent to the existing Carbon Facial brochure, but a distinct mechanism -- V Carbon is a topical film/spray system (no laser), while Carbon Facial is laser-based -- kept separate, flag if you disagree. Source page images were generic/mismatched stock photos of facial masks, not clearly specific to this treatment -- none used. Placed under Facial. Brochure: v-carbon-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E141" t="str">
         <v>2026-07-25</v>
@@ -2817,7 +2817,7 @@
         <v>Completed</v>
       </c>
       <c r="D142" t="str">
-        <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/valmont-facial. No before/after images on source page. Placed under Facial. Brochure: valmont-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E142" t="str">
         <v>2026-07-25</v>
@@ -2851,7 +2851,7 @@
         <v>Completed</v>
       </c>
       <c r="D144" t="str">
-        <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Dermapen 4 (dermapen-4-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E144" t="str">
         <v>2026-06-26</v>
@@ -2868,7 +2868,7 @@
         <v>Completed</v>
       </c>
       <c r="D145" t="str">
-        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/jet-peel-facial-or-dolphin-facial (titled "Jet Peel Facial" in the brochure). No before/after images on source page. Placed under Facial. Brochure: jet-peel-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E145" t="str">
         <v>2026-07-25</v>
@@ -2902,7 +2902,7 @@
         <v>Completed</v>
       </c>
       <c r="D147" t="str">
-        <v>Existing brochure: Exosome Scalp Treatment (exosome-scalp-treatment-brochure.html). Missed in the original cross-reference due to naming difference ("Exosome- Hair" vs "Exosome Scalp Treatment").</v>
+        <v>Existing brochure: Exosome Scalp Treatment (exosome-scalp-treatment-brochure.html). Missed in the original cross-reference due to naming difference ("Exosome- Hair" vs "Exosome Scalp Treatment"). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E147" t="str">
         <v>2026-06-26</v>
@@ -2987,7 +2987,7 @@
         <v>Completed</v>
       </c>
       <c r="D152" t="str">
-        <v>Existing brochure: QR678 Hair Science (QR678-hair-science-brochure.html). Missed in the original cross-reference due to word order ("Hair science- QR678" vs "QR678 Hair Science").</v>
+        <v>Existing brochure: QR678 Hair Science (QR678-hair-science-brochure.html). Missed in the original cross-reference due to word order ("Hair science- QR678" vs "QR678 Hair Science"). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E152" t="str">
         <v>2026-06-26</v>
@@ -3004,7 +3004,7 @@
         <v>Completed</v>
       </c>
       <c r="D153" t="str">
-        <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/hair-transplant. No before/after images on source page (only a placeholder image path). Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-transplant-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E153" t="str">
         <v>2026-07-24</v>
@@ -3038,7 +3038,7 @@
         <v>Completed</v>
       </c>
       <c r="D155" t="str">
-        <v>Brochure already exists: Luxe Keravive (keravive-brochure.html) [exact]</v>
+        <v>Brochure already exists: Luxe Keravive (keravive-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E155" t="str">
         <v>2026-06-26</v>
@@ -3072,7 +3072,7 @@
         <v>Completed</v>
       </c>
       <c r="D157" t="str">
-        <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 10 (Anti Aging)]</v>
+        <v>Brochure already exists: Pink Treatment (pink-treatment-brochure.html) [exact] [Duplicate name also appears at: row 10 (Anti Aging)] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E157" t="str">
         <v>2026-06-26</v>
@@ -3191,7 +3191,7 @@
         <v>Completed</v>
       </c>
       <c r="D164" t="str">
-        <v>Brochure already exists: HydraFacial MD Elite (hydrafacial-md-elite-brocher.html) [fuzzy]</v>
+        <v>Brochure already exists: HydraFacial MD Elite (hydrafacial-md-elite-brocher.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E164" t="str">
         <v>2026-06-26</v>
@@ -3378,7 +3378,7 @@
         <v>Completed</v>
       </c>
       <c r="D175" t="str">
-        <v>Brochure already exists: Botox (botox-treatment-brochure.html) [exact]</v>
+        <v>Brochure already exists: Botox (botox-treatment-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E175" t="str">
         <v>2026-06-26</v>
@@ -3463,7 +3463,7 @@
         <v>Completed</v>
       </c>
       <c r="D180" t="str">
-        <v>Previously "Missing - No Source" -- this is the same treatment as the "Kenacort Injection" row (reversed word order), which was built this session from isaacluxe.co/kenacort-injection. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Previously "Missing - No Source" -- this is the same treatment as the "Kenacort Injection" row (reversed word order), which was built this session from isaacluxe.co/kenacort-injection. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E180" t="str">
         <v>2026-07-25</v>
@@ -3548,7 +3548,7 @@
         <v>Completed</v>
       </c>
       <c r="D185" t="str">
-        <v>Brochure already exists: Polypeptide (polypeptide-brochure.html) [exact]</v>
+        <v>Brochure already exists: Polypeptide (polypeptide-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E185" t="str">
         <v>2026-06-26</v>
@@ -3582,7 +3582,7 @@
         <v>Completed</v>
       </c>
       <c r="D187" t="str">
-        <v>Brochure already exists: Profhilo (profhilo-brochure.html) [exact]</v>
+        <v>Brochure already exists: Profhilo (profhilo-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E187" t="str">
         <v>2026-06-26</v>
@@ -3599,7 +3599,7 @@
         <v>Completed</v>
       </c>
       <c r="D188" t="str">
-        <v>Brochure already exists: Rejuran (rejuran-brochure.html) [exact]</v>
+        <v>Brochure already exists: Rejuran (rejuran-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E188" t="str">
         <v>2026-06-26</v>
@@ -3616,7 +3616,7 @@
         <v>Completed</v>
       </c>
       <c r="D189" t="str">
-        <v>Brochure already exists: Rejuran (rejuran-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: Rejuran (rejuran-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E189" t="str">
         <v>2026-06-26</v>
@@ -3633,7 +3633,7 @@
         <v>Completed</v>
       </c>
       <c r="D190" t="str">
-        <v>Brochure already exists: Restylane (restylane-brochure.html) [exact]</v>
+        <v>Brochure already exists: Restylane (restylane-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E190" t="str">
         <v>2026-07-23</v>
@@ -3667,7 +3667,7 @@
         <v>Completed</v>
       </c>
       <c r="D192" t="str">
-        <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/skinfill-bacio-lip-booster. Only 1 hero image found, not a before/after pair -- not used. Placed under Injectable. Brochure: skinfill-lip-booster-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E192" t="str">
         <v>2026-07-24</v>
@@ -3752,7 +3752,7 @@
         <v>Completed</v>
       </c>
       <c r="D197" t="str">
-        <v>Built from bioretherapy.pdf (BioRePeelCl3 FND + Body variants, real before/after photos). Brochure: biorepeel-brochure.html.</v>
+        <v>Built from bioretherapy.pdf (BioRePeelCl3 FND + Body variants, real before/after photos). Brochure: biorepeel-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E197" t="str">
         <v>2026-07-24</v>
@@ -3803,7 +3803,7 @@
         <v>Completed</v>
       </c>
       <c r="D200" t="str">
-        <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/cosmelan-peel-treatment. No before/after images on source page. Placed under Peel. Brochure: cosmelan-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E200" t="str">
         <v>2026-07-24</v>
@@ -3922,7 +3922,7 @@
         <v>Completed</v>
       </c>
       <c r="D207" t="str">
-        <v>Brochure already exists: House of Peels (house-of-peels-brochure.html) [fuzzy]</v>
+        <v>Brochure already exists: House of Peels (house-of-peels-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E207" t="str">
         <v>2026-06-26</v>
@@ -4007,7 +4007,7 @@
         <v>Completed</v>
       </c>
       <c r="D212" t="str">
-        <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/yellow-peel-treatment-in-mumbai. No before/after images existed on the source page. Brochure: yellow-peel-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E212" t="str">
         <v>2026-07-24</v>
@@ -5265,7 +5265,7 @@
         <v>Completed</v>
       </c>
       <c r="D286" t="str">
-        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/gynaecomastia. No before/after images on source page. Placed under Body Contouring. Brochure: gynaecomastia-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E286" t="str">
         <v>2026-07-24</v>
@@ -5282,7 +5282,7 @@
         <v>Completed</v>
       </c>
       <c r="D287" t="str">
-        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/liposuction-surgery. No before/after images on source page. Placed under Body Contouring. Brochure: liposuction-surgery-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E287" t="str">
         <v>2026-07-24</v>
@@ -5299,7 +5299,7 @@
         <v>Completed</v>
       </c>
       <c r="D288" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/non-surgical-breast-lift. Source had a banner + section image, not a before/after pair -- none used. Placed under Body Contouring. Brochure: non-surgical-breast-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E288" t="str">
         <v>2026-07-24</v>
@@ -5316,7 +5316,7 @@
         <v>Completed</v>
       </c>
       <c r="D289" t="str">
-        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/cryolipolysis-treatment. Source images were generic device-in-use hero shots, not before/after -- none used. Placed under Body Contouring. Brochure: cryolipolysis-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E289" t="str">
         <v>2026-07-24</v>
@@ -5333,7 +5333,7 @@
         <v>Completed</v>
       </c>
       <c r="D290" t="str">
-        <v>Scraped from isaacluxe.co/instasculpt. No before/after images on source page. Placed under Body Contouring. Brochure: instasculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/instasculpt. No before/after images on source page. Placed under Body Contouring. Brochure: instasculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E290" t="str">
         <v>2026-07-25</v>
@@ -5350,7 +5350,7 @@
         <v>Completed</v>
       </c>
       <c r="D291" t="str">
-        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Structure cards already on the Treatment page, so no Journey page was added to avoid redundancy.</v>
       </c>
       <c r="E291" t="str">
         <v>2026-07-25</v>
@@ -5367,7 +5367,7 @@
         <v>Completed</v>
       </c>
       <c r="D292" t="str">
-        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Goals cards already on the Treatment page, so no Journey page was added to avoid redundancy.</v>
       </c>
       <c r="E292" t="str">
         <v>2026-07-25</v>
@@ -5384,7 +5384,7 @@
         <v>Completed</v>
       </c>
       <c r="D293" t="str">
-        <v>Scraped from isaacluxe.co/tummy-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: tummy-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/tummy-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: tummy-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E293" t="str">
         <v>2026-07-25</v>
@@ -5401,7 +5401,7 @@
         <v>Completed</v>
       </c>
       <c r="D294" t="str">
-        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E294" t="str">
         <v>2026-07-25</v>
@@ -5418,7 +5418,7 @@
         <v>Completed</v>
       </c>
       <c r="D295" t="str">
-        <v>Scraped from isaacluxe.co/ballancer-pro-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: ballancer-pro-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/ballancer-pro-treatment. No before/after images on source page. Placed under Body Contouring. Brochure: ballancer-pro-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E295" t="str">
         <v>2026-07-25</v>
@@ -5435,7 +5435,7 @@
         <v>Completed</v>
       </c>
       <c r="D296" t="str">
-        <v>Scraped from isaacluxe.co/femme-360-vaginal-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: femme-360-vaginal-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/femme-360-vaginal-tightening. No before/after images on source page. Placed under Body Contouring. Brochure: femme-360-vaginal-tightening-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E296" t="str">
         <v>2026-07-25</v>
@@ -5452,7 +5452,7 @@
         <v>Completed</v>
       </c>
       <c r="D297" t="str">
-        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/vaginal-fillers (content titled "Vaginal Tightening" on the page itself, HA filler mechanism). No before/after images. Placed under Body Contouring. Brochure: vaginal-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E297" t="str">
         <v>2026-07-24</v>
@@ -5469,7 +5469,7 @@
         <v>Completed</v>
       </c>
       <c r="D298" t="str">
-        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E298" t="str">
         <v>2026-07-25</v>
@@ -5486,7 +5486,7 @@
         <v>Completed</v>
       </c>
       <c r="D299" t="str">
-        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E299" t="str">
         <v>2026-07-25</v>
@@ -5520,7 +5520,7 @@
         <v>Completed</v>
       </c>
       <c r="D301" t="str">
-        <v>Scraped from isaacluxe.co/sculptone-plus. No before/after images on source page; source page also gave no explicit session count/frequency. Note: conceptually similar in goal (fat reduction + muscle building) to the existing Emsculpt NEO brochure. Placed under Body Contouring. Brochure: sculpt-tone-plus-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/sculptone-plus. No before/after images on source page; source page also gave no explicit session count/frequency. Note: conceptually similar in goal (fat reduction + muscle building) to the existing Emsculpt NEO brochure. Placed under Body Contouring. Brochure: sculpt-tone-plus-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E301" t="str">
         <v>2026-07-25</v>
@@ -5537,7 +5537,7 @@
         <v>Completed</v>
       </c>
       <c r="D302" t="str">
-        <v>Scraped from isaacluxe.co/cool-tech. One banner image found, not a before/after pair. Note: this is a cooling/cryolipolysis-based fat-freezing technology, likely the same core mechanism as the existing Cryolipolysis and CoolSculpting brochures (three separate branded fat-freezing entries now) -- kept as its own distinct catalog item per its own sitemap page, flag if you would like these consolidated or cross-referenced. Placed under Body Contouring. Brochure: cool-tech-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/cool-tech. One banner image found, not a before/after pair. Note: this is a cooling/cryolipolysis-based fat-freezing technology, likely the same core mechanism as the existing Cryolipolysis and CoolSculpting brochures (three separate branded fat-freezing entries now) -- kept as its own distinct catalog item per its own sitemap page, flag if you would like these consolidated or cross-referenced. Placed under Body Contouring. Brochure: cool-tech-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E302" t="str">
         <v>2026-07-25</v>
@@ -5554,7 +5554,7 @@
         <v>Completed</v>
       </c>
       <c r="D303" t="str">
-        <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting).</v>
+        <v>Confirmed via isaacluxe.co/ulthera-face-lifting that Ulthera and Ultherapy are the same treatment -- no new brochure built, this is covered by the existing ultherapy-treatment-brochure.html (Face Lifting). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E303" t="str">
         <v>2026-06-26</v>
@@ -5571,7 +5571,7 @@
         <v>Completed</v>
       </c>
       <c r="D304" t="str">
-        <v>Scraped from isaacluxe.co/thread-face-lift-treatment. Note: conceptually overlaps with the existing "Thread Lift" and "Aptos Thread Lift" brochures (all use PDO/PLLA-style threads), but is its own distinct catalog line item, so built separately -- flag if you want these consolidated. No before/after photos (only hero images). Placed under Face Lifting. Brochure: thread-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/thread-face-lift-treatment. Note: conceptually overlaps with the existing "Thread Lift" and "Aptos Thread Lift" brochures (all use PDO/PLLA-style threads), but is its own distinct catalog line item, so built separately -- flag if you want these consolidated. No before/after photos (only hero images). Placed under Face Lifting. Brochure: thread-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E304" t="str">
         <v>2026-07-25</v>
@@ -5588,7 +5588,7 @@
         <v>Completed</v>
       </c>
       <c r="D305" t="str">
-        <v>Scraped from isaacluxe.co/liquid-facelift-treatment. No before/after images on source page. Placed under Face Lifting. Brochure: liquid-facelift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/liquid-facelift-treatment. No before/after images on source page. Placed under Face Lifting. Brochure: liquid-facelift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E305" t="str">
         <v>2026-07-25</v>
@@ -5605,7 +5605,7 @@
         <v>Completed</v>
       </c>
       <c r="D306" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/non-surgical-face-lift. Used 1 hero image URL found but not a before/after pair, so no photos added. Placed under Face Lifting. Brochure: non-surgical-face-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E306" t="str">
         <v>2026-07-24</v>
@@ -5622,7 +5622,7 @@
         <v>Completed</v>
       </c>
       <c r="D307" t="str">
-        <v>Scraped from isaacluxe.co/sygma-lift-treatment-in-gurgaon. No before/after images on source page. Placed under Face Lifting. Brochure: sygma-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/sygma-lift-treatment-in-gurgaon. No before/after images on source page. Placed under Face Lifting. Brochure: sygma-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E307" t="str">
         <v>2026-07-25</v>
@@ -5639,7 +5639,7 @@
         <v>Completed</v>
       </c>
       <c r="D308" t="str">
-        <v>Scraped from isaacluxe.co/4-d-lift. No before/after images on source page. Placed under Face Lifting. Brochure: 4d-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/4-d-lift. No before/after images on source page. Placed under Face Lifting. Brochure: 4d-lift-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E308" t="str">
         <v>2026-07-25</v>
@@ -5656,7 +5656,7 @@
         <v>Completed</v>
       </c>
       <c r="D309" t="str">
-        <v>Scraped from isaacluxe.co/face-lift-filler-in-delhi. No before/after images on source page. Placed under Face Lifting. Brochure: face-lift-filler-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/face-lift-filler-in-delhi. No before/after images on source page. Placed under Face Lifting. Brochure: face-lift-filler-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E309" t="str">
         <v>2026-07-25</v>
@@ -5673,7 +5673,7 @@
         <v>Completed</v>
       </c>
       <c r="D310" t="str">
-        <v>Scraped from isaacluxe.co/square-jaw-treatment-in-delhi. Source images were generic treatment photos, not before/after -- none used. Note: this is a surgical jawline-implant procedure (general anesthesia), distinct in mechanism from the mostly non-surgical treatments elsewhere in Face Lifting -- kept in Face Lifting per its category match. Brochure: square-jaw-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/square-jaw-treatment-in-delhi. Source images were generic treatment photos, not before/after -- none used. Note: this is a surgical jawline-implant procedure (general anesthesia), distinct in mechanism from the mostly non-surgical treatments elsewhere in Face Lifting -- kept in Face Lifting per its category match. Brochure: square-jaw-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E310" t="str">
         <v>2026-07-25</v>
@@ -5690,7 +5690,7 @@
         <v>Completed</v>
       </c>
       <c r="D311" t="str">
-        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E311" t="str">
         <v>2026-07-25</v>
@@ -5707,7 +5707,7 @@
         <v>Completed</v>
       </c>
       <c r="D312" t="str">
-        <v>Confirmed via isaacluxe.co/br-facial that "BR Facial" is the same Biologique Recherche treatment (same brand, same Lotion P50 cleanser/mechanism) as the existing biologique-recherche-facial-brochure.html -- no new brochure built, this row is covered by that existing file (Facial category). Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Confirmed via isaacluxe.co/br-facial that "BR Facial" is the same Biologique Recherche treatment (same brand, same Lotion P50 cleanser/mechanism) as the existing biologique-recherche-facial-brochure.html -- no new brochure built, this row is covered by that existing file (Facial category). Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E312" t="str">
         <v>2026-07-25</v>
@@ -5724,7 +5724,7 @@
         <v>Completed</v>
       </c>
       <c r="D313" t="str">
-        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E313" t="str">
         <v>2026-07-25</v>
@@ -5775,7 +5775,7 @@
         <v>Completed</v>
       </c>
       <c r="D316" t="str">
-        <v>Scraped from isaacluxe.co/meso-glow. Real treatment image found and used. Note: conceptually overlaps with the existing Mesotherapy brochure (both are micro-injected vitamin/nutrient infusions), but MesoGlow is its own named protocol with a distinct ingredient profile (HA/vitamin C/E) and timeline -- kept separate, flag if you want these consolidated. Placed under Facial. Brochure: meso-glow-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/meso-glow. Real treatment image found and used. Note: conceptually overlaps with the existing Mesotherapy brochure (both are micro-injected vitamin/nutrient infusions), but MesoGlow is its own named protocol with a distinct ingredient profile (HA/vitamin C/E) and timeline -- kept separate, flag if you want these consolidated. Placed under Facial. Brochure: meso-glow-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E316" t="str">
         <v>2026-07-25</v>
@@ -5843,7 +5843,7 @@
         <v>Completed</v>
       </c>
       <c r="D320" t="str">
-        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/vampire-facial. No before/after images on source page. Placed under Facial. Brochure: vampire-facial-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E320" t="str">
         <v>2026-07-25</v>
@@ -5860,7 +5860,7 @@
         <v>Completed</v>
       </c>
       <c r="D321" t="str">
-        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html. PHOTO CHECK: source page's only non-logo image was mislabeled/mismatched (a photo captioned "Ultherapy" appearing on the Dermabrasion page) -- not used to avoid misrepresenting the treatment. No photo added.</v>
+        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html. PHOTO CHECK: source page's only non-logo image was mislabeled/mismatched (a photo captioned "Ultherapy" appearing on the Dermabrasion page) -- not used to avoid misrepresenting the treatment. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E321" t="str">
         <v>2026-07-25</v>
@@ -5877,7 +5877,7 @@
         <v>Completed</v>
       </c>
       <c r="D322" t="str">
-        <v>Scraped from isaacluxe.co/microdermabrasion-treatment. Real before/after composite image found and used. Placed under Facial. Brochure: microdermabrasion-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/microdermabrasion-treatment. Real before/after composite image found and used. Placed under Facial. Brochure: microdermabrasion-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E322" t="str">
         <v>2026-07-25</v>
@@ -5894,7 +5894,7 @@
         <v>Completed</v>
       </c>
       <c r="D323" t="str">
-        <v>Scraped from isaacluxe.co/skin-polishing (a body-wide treatment; titled "Body Polishing" in the brochure). No before/after images on source page. Placed under Facial as closest fit. Brochure: skin-polishing-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/skin-polishing (a body-wide treatment; titled "Body Polishing" in the brochure). No before/after images on source page. Placed under Facial as closest fit. Brochure: skin-polishing-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E323" t="str">
         <v>2026-07-25</v>
@@ -5911,7 +5911,7 @@
         <v>Completed</v>
       </c>
       <c r="D324" t="str">
-        <v>Scraped from isaacluxe.co/dermamelan-treatment. Only a process-diagram image found, not before/after. Placed under Facial. Brochure: dermamelan-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/dermamelan-treatment. Only a process-diagram image found, not before/after. Placed under Facial. Brochure: dermamelan-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E324" t="str">
         <v>2026-07-25</v>
@@ -6013,7 +6013,7 @@
         <v>Completed</v>
       </c>
       <c r="D330" t="str">
-        <v>Scraped from isaacluxe.co/acne-treatment-in-bangalore. Hero/treatment photos only, not before/after. Placed under Facial. Brochure: acne-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/acne-treatment-in-bangalore. Hero/treatment photos only, not before/after. Placed under Facial. Brochure: acne-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E330" t="str">
         <v>2026-07-25</v>
@@ -6030,7 +6030,7 @@
         <v>Completed</v>
       </c>
       <c r="D331" t="str">
-        <v>Scraped from isaacluxe.co/acne-scar-treatment-in-gurgaon. Stock portrait photos only, not before/after. Placed under Facial. Brochure: acne-scar-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/acne-scar-treatment-in-gurgaon. Stock portrait photos only, not before/after. Placed under Facial. Brochure: acne-scar-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E331" t="str">
         <v>2026-07-25</v>
@@ -6115,7 +6115,7 @@
         <v>Completed</v>
       </c>
       <c r="D336" t="str">
-        <v>Scraped from isaacluxe.co/dark-circles. This is a condition/menu page listing multiple approaches (fillers, Eye Light, peels, laser) similar in structure to the Melasma/Rosacea/Square Jaw pattern -- two of its named modalities (Eye Light, Under Eye/Tear Trough Fillers) already have their own dedicated brochures, referenced here as part of the combined protocol rather than duplicated. No images found on the source page. Placed under Facial. Brochure: dark-circles-treatment-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/dark-circles. This is a condition/menu page listing multiple approaches (fillers, Eye Light, peels, laser) similar in structure to the Melasma/Rosacea/Square Jaw pattern -- two of its named modalities (Eye Light, Under Eye/Tear Trough Fillers) already have their own dedicated brochures, referenced here as part of the combined protocol rather than duplicated. No images found on the source page. Placed under Facial. Brochure: dark-circles-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E336" t="str">
         <v>2026-07-25</v>
@@ -6132,7 +6132,7 @@
         <v>Completed</v>
       </c>
       <c r="D337" t="str">
-        <v>Confirmed via isaacluxe.co/tear-trough-treatment-in-delhi that this is the same hyaluronic-acid tear trough filler treatment already covered by the existing Under Eye Fillers brochure (which explicitly describes itself as "also known as tear trough fillers"). No new brochure built, this row is covered by under-eye-fillers-brochure.html (Injectable category).</v>
+        <v>Confirmed via isaacluxe.co/tear-trough-treatment-in-delhi that this is the same hyaluronic-acid tear trough filler treatment already covered by the existing Under Eye Fillers brochure (which explicitly describes itself as "also known as tear trough fillers"). No new brochure built, this row is covered by under-eye-fillers-brochure.html (Injectable category). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E337" t="str">
         <v>2026-07-25</v>
@@ -6149,7 +6149,7 @@
         <v>Completed</v>
       </c>
       <c r="D338" t="str">
-        <v>Scraped from isaacluxe.co/under-eye-fillers-treatment. No before/after images on source page. Placed under Injectable. Brochure: under-eye-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/under-eye-fillers-treatment. No before/after images on source page. Placed under Injectable. Brochure: under-eye-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E338" t="str">
         <v>2026-07-25</v>
@@ -6166,7 +6166,7 @@
         <v>Completed</v>
       </c>
       <c r="D339" t="str">
-        <v>Scraped from isaacluxe.co/melasma. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: melasma-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/melasma. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: melasma-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E339" t="str">
         <v>2026-07-25</v>
@@ -6183,7 +6183,7 @@
         <v>Completed</v>
       </c>
       <c r="D340" t="str">
-        <v>Scraped from isaacluxe.co/rosacea. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: rosacea-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/rosacea. Source had a banner image and a single treatment image, not a before/after pair -- none used. Placed under Facial. Brochure: rosacea-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E340" t="str">
         <v>2026-07-25</v>
@@ -6217,7 +6217,7 @@
         <v>Completed</v>
       </c>
       <c r="D342" t="str">
-        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E342" t="str">
         <v>2026-07-25</v>
@@ -6285,7 +6285,7 @@
         <v>Completed</v>
       </c>
       <c r="D346" t="str">
-        <v>Scraped from isaacluxe.co/stretch-marks. Source had a banner image and one treatment image, not a before/after pair -- none used. Note: conceptually overlaps with the existing Derma Roller brochure, which lists stretch marks as one of its uses, but this dedicated page covers the fuller multi-modality approach (laser, MNRF, PRP/exosomes, peels) -- kept separate per its own sitemap URL/Excel row, flag if you want these consolidated. Placed under Facial. Brochure: stretch-marks-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/stretch-marks. Source had a banner image and one treatment image, not a before/after pair -- none used. Note: conceptually overlaps with the existing Derma Roller brochure, which lists stretch marks as one of its uses, but this dedicated page covers the fuller multi-modality approach (laser, MNRF, PRP/exosomes, peels) -- kept separate per its own sitemap URL/Excel row, flag if you want these consolidated. Placed under Facial. Brochure: stretch-marks-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E346" t="str">
         <v>2026-07-25</v>
@@ -6438,7 +6438,7 @@
         <v>Completed</v>
       </c>
       <c r="D355" t="str">
-        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/lip-fillers. No before/after images on source page. Placed under Injectable. Brochure: lip-fillers-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E355" t="str">
         <v>2026-07-24</v>
@@ -6472,7 +6472,7 @@
         <v>Completed</v>
       </c>
       <c r="D357" t="str">
-        <v>Scraped from isaacluxe.co/fat-lipolysis-injection. No before/after images on source page. Placed under Injectable. Brochure: fat-lipolysis-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/fat-lipolysis-injection. No before/after images on source page. Placed under Injectable. Brochure: fat-lipolysis-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E357" t="str">
         <v>2026-07-25</v>
@@ -6489,7 +6489,7 @@
         <v>Completed</v>
       </c>
       <c r="D358" t="str">
-        <v>Scraped from isaacluxe.co/kenacort-injection. No before/after images on source page. Placed under Injectable. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/kenacort-injection. No before/after images on source page. Placed under Injectable. Brochure: kenacort-injection-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E358" t="str">
         <v>2026-07-25</v>
@@ -6523,7 +6523,7 @@
         <v>Completed</v>
       </c>
       <c r="D360" t="str">
-        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E360" t="str">
         <v>2026-07-25</v>
@@ -6557,7 +6557,7 @@
         <v>Completed</v>
       </c>
       <c r="D362" t="str">
-        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E362" t="str">
         <v>2026-07-25</v>
@@ -6591,7 +6591,7 @@
         <v>Completed</v>
       </c>
       <c r="D364" t="str">
-        <v>Scraped from isaacluxe.co/calecim-professional-brand. One product image found, not before/after. Placed under Injectable. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/calecim-professional-brand. One product image found, not before/after. Placed under Injectable. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E364" t="str">
         <v>2026-07-25</v>
@@ -6608,7 +6608,7 @@
         <v>Completed</v>
       </c>
       <c r="D365" t="str">
-        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html. PHOTO CHECK: source page has only the generic site logo and footer photo, no treatment-specific image. No photo added.</v>
+        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html. PHOTO CHECK: source page has only the generic site logo and footer photo, no treatment-specific image. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E365" t="str">
         <v>2026-07-24</v>
@@ -6625,7 +6625,7 @@
         <v>Completed</v>
       </c>
       <c r="D366" t="str">
-        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/regenera-activa-hair-treatment. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: regenera-activa-hair-treatment-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E366" t="str">
         <v>2026-07-24</v>
@@ -6642,7 +6642,7 @@
         <v>Completed</v>
       </c>
       <c r="D367" t="str">
-        <v>Scraped from isaacluxe.co/non-surgical-hair-replacement. One product image found, not before/after. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: non-surgical-hair-replacement-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Scraped from isaacluxe.co/non-surgical-hair-replacement. One product image found, not before/after. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: non-surgical-hair-replacement-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E367" t="str">
         <v>2026-07-25</v>
@@ -6659,7 +6659,7 @@
         <v>Completed</v>
       </c>
       <c r="D368" t="str">
-        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E368" t="str">
         <v>2026-07-25</v>
@@ -6676,7 +6676,7 @@
         <v>Completed</v>
       </c>
       <c r="D369" t="str">
-        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E369" t="str">
         <v>2026-07-25</v>
@@ -6761,7 +6761,7 @@
         <v>Completed</v>
       </c>
       <c r="D374" t="str">
-        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added.</v>
+        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E374" t="str">
         <v>2026-07-25</v>
@@ -6778,7 +6778,7 @@
         <v>Completed</v>
       </c>
       <c r="D375" t="str">
-        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category).</v>
+        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E375" t="str">
         <v>2026-06-26</v>
@@ -6812,7 +6812,7 @@
         <v>Completed</v>
       </c>
       <c r="D377" t="str">
-        <v>Confirmed via isaacluxe.co/soprano-ice-platinum that this Alma Soprano ICE Platinum device uses the same triple-wavelength (755nm Alexandrite / 810nm Diode / 1064nm Nd:YAG) technology already documented in the existing laser-hair-reduction-brochure.html (built around Soprano Titanium). Per user decision, treated as the same core device -- no new brochure built, this row is covered by the existing Laser Hair Reduction brochure.</v>
+        <v>Confirmed via isaacluxe.co/soprano-ice-platinum that this Alma Soprano ICE Platinum device uses the same triple-wavelength (755nm Alexandrite / 810nm Diode / 1064nm Nd:YAG) technology already documented in the existing laser-hair-reduction-brochure.html (built around Soprano Titanium). Per user decision, treated as the same core device -- no new brochure built, this row is covered by the existing Laser Hair Reduction brochure. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E377" t="str">
         <v>2026-06-27</v>
@@ -6829,7 +6829,7 @@
         <v>Completed</v>
       </c>
       <c r="D378" t="str">
-        <v>Confirmed via isaacluxe.co/soprano-ice-titanium that this device has essentially identical specs (same 3 wavelengths, ICE cooling, ~30-min sessions) to the existing laser-hair-reduction-brochure.html, which is already built around Soprano Titanium. No new brochure built, this row is covered by the existing Laser Hair Reduction brochure.</v>
+        <v>Confirmed via isaacluxe.co/soprano-ice-titanium that this device has essentially identical specs (same 3 wavelengths, ICE cooling, ~30-min sessions) to the existing laser-hair-reduction-brochure.html, which is already built around Soprano Titanium. No new brochure built, this row is covered by the existing Laser Hair Reduction brochure. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E378" t="str">
         <v>2026-06-27</v>
@@ -6880,7 +6880,7 @@
         <v>Completed</v>
       </c>
       <c r="D381" t="str">
-        <v>Confirmed via isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi that this describes the same pressurised-oxygen-chamber treatment already covered by the existing Hyperbaric Oxygen Chamber brochure (same mechanism, chamber types, and benefit list, just a city-specific page). No new brochure built, this row is covered by hyperbaric-oxygen-chamber-brochure.html (Drip Therapy category).</v>
+        <v>Confirmed via isaacluxe.co/hyperbaric-oxygen-therapy-in-delhi that this describes the same pressurised-oxygen-chamber treatment already covered by the existing Hyperbaric Oxygen Chamber brochure (same mechanism, chamber types, and benefit list, just a city-specific page). No new brochure built, this row is covered by hyperbaric-oxygen-chamber-brochure.html (Drip Therapy category). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E381" t="str">
         <v>2026-07-25</v>
@@ -6897,7 +6897,7 @@
         <v>Completed</v>
       </c>
       <c r="D382" t="str">
-        <v>Scraped from isaacluxe.co/colon-hydrotherapy-in-delhi. Real treatment image found and used. Placed under Drip Therapy as closest fit (a wellness treatment, not a literal IV drip) -- flag if a dedicated category is preferred. Brochure: colon-hydrotherapy-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/colon-hydrotherapy-in-delhi. Real treatment image found and used. Placed under Drip Therapy as closest fit (a wellness treatment, not a literal IV drip) -- flag if a dedicated category is preferred. Brochure: colon-hydrotherapy-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E382" t="str">
         <v>2026-07-25</v>
@@ -6914,7 +6914,7 @@
         <v>Completed</v>
       </c>
       <c r="D383" t="str">
-        <v>Scraped from isaacluxe.co/pink-himalayan-salt-infrared-sauna. Real treatment banner image found and used. This fulfills the item flagged as "mentioned but not yet built" during the House of Sculpt brochure (batch 11). Placed under Drip Therapy as closest fit (same convention as Hyperbaric Oxygen Chamber) -- flag if a dedicated Wellness category is preferred. Brochure: pink-himalayan-salt-infrared-sauna-brochure.html.</v>
+        <v>Scraped from isaacluxe.co/pink-himalayan-salt-infrared-sauna. Real treatment banner image found and used. This fulfills the item flagged as "mentioned but not yet built" during the House of Sculpt brochure (batch 11). Placed under Drip Therapy as closest fit (same convention as Hyperbaric Oxygen Chamber) -- flag if a dedicated Wellness category is preferred. Brochure: pink-himalayan-salt-infrared-sauna-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E383" t="str">
         <v>2026-07-25</v>
@@ -6999,7 +6999,7 @@
         <v>Completed</v>
       </c>
       <c r="D388" t="str">
-        <v>Source URL isaacluxe.co/calecim-product/ returns an HTTP 301 redirect, landing on the same content already scraped as "Calecim Professional Brand". Same product, old URL slug. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25).</v>
+        <v>Source URL isaacluxe.co/calecim-product/ returns an HTTP 301 redirect, landing on the same content already scraped as "Calecim Professional Brand". Same product, old URL slug. Brochure: calecim-professional-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
       </c>
       <c r="E388" t="str">
         <v>2026-07-25</v>
@@ -7067,7 +7067,7 @@
         <v>Completed</v>
       </c>
       <c r="D392" t="str">
-        <v>Category-level umbrella brochure covering the full drip menu, not an individual treatment line item -- no row existed in the original 285-row export. Brochure: house-of-drips-brochure.html.</v>
+        <v>Category-level umbrella brochure covering the full drip menu, not an individual treatment line item -- no row existed in the original 285-row export. Brochure: house-of-drips-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E392" t="str">
         <v>2026-06-26</v>
@@ -7084,7 +7084,7 @@
         <v>Completed</v>
       </c>
       <c r="D393" t="str">
-        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html. PHOTO CHECK: no corresponding live isaacluxe.co page exists for Qlara (confirmed via sitemap search) -- no compliant photo source available. No photo added.</v>
+        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html. PHOTO CHECK: no corresponding live isaacluxe.co page exists for Qlara (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E393" t="str">
         <v>2026-07-16</v>
@@ -7101,7 +7101,7 @@
         <v>Completed</v>
       </c>
       <c r="D394" t="str">
-        <v>Existing brochure covering dermal fillers generally (closest Excel row was "Juvederm-Filler", a specific brand, not a match) -- no row existed for the generic treatment. Brochure: dermal-fillers-brochure.html.</v>
+        <v>Existing brochure covering dermal fillers generally (closest Excel row was "Juvederm-Filler", a specific brand, not a match) -- no row existed for the generic treatment. Brochure: dermal-fillers-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E394" t="str">
         <v>2026-06-26</v>
@@ -7118,7 +7118,7 @@
         <v>Completed</v>
       </c>
       <c r="D395" t="str">
-        <v>Existing brochure covering laser hair reduction generally -- the Excel only had specific device variants (Soprano Platinum/Titanium, Triton), no generic row. Brochure: laser-hair-reduction-brochure.html.</v>
+        <v>Existing brochure covering laser hair reduction generally -- the Excel only had specific device variants (Soprano Platinum/Titanium, Triton), no generic row. Brochure: laser-hair-reduction-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
       </c>
       <c r="E395" t="str">
         <v>2026-06-27</v>

</xml_diff>

<commit_message>
Mark batch 15 brochures Completed in brochure.xlsx; merge Removal and IV Drip Therapy into existing brochures
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -402,8 +402,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="100.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
@@ -1301,13 +1301,13 @@
         <v>Removal</v>
       </c>
       <c r="C53" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D53" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/get-hair-free-smooth-skin-with-laser-hair-removal-technology/ [fuzzy]. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/get-hair-free-smooth-skin-with-laser-hair-removal-technology that this page explicitly names "Soprano Titanium" (patient testimonial) as its laser hair removal device -- the same technology already covered by the existing Laser Hair Reduction brochure. No new brochure built, this row is covered by laser-hair-reduction-brochure.html (Laser Hair Reduction category).</v>
       </c>
       <c r="E53" t="str">
-        <v/>
+        <v>2026-06-27</v>
       </c>
     </row>
     <row r="54">
@@ -5738,13 +5738,13 @@
         <v>O2Derm Facial</v>
       </c>
       <c r="C314" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D314" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/o2derm-facial/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/o2derm-facial. Real hero banner image found and used. Placed under Facial. Brochure: o2derm-facial-brochure.html.</v>
       </c>
       <c r="E314" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="315">
@@ -5755,13 +5755,13 @@
         <v>Exo Glow Treatment</v>
       </c>
       <c r="C315" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D315" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/exo-glow-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/exo-glow-treatment. Real treatment image found and used. Placed under Facial. Brochure: exo-glow-treatment-brochure.html.</v>
       </c>
       <c r="E315" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="316">
@@ -5789,13 +5789,13 @@
         <v>Lumi Face</v>
       </c>
       <c r="C317" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D317" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-face/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/lumi-face. Real hero image found and used. Note: shares a similar salmon-DNA/polynucleotide mechanism with the existing Salmon DNA Facial brochure, but uses the specific branded Dermaren Lumi 10.0 device/protocol targeting face and neck -- kept separate, flag if you want these consolidated. Placed under Facial. Brochure: lumi-face-brochure.html.</v>
       </c>
       <c r="E317" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="318">
@@ -5806,13 +5806,13 @@
         <v>Lumi Eyes</v>
       </c>
       <c r="C318" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D318" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/lumi-eyes/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/lumi-eyes. Real dedicated image found and used (a second image on the page was an unrelated eyebrow-transplant photo, not used). Note: addresses the same under-eye area as the existing Under Eye Fillers brochure but uses PDRN/salmon-DNA polynucleotides rather than hyaluronic acid filler -- kept separate as a distinct product class, flag if overlap is a concern. Placed under Injectable. Brochure: lumi-eyes-brochure.html.</v>
       </c>
       <c r="E318" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="319">
@@ -6843,13 +6843,13 @@
         <v>IV Drip Therapy</v>
       </c>
       <c r="C379" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D379" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/iv-drip-therapy-delhi/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/iv-drip-therapy-delhi that this is a general educational overview of drip categories (hydration, glutathione, vitamin C/B-complex, recovery), process, benefits, and FAQs -- not a specific named drip. This heavily overlaps with the existing House of Drips brochure (16 pages already covering "The Drip Menu", "How Does It Work", "IV Drips vs Oral Supplements", "Your Drip Schedule", FAQ). No new brochure built, this row is covered by house-of-drips-brochure.html (Drip Therapy category) -- flag if you would prefer a separate brochure for this specific page instead.</v>
       </c>
       <c r="E379" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="380">
@@ -6860,13 +6860,13 @@
         <v>Stem Cell Therapy</v>
       </c>
       <c r="C380" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D380" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/stem-cell-therapy/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/stem-cell-therapy. Real banner image found and used. Note: mechanism (scalp tissue biopsy -&gt; centrifuge processing -&gt; reinjection) strongly overlaps with the existing Regenera Activa brochure (also biopsy-based autologous regenerative hair therapy) -- protocols differ (4 sessions over months here vs. Regenera Activa's single session), so kept as a distinct catalog item, flag if you want these consolidated or cross-referenced. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: stem-cell-therapy-brochure.html.</v>
       </c>
       <c r="E380" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="381">
@@ -6962,13 +6962,13 @@
         <v>Deesse Pro LED Mask</v>
       </c>
       <c r="C386" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D386" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/deesse-pro-led-mask/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/deesse-pro-led-mask. Real product images found and used. Placed under Facial. Brochure: deesse-pro-led-mask-brochure.html.</v>
       </c>
       <c r="E386" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="387">

</xml_diff>

<commit_message>
Mark batch 16 brochures Completed in brochure.xlsx; merge Dermarolling, Dermapen Treatment, Tricort, IPL Therapy, and PRP Treatment into existing brochures
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -2729,13 +2729,13 @@
         <v>Signature Facial</v>
       </c>
       <c r="C137" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D137" t="str">
-        <v>Live site page found for scraping: https://www.isaacluxe.co/signature-facial-treatment-3/ [fuzzy]. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/signature-facial-treatment-3. Real treatment image found and used. Placed under Facial. Brochure: signature-facial-brochure.html.</v>
       </c>
       <c r="E137" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="138">
@@ -3052,13 +3052,13 @@
         <v>Morphiya Scalp</v>
       </c>
       <c r="C156" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D156" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Existing brochure: Morphyia (morphyia-skin-hair-treatment-brochure.html). Missed in the original cross-reference due to a typo in this row ("Morphiya" vs "Morphyia").</v>
       </c>
       <c r="E156" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="157">
@@ -5942,13 +5942,13 @@
         <v>Tribeam Laser</v>
       </c>
       <c r="C326" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D326" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tribeam-laser/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/tribeam-laser. Real banner image found and used. Note: this page is actually about a specific Q-switch Nd:YAG tattoo-removal device (Tri-Beam Premium, Rich-PTP dual pulse) despite the "Facial" category label -- conceptually overlaps with the existing Tattoo Removal brochure (also Q-switched laser), but is a distinctly named device with its own dedicated page, kept separate similar to the CoolSculpting/Cryolipolysis precedent -- flag if you want these consolidated. Placed under Facial per its Excel category. Brochure: tribeam-laser-brochure.html.</v>
       </c>
       <c r="E326" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="327">
@@ -5976,13 +5976,13 @@
         <v>IPL Therapy</v>
       </c>
       <c r="C328" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D328" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/ipl-therapy/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/ipl-therapy that this describes the same Intense Pulsed Light technology and treats the same conditions (pigmentation, redness/broken capillaries, acne scars) as the existing Photo Facial brochure. No new brochure built, this row is covered by photo-facial-brochure.html (Facial category).</v>
       </c>
       <c r="E328" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="329">
@@ -6316,13 +6316,13 @@
         <v>MNRF Treatment</v>
       </c>
       <c r="C348" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D348" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mnrf-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/mnrf-treatment. Real treatment demonstration image found and used. Placed under Facial. Brochure: mnrf-treatment-brochure.html.</v>
       </c>
       <c r="E348" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="349">
@@ -6333,13 +6333,13 @@
         <v>Dermarolling / Advanced Microneedling</v>
       </c>
       <c r="C349" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D349" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/dermarolling-treatment-advance-microneedling-therapy that this page describes microneedling generically without naming any distinct device/brand -- the same technique already covered by the existing Derma Roller brochure. No new brochure built, this row is covered by dermaroller-brochure.html (Facial category).</v>
       </c>
       <c r="E349" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="350">
@@ -6350,13 +6350,13 @@
         <v>Dermapen Treatment</v>
       </c>
       <c r="C350" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D350" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermapen-treatment/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/dermapen-treatment that this page explicitly and repeatedly names "Dermapen 4" as the device -- the same treatment already covered by the existing Dermapen 4 brochure (one of the richer original-template brochures, 16 pages). No new brochure built, this row is covered by dermapen-4-brochure.html.</v>
       </c>
       <c r="E350" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
     </row>
     <row r="351">
@@ -6384,13 +6384,13 @@
         <v>Electrocautery Treatment</v>
       </c>
       <c r="C352" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D352" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/electrocautery-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/electrocautery-treatment. Real treatment demonstration image found and used. Placed under Facial. Brochure: electrocautery-treatment-brochure.html.</v>
       </c>
       <c r="E352" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="353">
@@ -6503,13 +6503,13 @@
         <v>Tricort Injection</v>
       </c>
       <c r="C359" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D359" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/tricort-injection/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/tricort-injection that Tricort is Triamcinolone Acetonide -- the same active drug/corticosteroid already covered by the existing Kenacort Injection brochure (also Triamcinolone Acetonide), just a different brand name for the identical drug. No new brochure built, this row is covered by kenacort-injection-brochure.html.</v>
       </c>
       <c r="E359" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="360">
@@ -6707,13 +6707,13 @@
         <v>PRP Treatment</v>
       </c>
       <c r="C371" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D371" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/prp-treatment-in-bangalore/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/prp-treatment-in-bangalore that this page is exclusively about PRP for hair loss (not face/skin) -- the same treatment already covered by the existing PRP Hair Treatment brochure, just a city-specific (Bangalore) landing page. No new brochure built, this row is covered by prp-hair-treatment-brochure.html.</v>
       </c>
       <c r="E371" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="372">
@@ -6792,13 +6792,13 @@
         <v>Morphyia Skin and Hair Treatment</v>
       </c>
       <c r="C376" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D376" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/morphyia-skin-and-hair-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/morphyia-skin-and-hair-treatment. Real hero image found and used. Placed under Anti Aging -- Hair &amp; Scalp (treats both skin and hair, category chosen per Excel's "Hair" grouping). Brochure: morphyia-skin-hair-treatment-brochure.html.</v>
       </c>
       <c r="E376" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="377">
@@ -6979,13 +6979,13 @@
         <v>Skin Perfect Oasis</v>
       </c>
       <c r="C387" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D387" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-perfect-oasis/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/skin-perfect-oasis. Real hero image found and used. Note: similarly named to the existing "Oasis Facial" brochure, but this is a broader curated range/menu of treatments (waxing through advanced facials) rather than the same single iontophoresis facial -- kept separate as genuinely different scope, flag if the naming similarity is a concern. Placed under Facial as closest fit (Excel lists it as Wellness/Uncategorized). Brochure: skin-perfect-oasis-brochure.html.</v>
       </c>
       <c r="E387" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="388">

</xml_diff>

<commit_message>
Update brochure.xlsx: batch 16 + batch 17 completions and merges
Batch 16 (6 rows): Signature Facial, Tribeam Laser, Electrocautery Treatment, Morphyia Skin and Hair Treatment, MNRF Treatment, Skin Perfect Oasis, plus 6 merge/duplicate rows resolved.

Batch 17 (11 rows): 6 new builds (Eczema Treatment, Underarm Darkening, Permanent Beard Shaping, Scar Treatment, Skin Whitening Treatment, Sun/Age Spots) and 5 merges (Collagen Induction Therapy -> Dermaroller, Pink Anti-Aging Treatment -> Pink Treatment, Dermal Thread Treatment -> Thread Lift, Hyaluronic Acid Therapy -> Viscoderm Hydrobooster, Cryotherapy Facial -> Cryo Facial).

Reconciled: 142 unique files in index.html, all 142 marked Completed in Excel, zero gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -5823,13 +5823,13 @@
         <v>Cryotherapy Facial</v>
       </c>
       <c r="C319" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D319" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/cryotherapy-facial/. Not yet built.</v>
+        <v>Two separate scrapes of isaacluxe.co/cryotherapy-facial (batches 16 and 17) returned inconsistent mechanism descriptions, but both used the same image filenames (Cryo-Facial-.webp / Cryo-Facial_1000x1000...) as the existing Cryo Facial brochure -- confirmed as the same treatment/page. Merge decision confirmed with user. No new brochure built, this row is covered by cryo-facial-brochure.html.</v>
       </c>
       <c r="E319" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="320">
@@ -6061,13 +6061,13 @@
         <v>Pink Anti-Aging Treatment</v>
       </c>
       <c r="C333" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D333" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/pink-anti-aging-treatment/. Not yet built.</v>
+        <v>Confirmed this is the same treatment already covered by the existing Pink Treatment brochure (row 9/156) -- "Pink Anti-Aging Treatment" is a fuller descriptive name for the same carboxytherapy-based "Pink Treatment" already built. No new brochure built, this row is covered by pink-treatment-brochure.html.</v>
       </c>
       <c r="E333" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="334">
@@ -6197,13 +6197,13 @@
         <v>Eczema Treatment</v>
       </c>
       <c r="C341" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D341" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/eczema-treatment-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/eczema-treatment. Real treatment image found and used. Placed under Facial. Brochure: eczema-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E341" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="342">
@@ -6231,13 +6231,13 @@
         <v>Sun / Age Spots</v>
       </c>
       <c r="C343" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D343" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/sun-age-spots/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/sun-age-spots. Real treatment image found and used. Placed under Facial. Brochure: sun-age-spots-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E343" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="344">
@@ -6248,13 +6248,13 @@
         <v>Underarm Darkening</v>
       </c>
       <c r="C344" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D344" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/underarm-darkening/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/underarm-darkening (treatment/condition page). Real banner image found and used. Placed under Facial. Brochure: underarm-darkening-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E344" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="345">
@@ -6265,13 +6265,13 @@
         <v>Scar Treatment</v>
       </c>
       <c r="C345" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D345" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/scar-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/scar-treatment. Real before/after treatment images found and used. Note: distinct from the existing "Acne Scar Treatment" brochure (pitted/rolling/boxcar acne scarring specifically) -- this page covers acne, burn, surgical, and injury scars broadly, kept separate as genuinely different scope. Placed under Facial. Brochure: scar-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E345" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="346">
@@ -6299,13 +6299,13 @@
         <v>Skin Whitening Treatment</v>
       </c>
       <c r="C347" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D347" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-whitening-treatment-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/skin-whitening-treatment. Real treatment image found and used. Placed under Facial. Brochure: skin-whitening-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E347" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="348">
@@ -6367,13 +6367,13 @@
         <v>Collagen Induction Therapy</v>
       </c>
       <c r="C351" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D351" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/collagen-induction-therapy/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/derma-roller-treatment (the source page for this exact treatment name -- "Collagen Induction Therapy" is the clinical name for microneedling with a derma roller) that this is the same treatment already covered by the existing Dermaroller brochure. No new brochure built, this row is covered by dermaroller-brochure.html (Facial category).</v>
       </c>
       <c r="E351" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="352">
@@ -6401,13 +6401,13 @@
         <v>Permanent Beard Shaping</v>
       </c>
       <c r="C353" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D353" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/permanent-beard-shaping-treatment-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/permanent-beard-shaping. PHOTO CHECK: no images found on the source page or elsewhere on isaacluxe.co for this treatment. No photo added (9 images, baseline only). Placed under Facial. Brochure: permanent-beard-shaping-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
       </c>
       <c r="E353" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="354">
@@ -6537,13 +6537,13 @@
         <v>Hyaluronic Acid Therapy</v>
       </c>
       <c r="C361" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D361" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hyaluronic-acid-therapy/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/viscoderm-hydrobooster that this is the same hyaluronic-acid-based skin-boosting injectable already covered by the existing Viscoderm Hydrobooster brochure. No new brochure built, this row is covered by viscoderm-hydrobooster-brochure.html.</v>
       </c>
       <c r="E361" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="362">
@@ -6571,13 +6571,13 @@
         <v>Dermal Thread Treatment</v>
       </c>
       <c r="C363" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D363" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/dermal-thread-treatment/. Not yet built.</v>
+        <v>Confirmed this is the same PDO/PLLA thread-based treatment already covered by the existing Thread Lift brochure (row 97). No new brochure built, this row is covered by thread-lift-brochure.html. (Note: Aptos Thread Lift and Thread Face Lift are separately-built, distinctly named catalog items already flagged in their own rows -- this one maps to the base "Thread Lift" brochure specifically.)</v>
       </c>
       <c r="E363" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="364">

</xml_diff>

<commit_message>
Update brochure.xlsx: document photo additions from full site-wide audit
Annotated 34 rows covering the 26 brochures that received a new treatment photo (26 unique files + duplicate/merge rows referencing them), plus re-verification notes on the 3 brochures confirmed to still have no compliant source image (Permanent Beard Shaping, Qlara, Weight Loss).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -1389,10 +1389,10 @@
         <v>Completed</v>
       </c>
       <c r="D58" t="str">
-        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E58" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="59">
@@ -1406,10 +1406,10 @@
         <v>Completed</v>
       </c>
       <c r="D59" t="str">
-        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E59" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="60">
@@ -1457,10 +1457,10 @@
         <v>Completed</v>
       </c>
       <c r="D62" t="str">
-        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E62" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="63">
@@ -1525,10 +1525,10 @@
         <v>Completed</v>
       </c>
       <c r="D66" t="str">
-        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E66" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="67">
@@ -1593,10 +1593,10 @@
         <v>Completed</v>
       </c>
       <c r="D70" t="str">
-        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration.</v>
       </c>
       <c r="E70" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="71">
@@ -1610,10 +1610,10 @@
         <v>Completed</v>
       </c>
       <c r="D71" t="str">
-        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E71" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="72">
@@ -1661,10 +1661,10 @@
         <v>Completed</v>
       </c>
       <c r="D74" t="str">
-        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E74" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="75">
@@ -1950,10 +1950,10 @@
         <v>Completed</v>
       </c>
       <c r="D91" t="str">
-        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
       </c>
       <c r="E91" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="92">
@@ -2018,7 +2018,7 @@
         <v>Completed</v>
       </c>
       <c r="D95" t="str">
-        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added.</v>
+        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added. RE-VERIFIED 2026-07-28 during full site-wide photo audit: still no compliant image available on isaacluxe.co. Remains the only 3 brochures site-wide without a treatment photo.</v>
       </c>
       <c r="E95" t="str">
         <v>2026-07-15</v>
@@ -2800,10 +2800,10 @@
         <v>Completed</v>
       </c>
       <c r="D141" t="str">
-        <v>Scraped from isaacluxe.co/v-carbon-treatment (also called "Erase Treatment"). Note: conceptually adjacent to the existing Carbon Facial brochure, but a distinct mechanism -- V Carbon is a topical film/spray system (no laser), while Carbon Facial is laser-based -- kept separate, flag if you disagree. Source page images were generic/mismatched stock photos of facial masks, not clearly specific to this treatment -- none used. Placed under Facial. Brochure: v-carbon-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/v-carbon-treatment (also called "Erase Treatment"). Note: conceptually adjacent to the existing Carbon Facial brochure, but a distinct mechanism -- V Carbon is a topical film/spray system (no laser), while Carbon Facial is laser-based -- kept separate, flag if you disagree. Source page images were generic/mismatched stock photos of facial masks, not clearly specific to this treatment -- none used. Placed under Facial. Brochure: v-carbon-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real carbon mask application image added from isaacluxe.co/v-carbon-treatment (previously missing).</v>
       </c>
       <c r="E141" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="142">
@@ -2902,10 +2902,10 @@
         <v>Completed</v>
       </c>
       <c r="D147" t="str">
-        <v>Existing brochure: Exosome Scalp Treatment (exosome-scalp-treatment-brochure.html). Missed in the original cross-reference due to naming difference ("Exosome- Hair" vs "Exosome Scalp Treatment"). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
+        <v>Existing brochure: Exosome Scalp Treatment (exosome-scalp-treatment-brochure.html). Missed in the original cross-reference due to naming difference ("Exosome- Hair" vs "Exosome Scalp Treatment"). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: real before/after hair regrowth image added from isaacluxe.co/exosome-therapy (no dedicated exosome-scalp-specific page exists; used the general Exosome Therapy page's scalp/hair result photo). Also fixed a pre-existing mojibake typo ("Wnt/Î²-catenin" -&gt; "Wnt/β-catenin").</v>
       </c>
       <c r="E147" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="148">
@@ -3922,10 +3922,10 @@
         <v>Completed</v>
       </c>
       <c r="D207" t="str">
-        <v>Brochure already exists: House of Peels (house-of-peels-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
+        <v>Brochure already exists: House of Peels (house-of-peels-brochure.html) [fuzzy] JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: real chemical peel treatment image added from isaacluxe.co/chemical-peel-treatment (no dedicated "House of Peels" page exists; used the general Chemical Peel Treatment page's photo).</v>
       </c>
       <c r="E207" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="208">
@@ -5401,10 +5401,10 @@
         <v>Completed</v>
       </c>
       <c r="D294" t="str">
-        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/tight-pro. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Multipolar Radio Frequency) -- kept separate as its own distinct branded device/sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: tight-pro-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real banner image added from isaacluxe.co/tight-pro (previously missing).</v>
       </c>
       <c r="E294" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="295">
@@ -5469,10 +5469,10 @@
         <v>Completed</v>
       </c>
       <c r="D298" t="str">
-        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/multipolar-radio-frequency-in-delhi. No before/after images on source page. Note: conceptually overlaps with other RF-based skin tightening brochures already built (Forma, IntraGen, Tight Pro) -- kept separate as its own distinct sitemap entry, flag if you want these consolidated. Placed under Body Contouring. Brochure: multipolar-radio-frequency-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/multipolar-radio-frequency-in-delhi (previously missing).</v>
       </c>
       <c r="E298" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="299">
@@ -5486,10 +5486,10 @@
         <v>Completed</v>
       </c>
       <c r="D299" t="str">
-        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3. No before/after images on source page. Note: this generic (non-branded) HIFU device treatment overlaps conceptually with the existing Ultherapy brochure (also focused-ultrasound/HIFU technology, branded Merz device, Face Lifting category) -- source page does not name a specific device/brand, so built as its own line item per its own sitemap URL and Excel row; flag if this should instead be merged into/pointed at Ultherapy. Placed under Body Contouring per its Excel category. Brochure: hifu-skin-tightening-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/hifu-skin-tightening-treatment-in-mumbai-3 (previously missing).</v>
       </c>
       <c r="E299" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="300">
@@ -5690,10 +5690,10 @@
         <v>Completed</v>
       </c>
       <c r="D311" t="str">
-        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/poppy-chin-treatment-in-mumbai. No before/after images on source page. Note: conceptually related to the Square Jaw Treatment brochure (both address chin/jawline definition) but treats a distinct condition (dimple/poppy chin from fat and muscle, vs. bone-structure augmentation) -- kept separate, flag if overlap is a concern. Placed under Face Lifting. Brochure: poppy-chin-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real before/after image added from isaacluxe.co/poppy-chin-treatment-in-mumbai (previously missing).</v>
       </c>
       <c r="E311" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="312">
@@ -5724,10 +5724,10 @@
         <v>Completed</v>
       </c>
       <c r="D313" t="str">
-        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/eve-lom-facial. No before/after images on source page. Placed under Facial. Brochure: eve-lom-facial-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment banner image added from isaacluxe.co/eve-lom-facial (previously missing).</v>
       </c>
       <c r="E313" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="314">
@@ -5860,10 +5860,10 @@
         <v>Completed</v>
       </c>
       <c r="D321" t="str">
-        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html. PHOTO CHECK: source page's only non-logo image was mislabeled/mismatched (a photo captioned "Ultherapy" appearing on the Dermabrasion page) -- not used to avoid misrepresenting the treatment. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/dermabrasion-treatment. No before/after images on source page. Placed under Facial. Brochure: dermabrasion-treatment-brochure.html. PHOTO CHECK: source page's only non-logo image was mislabeled/mismatched (a photo captioned "Ultherapy" appearing on the Dermabrasion page) -- not used to avoid misrepresenting the treatment. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/dermabrasion-treatment (previously missing). Note: image alt-tag on source site says "Ultherapy" but visually depicts a microdermabrasion-style device treatment -- used as the closest genuine on-site match.</v>
       </c>
       <c r="E321" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="322">
@@ -5877,10 +5877,10 @@
         <v>Completed</v>
       </c>
       <c r="D322" t="str">
-        <v>Scraped from isaacluxe.co/microdermabrasion-treatment. Real before/after composite image found and used. Placed under Facial. Brochure: microdermabrasion-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/microdermabrasion-treatment. Real before/after composite image found and used. Placed under Facial. Brochure: microdermabrasion-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/dermabrasion-treatment (previously missing). Note: image alt-tag on source site says "Ultherapy" but visually depicts a microdermabrasion-style device treatment -- used as the closest genuine on-site match.</v>
       </c>
       <c r="E322" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="323">
@@ -6115,10 +6115,10 @@
         <v>Completed</v>
       </c>
       <c r="D336" t="str">
-        <v>Scraped from isaacluxe.co/dark-circles. This is a condition/menu page listing multiple approaches (fillers, Eye Light, peels, laser) similar in structure to the Melasma/Rosacea/Square Jaw pattern -- two of its named modalities (Eye Light, Under Eye/Tear Trough Fillers) already have their own dedicated brochures, referenced here as part of the combined protocol rather than duplicated. No images found on the source page. Placed under Facial. Brochure: dark-circles-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/dark-circles. This is a condition/menu page listing multiple approaches (fillers, Eye Light, peels, laser) similar in structure to the Melasma/Rosacea/Square Jaw pattern -- two of its named modalities (Eye Light, Under Eye/Tear Trough Fillers) already have their own dedicated brochures, referenced here as part of the combined protocol rather than duplicated. No images found on the source page. Placed under Facial. Brochure: dark-circles-treatment-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/dark-circles (previously missing).</v>
       </c>
       <c r="E336" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="337">
@@ -6217,10 +6217,10 @@
         <v>Completed</v>
       </c>
       <c r="D342" t="str">
-        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/keratosis-pilaris. No images found on source page at all. Source page also gave no explicit session count, frequency, or downtime -- omitted rather than fabricated; whoFor section left general. Placed under Facial. Brochure: keratosis-pilaris-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment banner image added from isaacluxe.co/keratosis-pilaris (previously missing).</v>
       </c>
       <c r="E342" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="343">
@@ -6404,7 +6404,7 @@
         <v>Completed</v>
       </c>
       <c r="D353" t="str">
-        <v>Scraped from isaacluxe.co/permanent-beard-shaping. PHOTO CHECK: no images found on the source page or elsewhere on isaacluxe.co for this treatment. No photo added (9 images, baseline only). Placed under Facial. Brochure: permanent-beard-shaping-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/permanent-beard-shaping. PHOTO CHECK: no images found on the source page or elsewhere on isaacluxe.co for this treatment. No photo added (9 images, baseline only). Placed under Facial. Brochure: permanent-beard-shaping-brochure.html. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results), 9 pages total. RE-VERIFIED 2026-07-28 during full site-wide photo audit: still no compliant image available on isaacluxe.co. Remains the only 3 brochures site-wide without a treatment photo.</v>
       </c>
       <c r="E353" t="str">
         <v>2026-07-28</v>
@@ -6523,10 +6523,10 @@
         <v>Completed</v>
       </c>
       <c r="D360" t="str">
-        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/hyaluron-pen-needle-free-filler. No before/after images on source page. Placed under Injectable. Brochure: hyaluron-pen-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment banner image added from isaacluxe.co/hyaluron-pen-needle-free-filler (previously missing).</v>
       </c>
       <c r="E360" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="361">
@@ -6540,7 +6540,7 @@
         <v>Completed</v>
       </c>
       <c r="D361" t="str">
-        <v>Confirmed via isaacluxe.co/viscoderm-hydrobooster that this is the same hyaluronic-acid-based skin-boosting injectable already covered by the existing Viscoderm Hydrobooster brochure. No new brochure built, this row is covered by viscoderm-hydrobooster-brochure.html.</v>
+        <v>Confirmed via isaacluxe.co/viscoderm-hydrobooster that this is the same hyaluronic-acid-based skin-boosting injectable already covered by the existing Viscoderm Hydrobooster brochure. No new brochure built, this row is covered by viscoderm-hydrobooster-brochure.html. PHOTO UPDATE: real before/after image added from isaacluxe.co/viscoderm-hydrobooster (previously flagged as no images found -- re-checked and found on re-scrape).</v>
       </c>
       <c r="E361" t="str">
         <v>2026-07-28</v>
@@ -6557,10 +6557,10 @@
         <v>Completed</v>
       </c>
       <c r="D362" t="str">
-        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/viscoderm-hydrobooster. No before/after images on source page. Placed under Injectable. Brochure: viscoderm-hydrobooster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real before/after image added from isaacluxe.co/viscoderm-hydrobooster (previously flagged as no images found -- re-checked and found on re-scrape).</v>
       </c>
       <c r="E362" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="363">
@@ -6608,10 +6608,10 @@
         <v>Completed</v>
       </c>
       <c r="D365" t="str">
-        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html. PHOTO CHECK: source page has only the generic site logo and footer photo, no treatment-specific image. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/eyebrow-transplant. No before/after images on source page. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: eyebrow-transplant-brochure.html. PHOTO CHECK: source page has only the generic site logo and footer photo, no treatment-specific image. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/eyebrow-transplant (previously missing).</v>
       </c>
       <c r="E365" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="366">
@@ -6659,10 +6659,10 @@
         <v>Completed</v>
       </c>
       <c r="D368" t="str">
-        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/hairgen-booster. No before/after images on source page; source page also gave no explicit session count/frequency. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hairgen-booster-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real product-in-use image added from isaacluxe.co/hairgen-booster (previously missing).</v>
       </c>
       <c r="E368" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="369">
@@ -6676,10 +6676,10 @@
         <v>Completed</v>
       </c>
       <c r="D369" t="str">
-        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/prp-hair-treatment. No before/after images on source page. Distinct from existing Regenera Activa (autologous micrograft) and Mesotherapy (vitamin injection) brochures. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: prp-hair-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment image added from isaacluxe.co/prp-hair-treatment (previously missing).</v>
       </c>
       <c r="E369" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="370">
@@ -6710,10 +6710,10 @@
         <v>Completed</v>
       </c>
       <c r="D371" t="str">
-        <v>Confirmed via isaacluxe.co/prp-treatment-in-bangalore that this page is exclusively about PRP for hair loss (not face/skin) -- the same treatment already covered by the existing PRP Hair Treatment brochure, just a city-specific (Bangalore) landing page. No new brochure built, this row is covered by prp-hair-treatment-brochure.html.</v>
+        <v>Confirmed via isaacluxe.co/prp-treatment-in-bangalore that this page is exclusively about PRP for hair loss (not face/skin) -- the same treatment already covered by the existing PRP Hair Treatment brochure, just a city-specific (Bangalore) landing page. No new brochure built, this row is covered by prp-hair-treatment-brochure.html. PHOTO UPDATE: real treatment image added from isaacluxe.co/prp-hair-treatment (previously missing).</v>
       </c>
       <c r="E371" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="372">
@@ -6761,10 +6761,10 @@
         <v>Completed</v>
       </c>
       <c r="D374" t="str">
-        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total.</v>
+        <v>Scraped from isaacluxe.co/alopecia-areata. No images on source page; source page also gave no explicit session count/downtime, so whoFor section left general rather than fabricated. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: alopecia-areata-treatment-brochure.html. PHOTO CHECK: no images at all found on the source page. No photo added. Added a "Your Treatment Journey" page (Consultation/Procedure/Aftercare/Results) sourced from the same isaacluxe.co page, now 9 pages total. PHOTO UPDATE: real treatment banner image added from isaacluxe.co/alopecia-areata (previously missing).</v>
       </c>
       <c r="E374" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="375">
@@ -6778,10 +6778,10 @@
         <v>Completed</v>
       </c>
       <c r="D375" t="str">
-        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
+        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration.</v>
       </c>
       <c r="E375" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="376">
@@ -6846,10 +6846,10 @@
         <v>Completed</v>
       </c>
       <c r="D379" t="str">
-        <v>Confirmed via isaacluxe.co/iv-drip-therapy-delhi that this is a general educational overview of drip categories (hydration, glutathione, vitamin C/B-complex, recovery), process, benefits, and FAQs -- not a specific named drip. This heavily overlaps with the existing House of Drips brochure (16 pages already covering "The Drip Menu", "How Does It Work", "IV Drips vs Oral Supplements", "Your Drip Schedule", FAQ). No new brochure built, this row is covered by house-of-drips-brochure.html (Drip Therapy category) -- flag if you would prefer a separate brochure for this specific page instead.</v>
+        <v>Confirmed via isaacluxe.co/iv-drip-therapy-delhi that this is a general educational overview of drip categories (hydration, glutathione, vitamin C/B-complex, recovery), process, benefits, and FAQs -- not a specific named drip. This heavily overlaps with the existing House of Drips brochure (16 pages already covering "The Drip Menu", "How Does It Work", "IV Drips vs Oral Supplements", "Your Drip Schedule", FAQ). No new brochure built, this row is covered by house-of-drips-brochure.html (Drip Therapy category) -- flag if you would prefer a separate brochure for this specific page instead. PHOTO UPDATE: real "House of Drip" banner image added from isaacluxe.co/house-of-drips (previously missing -- this menu/hub brochure itself had no unique photo beyond the shared baseline).</v>
       </c>
       <c r="E379" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="380">
@@ -7067,10 +7067,10 @@
         <v>Completed</v>
       </c>
       <c r="D392" t="str">
-        <v>Category-level umbrella brochure covering the full drip menu, not an individual treatment line item -- no row existed in the original 285-row export. Brochure: house-of-drips-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
+        <v>Category-level umbrella brochure covering the full drip menu, not an individual treatment line item -- no row existed in the original 285-row export. Brochure: house-of-drips-brochure.html. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: real "House of Drip" banner image added from isaacluxe.co/house-of-drips (previously missing -- this menu/hub brochure itself had no unique photo beyond the shared baseline).</v>
       </c>
       <c r="E392" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="393">
@@ -7084,7 +7084,7 @@
         <v>Completed</v>
       </c>
       <c r="D393" t="str">
-        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html. PHOTO CHECK: no corresponding live isaacluxe.co page exists for Qlara (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition.</v>
+        <v>Device/treatment not present in the original 285-row service-menu export at all. Brochure: qlara-brochure.html. PHOTO CHECK: no corresponding live isaacluxe.co page exists for Qlara (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. RE-VERIFIED 2026-07-28 during full site-wide photo audit: still no compliant image available on isaacluxe.co. Remains the only 3 brochures site-wide without a treatment photo.</v>
       </c>
       <c r="E393" t="str">
         <v>2026-07-16</v>

</xml_diff>

<commit_message>
Add missing photo to Weight Loss brochure; found via rigorous re-audit
User asked for a full re-check of every brochure. Ran a hash-based audit comparing every embedded image across all 142 files (not just counting totals) to catch anything the earlier count-based check missed. Found Weight Loss Drip had been incorrectly treated as unsourceable -- it's actually another IV drip formulation like the other 8, so it gets the same real "House of Drip" banner photo. Only 2 brochures site-wide now have no photo (Permanent Beard Shaping, Qlara), both confirmed via exhaustive sitemap search to have no compliant image anywhere on isaacluxe.co.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -2018,10 +2018,10 @@
         <v>Completed</v>
       </c>
       <c r="D95" t="str">
-        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added. RE-VERIFIED 2026-07-28 during full site-wide photo audit: still no compliant image available on isaacluxe.co. Remains the only 3 brochures site-wide without a treatment photo.</v>
+        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added. PHOTO UPDATE: on a second, more rigorous re-check, recognised this is actually "Weight Loss Drip" (an IV drip formulation like the other 8 drips), so the same real "House of Drip" umbrella banner photo was added. Only 2 brochures site-wide (Permanent Beard Shaping, Qlara) remain without a treatment photo -- both confirmed via exhaustive sitemap search to have no compliant source image anywhere on isaacluxe.co.</v>
       </c>
       <c r="E95" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-28</v>
       </c>
     </row>
     <row r="96">

</xml_diff>

<commit_message>
Update brochure.xlsx: batch 19 completions, merges, and scope decisions
10 new brochures (11 rows, Hair Fall + Baldness both point to the combined Hair Loss & Baldness hub), 2 merges (Crow's Feet -> Botox, Anti-Wrinkle Injection/Facelift Filler -> Face Lift Filler), 1 marked Out of Scope (Skin Tightening Treatment -- generic skincare content, no device/procedure), and 2 marked Missing - No Source (Spa Therapy, Forest Essentials Body Spa -- both pages return broken 301 redirects on the live site).

This clears the "To Build (source available)" queue to zero. Reconciled: 152 unique files in index.html, all 152 marked Completed in Excel, zero gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -5500,13 +5500,13 @@
         <v>Skin Tightening Treatment</v>
       </c>
       <c r="C300" t="str">
-        <v>To Build (source available)</v>
+        <v>Out of Scope</v>
       </c>
       <c r="D300" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-tightening-treatment-in-vasant-vihar/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/skin-tightening-treatment-in-vasant-vihar that this page is entirely generic skincare-product content (oils, antioxidants, ingredients like Cynergy TK) with no medical device or bookable procedure described -- unlike the 5 device-specific skin tightening brochures already built (HIFU, Forma, IntraGen, Tight Pro, Multipolar RF). Marked Out of Scope, confirmed with user -- not a real gap in the brochure lineup.</v>
       </c>
       <c r="E300" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="301">
@@ -5925,13 +5925,13 @@
         <v>Skin Lightening Treatment</v>
       </c>
       <c r="C325" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D325" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/skin-lightening-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/skin-lightening-treatment. This page describes a curated multi-modality programme (V Bianco IV therapy, chemical/carbon peels, dermabrasion, medi-facials) rather than one single treatment -- built as a short concern-focused overview brochure (confirmed with user) rather than duplicating the full protocol detail already covered in the existing V-Bianco, House of Peels, and Dermabrasion Treatment brochures. Real treatment image found and used. Placed under Facial. Brochure: skin-lightening-treatment-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E325" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="326">
@@ -5959,13 +5959,13 @@
         <v>Fractional Laser Skin</v>
       </c>
       <c r="C327" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D327" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/fractional-laser-skin/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/fractional-laser-skin. Describes fractional CO2 laser resurfacing (microthermal zones) -- a distinct ablative mechanism from the existing Laser Toning (Q-Switch) and Scar Treatment/Sun-Age Spots (non-ablative) brochures, kept separate as genuinely different technology, flagged for awareness. Real treatment image found and used (note: page's first-listed "background" image was actually an unrelated injection photo -- used the correct main banner image instead after a second, more careful check). Placed under Facial. Brochure: fractional-laser-skin-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E327" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="328">
@@ -5993,13 +5993,13 @@
         <v>Face Brightening Treatment</v>
       </c>
       <c r="C329" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D329" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/face-brightening-treatments-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/face-brightening-treatments-in-mumbai. Describes a combination of already-built modalities (HydraFacial/SilkPeel, Q-Switch Laser Toning, Chemical Peels, Glutathione IV Drips) -- built as a short concern-focused overview brochure (confirmed with user) rather than duplicating existing HydraFacial MD Elite, Laser Toning, and House of Peels brochures. Real treatment image found and used. Placed under Facial. Brochure: face-brightening-treatment-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E329" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="330">
@@ -6044,13 +6044,13 @@
         <v>Anti-Ageing Laser Treatment</v>
       </c>
       <c r="C332" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D332" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-ageing-laser-treatment/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/anti-ageing-laser-treatment. Describes generic laser types (Fractional CO2, Erbium, non-ablative) without naming a specific device -- built as a short concern-focused overview brochure (confirmed with user), with an acknowledged conceptual overlap with the new Fractional Laser Skin brochure and the existing Laser Toning brochure (different laser types/mechanisms, kept separate). Real treatment image found and used. Placed under Facial. Brochure: anti-ageing-laser-treatment-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E332" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="333">
@@ -6078,13 +6078,13 @@
         <v>Wrinkles Treatment</v>
       </c>
       <c r="C334" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D334" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/wrinkles-treatment-in-mumbai/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/wrinkles-treatment-in-mumbai. Very generic page (mentions "laser therapy" and "dermal fillers" without specifics) -- built as a short concern-focused overview brochure (confirmed with user), with an acknowledged heavy conceptual overlap with the existing Botox, Dermal Fillers, and Laser Toning brochures. PHOTO CHECK: no treatment images found on the source page or elsewhere on isaacluxe.co -- no photo added (9 images, baseline only). Placed under Facial. Brochure: wrinkles-treatment-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E334" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="335">
@@ -6095,13 +6095,13 @@
         <v>Crow's Feet Treatment</v>
       </c>
       <c r="C335" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D335" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/crows-feet-treatment-in-delhi/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/crows-feet-treatment-in-delhi that Botox/neuromodulator injections are the primary described mechanism ("tiny injections...relax muscles"), framed alongside other modalities as a holistic combination approach -- merge into existing Botox brochure confirmed with user. No new brochure built, this row is covered by botox-treatment-brochure.html.</v>
       </c>
       <c r="E335" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="336">
@@ -6418,13 +6418,13 @@
         <v>Men's Grooming Treatments</v>
       </c>
       <c r="C354" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D354" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/mens-grooming-treatments/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/mens-grooming-treatments. Confirmed hub page listing 4 already-built treatments (Laser Hair Reduction for beard shaping, HydraFacial, Botox, PRP Hair Treatment) -- built as its own lightweight hub brochure (confirmed with user), similar precedent to House of Drips/House of Peels. Real hub graphic image found and used. Placed under Facial. Brochure: mens-grooming-treatments-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E354" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="355">
@@ -6452,13 +6452,13 @@
         <v>Anti-Wrinkle Injection (Facelift Filler)</v>
       </c>
       <c r="C356" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D356" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/anti-wrinkle-injection-for-facelift-filler/. Not yet built.</v>
+        <v>Confirmed via isaacluxe.co/anti-wrinkle-injection-for-facelift-filler that this describes a combination of neuromodulators, hyaluronic acid fillers, and biostimulators -- i.e. a "liquid facelift" -- matching the existing Face Lift Filler brochure's scope. No new brochure built, this row is covered by face-lift-filler-brochure.html.</v>
       </c>
       <c r="E356" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="357">
@@ -6690,13 +6690,13 @@
         <v>Advanced PRP Growth Factor Concentrate (GFC)</v>
       </c>
       <c r="C370" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D370" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/advanced-prp-growth-factor-concentrate-therapygfc. Confirmed genuinely distinct from the existing PRP Hair Treatment brochure -- GFC isolates pure growth factors (vs PRP's platelet+plasma mix), explicitly marketed on-site as "5x more potent" with its own comparison table. Real treatment image found and used. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: advanced-prp-gfc-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E370" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="371">
@@ -6724,13 +6724,13 @@
         <v>Hair Fall Treatment</v>
       </c>
       <c r="C372" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D372" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/hair-fall-treatment-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/hair-fall-treatment-in-delhi. Confirmed hub page listing already-built treatments (PRP, Hair Transplant, Mesotherapy, QR-678, Keravive, Hairgen Booster, Alopecia Areata, non-surgical replacement). Combined with Baldness Treatment (row 372) into a single "Hair Loss &amp; Baldness" hub brochure (confirmed with user) since both source pages list an almost identical treatment menu -- building two near-identical hub brochures would have been repetitive. Real before/after treatment image found and used. Placed under Anti Aging -- Hair &amp; Scalp. Brochure: hair-loss-and-baldness-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E372" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="373">
@@ -6741,13 +6741,13 @@
         <v>Baldness Treatment</v>
       </c>
       <c r="C373" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D373" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/baldness-treatment-in-delhi/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/baldness-treatment-in-delhi. Confirmed hub page listing the same set of already-built treatments as Hair Fall Treatment (row 371) -- combined with it into a single "Hair Loss &amp; Baldness" hub brochure (confirmed with user) rather than building two near-identical brochures. No new brochure built separately; covered by hair-loss-and-baldness-brochure.html.</v>
       </c>
       <c r="E373" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="374">
@@ -6928,13 +6928,13 @@
         <v>Spa Therapy</v>
       </c>
       <c r="C384" t="str">
-        <v>To Build (source available)</v>
+        <v>Missing - No Source</v>
       </c>
       <c r="D384" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/spa-therapy/. Not yet built.</v>
+        <v>isaacluxe.co/spa-therapy returns HTTP 301 with no redirect target (confirmed via curl with browser user-agent, both with and without trailing slash) -- page appears to have been removed from the live site despite still being listed in the sitemap. No source content available to build from.</v>
       </c>
       <c r="E384" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="385">
@@ -6945,13 +6945,13 @@
         <v>Forest Essentials Body Spa</v>
       </c>
       <c r="C385" t="str">
-        <v>To Build (source available)</v>
+        <v>Missing - No Source</v>
       </c>
       <c r="D385" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/forest-essentials-body-spa/. Not yet built.</v>
+        <v>isaacluxe.co/forest-essentials-body-spa returns HTTP 301 with no redirect target (confirmed via curl with browser user-agent, both with and without trailing slash) -- page appears to have been removed from the live site despite still being listed in the sitemap. No source content available to build from.</v>
       </c>
       <c r="E385" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="386">
@@ -7013,13 +7013,13 @@
         <v>Bridal Makeover</v>
       </c>
       <c r="C389" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D389" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/bridal-makeover/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/bridal-makeover. Genuinely distinct 5-step wedding-prep programme (consultation, timeline planning, skin correction, refinement, final checks). Real bridal image found and used. New "Wellness" category created in index.html for this and Groom Makeover. Brochure: bridal-makeover-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E389" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="390">
@@ -7030,13 +7030,13 @@
         <v>Groom Makeover</v>
       </c>
       <c r="C390" t="str">
-        <v>To Build (source available)</v>
+        <v>Completed</v>
       </c>
       <c r="D390" t="str">
-        <v>Found via reverse sitemap check (not in the original clinic service-menu Excel). Live page: https://www.isaacluxe.co/groom-makeover/. Not yet built.</v>
+        <v>Scraped from isaacluxe.co/groom-makeover. Genuinely distinct 1-month wedding-prep programme (spa sessions, PRP hair therapy, MedContour, laser hair reduction, beard shaping, CoolSculpting, Emface). Real treatment image found and used. Placed under new "Wellness" category. Brochure: groom-makeover-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E390" t="str">
-        <v/>
+        <v>2026-07-29</v>
       </c>
     </row>
     <row r="391">

</xml_diff>

<commit_message>
Add "Status Guide" tab to brochure.xlsx explaining what each status means
Documents the 3 statuses used in the main sheet (Completed/Missing - No Source/Out of Scope) with counts, plus a full breakdown of the 80 Out of Scope rows: 6 admin/billing line items (Common), 73 salon/hair/nail services (Salon, not clinical treatments), and 1 case-by-case judgment call (Skin Tightening Treatment). Generated from live data on the main sheet, not hand-written.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Status Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$395</definedName>
@@ -401,13 +402,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="100.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7129,4 +7123,141 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E395"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D18"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status Guide — What Each Status Means</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>As of 2026-07-29 — 394 total rows in the main sheet, every row falls into exactly one of these 3 statuses:</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Count</v>
+      </c>
+      <c r="C5" t="str">
+        <v>What it means</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="B6">
+        <v>184</v>
+      </c>
+      <c r="C6" t="str">
+        <v>A brochure exists and is live on index.html for this treatment (or this row is an intentional duplicate/merge pointing to an existing brochure).</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Missing - No Source</v>
+      </c>
+      <c r="B7">
+        <v>130</v>
+      </c>
+      <c r="C7" t="str">
+        <v>A real, legitimate treatment, but no usable source content exists yet on isaacluxe.co (no matching page, or the page is broken/removed) and no PDF/source has been supplied. Cannot build without fabricating content.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Out of Scope</v>
+      </c>
+      <c r="B8">
+        <v>80</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Not a clinical aesthetic treatment that warrants its own brochure — see breakdown below.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Out of Scope — Full Breakdown</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Group</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Count</v>
+      </c>
+      <c r="C13" t="str">
+        <v>What it is</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Example items</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Common (billing / admin line items)</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Administrative or add-on line items from the original service-menu export — not standalone treatments, so they don't need their own brochure.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Body Shaving, General Consultation, Massage, Meet-up, Refill, Sub-Session</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Salon (hair/nail/beauty-parlor services)</v>
+      </c>
+      <c r="B15">
+        <v>73</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Hair salon and nail/beauty-parlor services (haircuts, coloring, keratin, rebonding, manicure/pedicure, extensions, threading, mehendi, blow-dry, etc.) — salon-counter services, not clinical aesthetic procedures. (includes 1 blank placeholder row(s) in the source export.)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Acrylic extension, Advance Hair-Wig Long, Advance Hair-Wig Medium, Advance Hair-Wig Small, Aesthetic Training Program 180, Aesthetic Training Program 30, Back Relief Massage, Balyage - Hair Salon, Biotin Hair Treatments, Blepharoplasty, Blow Dry, Comedone Extraction, Diet-Advance-60 FU-180 Days, Diet-Basic-12 FU-90 Days, Diet-Basic-24 FU-180 Days, ... (57 more, see main sheet rows 213-284)</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Body Contouring (case-by-case)</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Reviewed individually and confirmed with the user to be out of scope (e.g. generic content with no real device/procedure behind it).</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Skin Tightening Treatment</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Note: this sheet is a point-in-time summary generated from the main sheet on 2026-07-29. If rows are added/reclassified later, re-generate rather than hand-editing counts here.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update brochure.xlsx: document the 12 Journey-page content fixes from the full-site audit
Notes added to the 9 IV drip brochures, House of Sculpt, House of Proportion, and Retix C explaining the added Journey page and its source (each brochure's own existing content, not fabricated). Reconciled: 152 unique files in index.html, all 152 marked Completed in Excel, zero gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Status Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$395</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -402,6 +402,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E395"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="100.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1383,10 +1390,10 @@
         <v>Completed</v>
       </c>
       <c r="D58" t="str">
-        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Beauty Infusion (beauty-infusion-brochure.html) [exact] PHOTO CHECK: this brochure predates the isaacluxe.co sitemap cross-reference and has no corresponding live page on the site (confirmed via sitemap search) -- no compliant (isaacluxe.co) photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E58" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="59">
@@ -1400,10 +1407,10 @@
         <v>Completed</v>
       </c>
       <c r="D59" t="str">
-        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Existing brochure: Celestial Drip (celestial-drip-brochure.html). Missed in the original cross-reference due to a typo in this row ("Celestrial" vs "Celestial"). PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E59" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="60">
@@ -1451,10 +1458,10 @@
         <v>Completed</v>
       </c>
       <c r="D62" t="str">
-        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Destress Drip (destress-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E62" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="63">
@@ -1519,10 +1526,10 @@
         <v>Completed</v>
       </c>
       <c r="D66" t="str">
-        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Eternal Drip (eternal-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E66" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="67">
@@ -1587,10 +1594,10 @@
         <v>Completed</v>
       </c>
       <c r="D70" t="str">
-        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration.</v>
+        <v>Brochure already exists: Hair Growth (hair-growth-brochure.html) [fuzzy] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E70" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="71">
@@ -1604,10 +1611,10 @@
         <v>Completed</v>
       </c>
       <c r="D71" t="str">
-        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Hangover Cure Drip (hangover-cure-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E71" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="72">
@@ -1655,10 +1662,10 @@
         <v>Completed</v>
       </c>
       <c r="D74" t="str">
-        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Immunity Plus Drip (immunity-plus-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E74" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="75">
@@ -1944,10 +1951,10 @@
         <v>Completed</v>
       </c>
       <c r="D91" t="str">
-        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations.</v>
+        <v>Brochure already exists: Sports Booster Drip (sports-booster-drip-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this drip (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this drip -- no additional source available, so no Journey page added. PHOTO UPDATE: no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration -- same delivery modality as all drip formulations. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E91" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="92">
@@ -2012,10 +2019,10 @@
         <v>Completed</v>
       </c>
       <c r="D95" t="str">
-        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added. PHOTO UPDATE: on a second, more rigorous re-check, recognised this is actually "Weight Loss Drip" (an IV drip formulation like the other 8 drips), so the same real "House of Drip" umbrella banner photo was added. Only 2 brochures site-wide (Permanent Beard Shaping, Qlara) remain without a treatment photo -- both confirmed via exhaustive sitemap search to have no compliant source image anywhere on isaacluxe.co.</v>
+        <v>Brochure already exists: Weight Loss (weight-loss-brochure.html) [exact] PHOTO CHECK: no corresponding live isaacluxe.co page exists for this treatment (confirmed via sitemap search) -- no compliant photo source available. No photo added. JOURNEY PAGE CHECK: no live isaacluxe.co page exists for this treatment -- no additional source available, so no Journey page added. PHOTO UPDATE: on a second, more rigorous re-check, recognised this is actually "Weight Loss Drip" (an IV drip formulation like the other 8 drips), so the same real "House of Drip" umbrella banner photo was added. Only 2 brochures site-wide (Permanent Beard Shaping, Qlara) remain without a treatment photo -- both confirmed via exhaustive sitemap search to have no compliant source image anywhere on isaacluxe.co. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E95" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="96">
@@ -2675,10 +2682,10 @@
         <v>Completed</v>
       </c>
       <c r="D134" t="str">
-        <v>Brochure already exists: Retix C (retix-c-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure was originally built from retixc.com (manufacturer site), not an isaacluxe.co page -- no Journey page added in this pass, flag if you want it sourced from retixc.com.</v>
+        <v>Brochure already exists: Retix C (retix-c-brochure.html) [exact] JOURNEY PAGE CHECK: this brochure was originally built from retixc.com (manufacturer site), not an isaacluxe.co page -- no Journey page added in this pass, flag if you want it sourced from retixc.com. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" section (Consultation/Application/Aftercare) -- retixc.com itself had no usable protocol detail on re-check.</v>
       </c>
       <c r="E134" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="135">
@@ -5344,10 +5351,10 @@
         <v>Completed</v>
       </c>
       <c r="D291" t="str">
-        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Structure cards already on the Treatment page, so no Journey page was added to avoid redundancy.</v>
+        <v>Scraped from isaacluxe.co/house-of-sculpt. This is a curated multi-treatment programme page, not a single technology -- most of its listed components (Exilis Elite, CoolSculpting, Emsculpt NEO, Med Contour, Ballancer Pro, X-Wave) already have their own dedicated brochures, so this brochure covers the programme structure itself rather than re-describing each modality. Note: the source page also mentions Morpheus8 and Pink Infrared Sauna as included treatments, neither of which has its own brochure yet -- flag if these should be added to the build queue. Banner/hero images only, no before/after pairs. Placed under Body Contouring. Brochure: house-of-sculpt-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Structure cards already on the Treatment page, so no Journey page was added to avoid redundancy. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built as a programme-level journey (consultation -&gt; multi-technology plan -&gt; aftercare -&gt; results), consistent with the pattern used for Men's Grooming Treatments and Hair Loss &amp; Baldness.</v>
       </c>
       <c r="E291" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="292">
@@ -5361,10 +5368,10 @@
         <v>Completed</v>
       </c>
       <c r="D292" t="str">
-        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Goals cards already on the Treatment page, so no Journey page was added to avoid redundancy.</v>
+        <v>Scraped from isaacluxe.co/house-of-proportion. CATEGORY FLAG: Excel lists this row under Body Contouring, but the source page content is entirely facial (golden-ratio facial symmetry programme built from dermal fillers, Botox, Ultherapy, Thread Face Lift, Profhilo) -- placed under Face Lifting on index.html instead as the better content match; flag if you want it moved back to Body Contouring or elsewhere. This is a curated multi-treatment programme; two of its components (Ultherapy, Thread Face Lift) already have their own dedicated brochures, and Profhilo is mentioned but has no brochure of its own yet -- flag if it should be added to the build queue. Banner/hero images only, no before/after pairs. Brochure: house-of-proportion-brochure.html. Real treatment photo added from isaacluxe.co (2026-07-25). JOURNEY PAGE CHECK: this is a curated multi-treatment programme (not a single procedure) -- a step-by-step "journey" would repeat the Programme Goals cards already on the Treatment page, so no Journey page was added to avoid redundancy. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built as a programme-level journey (consultation -&gt; multi-technology plan -&gt; aftercare -&gt; results), consistent with the pattern used for Men's Grooming Treatments and Hair Loss &amp; Baldness.</v>
       </c>
       <c r="E292" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="293">
@@ -6772,10 +6779,10 @@
         <v>Completed</v>
       </c>
       <c r="D375" t="str">
-        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration.</v>
+        <v>DUPLICATE CAUGHT: initially built as its own new brochure (qr678-neo-hair-growth-brochure.html), but discovered during cross-check that the pre-existing QR678-hair-science-brochure.html (already tracked at row "Hair science- QR678") covers this exact same QR678 Neo treatment. The new duplicate file and its index.html card were removed; this row is now marked Completed against the existing QR678-hair-science-brochure.html (Injectable category). JOURNEY PAGE CHECK: this brochure already uses the older, richer template (15-17 pages) and already includes an equivalent step-by-step/journey page plus FAQ, Myths vs Facts, and Pre &amp; Post Care sections -- verified via real page count, no addition needed to avoid repetition. PHOTO UPDATE: this is "Hair Growth Drip" (an IV drip, not a topical/device treatment) -- no dedicated page exists for this specific drip, so the real "House of Drip" umbrella banner photo (from isaacluxe.co/house-of-drips) was added, showing actual IV drip administration. JOURNEY PAGE UPDATE (2026-07-30 full-site audit): added a "Your Treatment Journey" page, now 9 pages total. Built from this brochure's own existing "How It Works" 3-step content (no dedicated isaacluxe.co page exists per drip formulation, so a generic re-scrape was not possible) -- not fabricated.</v>
       </c>
       <c r="E375" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="376">
@@ -7128,12 +7135,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D18"/>
-  <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7250,12 +7251,8 @@
         <v>Skin Tightening Treatment</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Note: this sheet is a point-in-time summary generated from the main sheet on 2026-07-29. If rows are added/reclassified later, re-generate rather than hand-editing counts here.</v>
-      </c>
-    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Reconcile 4 stale PRP rows in brochure.xlsx
Hair PRP, Prp, Prp (GFC), and Ultra PRP were marked Missing - No Source before PRP Hair Treatment (2026-07-28) and Advanced PRP GFC (2026-07-29) existed, and were never re-checked afterward. Reclassified as Completed, pointing to the existing brochures. The remaining 7 PRP-related rows (generic PRP, both Blue Tip variants, Neck/Under-Eye/Breast PRP) stay Missing - No Source -- genuinely distinct body-region-specific variants with no matching isaacluxe.co source.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Status Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$395</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2934,13 +2934,13 @@
         <v>Hair PRP</v>
       </c>
       <c r="C149" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D149" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before PRP Hair Treatment was built (2026-07-28). "Hair PRP" is the same generic hair PRP service now covered by the existing PRP Hair Treatment brochure. No new brochure built, this row is covered by prp-hair-treatment-brochure.html.</v>
       </c>
       <c r="E149" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="150">
@@ -3104,13 +3104,13 @@
         <v>Prp</v>
       </c>
       <c r="C159" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D159" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content. [Duplicate name also appears at: row 2 (Anti Aging)]</v>
+        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before PRP Hair Treatment was built (2026-07-28). "Prp" (Hair category) is the same generic hair PRP service now covered by the existing PRP Hair Treatment brochure. No new brochure built, this row is covered by prp-hair-treatment-brochure.html.</v>
       </c>
       <c r="E159" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="160">
@@ -3121,13 +3121,13 @@
         <v>Prp (GFC)</v>
       </c>
       <c r="C160" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D160" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before Advanced PRP GFC was built (2026-07-29). "Prp (GFC)" is the same Growth Factor Concentrate treatment now covered by the existing Advanced PRP GFC brochure. No new brochure built, this row is covered by advanced-prp-gfc-brochure.html.</v>
       </c>
       <c r="E160" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="161">
@@ -3138,13 +3138,13 @@
         <v>Ultra PRP</v>
       </c>
       <c r="C161" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D161" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before PRP Hair Treatment was built (2026-07-28). "Ultra PRP" is treated as the same generic hair PRP service now covered by the existing PRP Hair Treatment brochure -- flagged because the "Ultra" branding/tier is not independently confirmed identical (no isaacluxe.co page names an "Ultra PRP" variant specifically). No new brochure built, this row is covered by prp-hair-treatment-brochure.html.</v>
       </c>
       <c r="E161" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="162">
@@ -7134,7 +7134,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7254,7 +7254,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update brochure.xlsx: document the new PRP-GFC brochure
Face PRP reclassified as Completed -- its skin-rejuvenation content (melasma, wrinkles, acne scars, skin tightening) is covered by the new prp-gfc-brochure.html. Added a cross-reference note on the Prp (GFC) row pointing to this second, richer brochure. Reconciled: 153 unique files in index.html, all 153 marked Completed in Excel, zero gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -486,13 +486,13 @@
         <v>Face PRP</v>
       </c>
       <c r="C5" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D5" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Built from a user-supplied manufacturer PDF (Viyata GFC Kit, Flowrich Pharma) covering GFC-based skin rejuvenation for melasma, wrinkles &amp; fine lines, acne scars, and skin tightening -- matches the general "Face PRP" concern. No new brochure built separately, covered by prp-gfc-brochure.html. Flag if this specific naming was meant to reference a different technique.</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="6">
@@ -3124,7 +3124,7 @@
         <v>Completed</v>
       </c>
       <c r="D160" t="str">
-        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before Advanced PRP GFC was built (2026-07-29). "Prp (GFC)" is the same Growth Factor Concentrate treatment now covered by the existing Advanced PRP GFC brochure. No new brochure built, this row is covered by advanced-prp-gfc-brochure.html.</v>
+        <v>RECONCILED 2026-07-30: this row was marked Missing - No Source before Advanced PRP GFC was built (2026-07-29). "Prp (GFC)" is the same Growth Factor Concentrate treatment now covered by the existing Advanced PRP GFC brochure. No new brochure built, this row is covered by advanced-prp-gfc-brochure.html. CROSS-REFERENCE 2026-07-30: a second, richer PRP-GFC brochure (prp-gfc-brochure.html) was later built from a user-supplied manufacturer PDF (Viyata GFC Kit) covering both hair growth and skin rejuvenation with real photos and clinical stats -- kept as a separate brochure alongside advanced-prp-gfc-brochure.html per user's choice, rather than replacing it.</v>
       </c>
       <c r="E160" t="str">
         <v>2026-07-30</v>

</xml_diff>

<commit_message>
Update brochure.xlsx: mark NCTF as Completed
NCTF row (previously Missing - No Source, now resolved with a user-supplied Fillmed manufacturer PDF) marked Completed pointing to nctf-135-ha-brochure.html. NCTF Pro remains Missing - No Source as this PDF only covers standard NCTF 135 HA. Reconciled: 154 unique files in index.html, all 154 marked Completed in Excel, zero gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brochure.xlsx
+++ b/brochure.xlsx
@@ -3495,13 +3495,13 @@
         <v>NCTF</v>
       </c>
       <c r="C182" t="str">
-        <v>Missing - No Source</v>
+        <v>Completed</v>
       </c>
       <c r="D182" t="str">
-        <v>No existing brochure, no matching page on isaacluxe.co sitemap, and no PDF/source provided yet. Cannot build without fabricating content.</v>
+        <v>Built from a user-supplied Fillmed Laboratoires manufacturer training PDF (Skin Quality + NCTF + Nanosoft slidekit, Dec 2021) -- real active formula (hyaluronic acid + 59 skin-revitalising ingredients), 3-session mesotherapy protocol, Nanosoft micro-injector technique, and real clinical results. Real product photo and a genuine before/after clinical photo (Dr Riekie Smit) extracted directly from the PDF. Placed under Injectable. Brochure: nctf-135-ha-brochure.html. Includes "Your Treatment Journey" page, 9 pages total.</v>
       </c>
       <c r="E182" t="str">
-        <v/>
+        <v>2026-07-30</v>
       </c>
     </row>
     <row r="183">

</xml_diff>